<commit_message>
Refactor fog calculation in rendertype_clouds.fsh for improved visual consistency
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABB5246F-3655-426C-932D-120CEBDCE6E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0EE2656-A98F-4747-8846-90E9097A3B5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="421" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="64">
   <si>
     <t>Minecraft Version</t>
   </si>
@@ -226,6 +226,9 @@
   </si>
   <si>
     <t>1.21.6 / 1.21.7</t>
+  </si>
+  <si>
+    <t>Added golden dandelion texture</t>
   </si>
 </sst>
 </file>
@@ -404,7 +407,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -440,23 +443,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -474,6 +461,21 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -749,13 +751,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
       <c r="G1" s="7" t="s">
         <v>20</v>
       </c>
@@ -765,11 +767,11 @@
       <c r="K1" s="7"/>
     </row>
     <row r="2" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="20"/>
-      <c r="C2" s="20"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
       <c r="D2" s="2" t="s">
         <v>1</v>
       </c>
@@ -785,15 +787,15 @@
       <c r="K2" s="8"/>
     </row>
     <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A3" s="19" t="str">
+      <c r="A3" s="27" t="str">
         <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-build-" &amp; D3</f>
-        <v>v10.0.11_1-build-5340</v>
-      </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
+        <v>v10.0.11_1-build-5343</v>
+      </c>
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
       <c r="D3" s="9">
-        <f>SUM(2601,637,2026,27,49)</f>
-        <v>5340</v>
+        <f>SUM(2601,637,2026,27,52)</f>
+        <v>5343</v>
       </c>
       <c r="E3" s="17">
         <f>K4</f>
@@ -822,11 +824,11 @@
       <c r="B4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="26" t="s">
+      <c r="C4" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="27"/>
-      <c r="E4" s="28"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="22"/>
       <c r="G4" s="9" t="s">
         <v>13</v>
       </c>
@@ -838,22 +840,22 @@
       </c>
       <c r="J4" s="9">
         <f>D3</f>
-        <v>5340</v>
+        <v>5343</v>
       </c>
       <c r="K4" s="9">
         <v>26.1</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="25"/>
-      <c r="C5" s="29" t="s">
+      <c r="B5" s="8"/>
+      <c r="C5" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="30"/>
-      <c r="E5" s="31"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="25"/>
       <c r="G5" s="4" t="s">
         <v>8</v>
       </c>
@@ -866,10 +868,10 @@
       <c r="K5" s="14"/>
     </row>
     <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="B6" s="25"/>
+      <c r="B6" s="8"/>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
       <c r="E6" s="8"/>
@@ -886,7 +888,9 @@
       <c r="K6" s="14"/>
     </row>
     <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="8"/>
+      <c r="A7" s="8" t="s">
+        <v>63</v>
+      </c>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
@@ -897,7 +901,7 @@
       </c>
       <c r="H7" s="11" t="str">
         <f>H6 &amp; "-build-" &amp; J4</f>
-        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5340</v>
+        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5343</v>
       </c>
       <c r="I7" s="12"/>
       <c r="J7" s="13"/>
@@ -954,7 +958,7 @@
       </c>
       <c r="I10" s="9">
         <f>J4</f>
-        <v>5340</v>
+        <v>5343</v>
       </c>
       <c r="J10" s="9" t="s">
         <v>10</v>
@@ -1009,7 +1013,7 @@
       </c>
       <c r="H13" s="15" t="str">
         <f>H12 &amp; "-build-" &amp; I10</f>
-        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5340</v>
+        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5343</v>
       </c>
       <c r="I13" s="16"/>
       <c r="J13" s="8"/>
@@ -1051,7 +1055,7 @@
       </c>
       <c r="I15" s="9">
         <f>I10</f>
-        <v>5340</v>
+        <v>5343</v>
       </c>
       <c r="J15" s="9" t="s">
         <v>11</v>
@@ -1106,7 +1110,7 @@
       </c>
       <c r="H18" s="15" t="str">
         <f>H17 &amp; "-build-" &amp; I15</f>
-        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5340</v>
+        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5343</v>
       </c>
       <c r="I18" s="16"/>
       <c r="J18" s="8"/>
@@ -1148,7 +1152,7 @@
       </c>
       <c r="I20" s="9">
         <f>I15</f>
-        <v>5340</v>
+        <v>5343</v>
       </c>
       <c r="J20" s="9" t="s">
         <v>62</v>
@@ -1203,7 +1207,7 @@
       </c>
       <c r="H23" s="15" t="str">
         <f>H22 &amp; "-build-" &amp; I20</f>
-        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5340</v>
+        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5343</v>
       </c>
       <c r="I23" s="16"/>
       <c r="J23" s="8"/>
@@ -1245,7 +1249,7 @@
       </c>
       <c r="I25" s="9">
         <f>I20</f>
-        <v>5340</v>
+        <v>5343</v>
       </c>
       <c r="J25" s="9" t="s">
         <v>12</v>
@@ -1300,7 +1304,7 @@
       </c>
       <c r="H28" s="15" t="str">
         <f>H27 &amp; "-build-" &amp; I25</f>
-        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5340</v>
+        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5343</v>
       </c>
       <c r="I28" s="16"/>
       <c r="J28" s="8"/>
@@ -1357,7 +1361,7 @@
       </c>
       <c r="I31" s="9">
         <f>I25</f>
-        <v>5340</v>
+        <v>5343</v>
       </c>
       <c r="J31" s="9" t="s">
         <v>14</v>
@@ -1412,7 +1416,7 @@
       </c>
       <c r="H34" s="15" t="str">
         <f>H33 &amp; "-build-" &amp; I31</f>
-        <v>v10.0.3-Classic_Reimagined_10_SE-build-5340</v>
+        <v>v10.0.3-Classic_Reimagined_10_SE-build-5343</v>
       </c>
       <c r="I34" s="16"/>
       <c r="J34" s="8"/>
@@ -1469,7 +1473,7 @@
       </c>
       <c r="I37" s="9">
         <f>I31</f>
-        <v>5340</v>
+        <v>5343</v>
       </c>
       <c r="J37" s="9" t="s">
         <v>17</v>
@@ -1523,7 +1527,7 @@
       </c>
       <c r="H40" s="15" t="str">
         <f>H39 &amp; "-build-" &amp; I37</f>
-        <v>v10.0.2-Classic_Reimagined_10s-build-5340</v>
+        <v>v10.0.2-Classic_Reimagined_10s-build-5343</v>
       </c>
       <c r="I40" s="16"/>
       <c r="J40" s="8"/>
@@ -1580,7 +1584,7 @@
       </c>
       <c r="I43" s="9">
         <f>I37</f>
-        <v>5340</v>
+        <v>5343</v>
       </c>
       <c r="J43" s="9" t="s">
         <v>18</v>
@@ -1634,7 +1638,7 @@
       </c>
       <c r="H46" s="15" t="str">
         <f>H45 &amp; "-build-" &amp; I43</f>
-        <v>v10.0.1-Classic_Reimagined_10-build-5340</v>
+        <v>v10.0.1-Classic_Reimagined_10-build-5343</v>
       </c>
       <c r="I46" s="16"/>
       <c r="J46" s="8"/>
@@ -1706,7 +1710,7 @@
       </c>
       <c r="I50" s="9">
         <f>I43</f>
-        <v>5340</v>
+        <v>5343</v>
       </c>
       <c r="J50" s="9" t="s">
         <v>30</v>
@@ -1760,7 +1764,7 @@
       </c>
       <c r="H53" s="15" t="str">
         <f>H52 &amp; "-build-" &amp; I50</f>
-        <v>v8.10.32-Classic_Reimagined_8-build-5340</v>
+        <v>v8.10.32-Classic_Reimagined_8-build-5343</v>
       </c>
       <c r="I53" s="16"/>
       <c r="J53" s="8"/>
@@ -1817,7 +1821,7 @@
       </c>
       <c r="I56" s="9">
         <f>I50</f>
-        <v>5340</v>
+        <v>5343</v>
       </c>
       <c r="J56" s="9" t="s">
         <v>31</v>
@@ -1871,7 +1875,7 @@
       </c>
       <c r="H59" s="15" t="str">
         <f>H58 &amp; "-build-" &amp; I56</f>
-        <v>v8.10.31-Classic_Reimagined_8-build-5340</v>
+        <v>v8.10.31-Classic_Reimagined_8-build-5343</v>
       </c>
       <c r="I59" s="16"/>
       <c r="J59" s="8"/>
@@ -1928,7 +1932,7 @@
       </c>
       <c r="I62" s="9">
         <f>I56</f>
-        <v>5340</v>
+        <v>5343</v>
       </c>
       <c r="J62" s="9" t="s">
         <v>61</v>
@@ -1982,7 +1986,7 @@
       </c>
       <c r="H65" s="15" t="str">
         <f>H64 &amp; "-build-" &amp; I62</f>
-        <v>v7.11.3-Better_Default_7-build-5340</v>
+        <v>v7.11.3-Better_Default_7-build-5343</v>
       </c>
       <c r="I65" s="16"/>
       <c r="J65" s="8"/>
@@ -2009,12 +2013,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
     </row>
     <row r="2" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
@@ -2053,21 +2057,21 @@
       <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="28" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="22"/>
+      <c r="C5" s="29"/>
       <c r="D5" s="1"/>
     </row>
     <row r="6" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="21" t="str">
+      <c r="B6" s="28" t="str">
         <f>A4 &amp; "." &amp; B4 &amp; "." &amp; C4 &amp; "-" &amp; B5</f>
         <v>v6.0.7-Better_Default_6</v>
       </c>
-      <c r="C6" s="22"/>
+      <c r="C6" s="29"/>
       <c r="D6" s="1"/>
     </row>
     <row r="7" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2107,21 +2111,21 @@
       <c r="A10" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="21" t="s">
+      <c r="B10" s="28" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="22"/>
+      <c r="C10" s="29"/>
       <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="21" t="str">
+      <c r="B11" s="28" t="str">
         <f>A9 &amp; "." &amp; B9 &amp; "." &amp; C9 &amp; "-" &amp; B10</f>
         <v>v1.4.0-Better_Default_5</v>
       </c>
-      <c r="C11" s="22"/>
+      <c r="C11" s="29"/>
       <c r="D11" s="1"/>
     </row>
     <row r="12" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2161,21 +2165,21 @@
       <c r="A15" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B15" s="21" t="s">
+      <c r="B15" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="22"/>
+      <c r="C15" s="29"/>
       <c r="D15" s="1"/>
     </row>
     <row r="16" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="21" t="str">
+      <c r="B16" s="28" t="str">
         <f>A14 &amp; "." &amp; B14 &amp; "." &amp; C14 &amp; "-" &amp; B15</f>
         <v>v1.3.0-Better_Default_4</v>
       </c>
-      <c r="C16" s="22"/>
+      <c r="C16" s="29"/>
       <c r="D16" s="1"/>
     </row>
     <row r="17" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2215,21 +2219,21 @@
       <c r="A20" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B20" s="21" t="s">
+      <c r="B20" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="C20" s="22"/>
+      <c r="C20" s="29"/>
       <c r="D20" s="1"/>
     </row>
     <row r="21" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B21" s="21" t="str">
+      <c r="B21" s="28" t="str">
         <f>A19 &amp; "." &amp; B19 &amp; "." &amp; C19 &amp; "-" &amp; B20</f>
         <v>v1.2.2-Better_Default_3</v>
       </c>
-      <c r="C21" s="22"/>
+      <c r="C21" s="29"/>
       <c r="D21" s="1"/>
     </row>
     <row r="22" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2269,21 +2273,21 @@
       <c r="A25" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B25" s="21" t="s">
+      <c r="B25" s="28" t="s">
         <v>43</v>
       </c>
-      <c r="C25" s="22"/>
+      <c r="C25" s="29"/>
       <c r="D25" s="1"/>
     </row>
     <row r="26" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B26" s="21" t="str">
+      <c r="B26" s="28" t="str">
         <f>A24 &amp; "." &amp; B24 &amp; "." &amp; C24 &amp; "-" &amp; B25</f>
         <v>v1.2.1-Better_Default_3</v>
       </c>
-      <c r="C26" s="22"/>
+      <c r="C26" s="29"/>
       <c r="D26" s="1"/>
     </row>
     <row r="27" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2323,21 +2327,21 @@
       <c r="A30" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B30" s="21" t="s">
+      <c r="B30" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="C30" s="22"/>
+      <c r="C30" s="29"/>
       <c r="D30" s="1"/>
     </row>
     <row r="31" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B31" s="21" t="str">
+      <c r="B31" s="28" t="str">
         <f>A29 &amp; "." &amp; B29 &amp; "." &amp; C29 &amp; "-" &amp; B30</f>
         <v>v1.2.0-Better_Default_2</v>
       </c>
-      <c r="C31" s="22"/>
+      <c r="C31" s="29"/>
       <c r="D31" s="1"/>
     </row>
     <row r="32" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2377,21 +2381,21 @@
       <c r="A35" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B35" s="21" t="s">
+      <c r="B35" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="C35" s="22"/>
+      <c r="C35" s="29"/>
       <c r="D35" s="1"/>
     </row>
     <row r="36" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B36" s="21" t="str">
+      <c r="B36" s="28" t="str">
         <f>A34 &amp; "." &amp; B34 &amp; "." &amp; C34 &amp; "-" &amp; B35</f>
         <v>v1.1.1-Better_Default</v>
       </c>
-      <c r="C36" s="22"/>
+      <c r="C36" s="29"/>
       <c r="D36" s="1"/>
     </row>
     <row r="37" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2431,21 +2435,21 @@
       <c r="A40" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B40" s="21" t="s">
+      <c r="B40" s="28" t="s">
         <v>47</v>
       </c>
-      <c r="C40" s="22"/>
+      <c r="C40" s="29"/>
       <c r="D40" s="1"/>
     </row>
     <row r="41" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B41" s="21" t="str">
+      <c r="B41" s="28" t="str">
         <f>A39 &amp; "." &amp; B39 &amp; "." &amp; C39 &amp; "-" &amp; B40</f>
         <v>v1.1.0-Better_Default</v>
       </c>
-      <c r="C41" s="22"/>
+      <c r="C41" s="29"/>
       <c r="D41" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix environmental fog calculation by adjusting clamp logic for improved accuracy
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B215DA1B-C05F-4AA7-97AC-FA423FB2A3C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C444AE81-E89D-403E-ACFE-2D476726762C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="421" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="68">
   <si>
     <t>Minecraft Version</t>
   </si>
@@ -238,6 +238,9 @@
   </si>
   <si>
     <t>Crackers0106 (golden dandelion texture)</t>
+  </si>
+  <si>
+    <t>Fixed entity lighting</t>
   </si>
 </sst>
 </file>
@@ -936,7 +939,9 @@
       <c r="K8" s="8"/>
     </row>
     <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
+      <c r="A9" s="8" t="s">
+        <v>67</v>
+      </c>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
@@ -2467,6 +2472,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2479,11 +2489,6 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Move polytone assets to versioned directory
Renamed various polytone asset files and directories to the v8.10.31-Classic_Reimagined_8 path for better version organization. Also updated version_guide.xlsx.
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C444AE81-E89D-403E-ACFE-2D476726762C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D0E22BF-734E-446C-8171-FD53E67EB43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="421" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="70">
   <si>
     <t>Minecraft Version</t>
   </si>
@@ -241,6 +241,12 @@
   </si>
   <si>
     <t>Fixed entity lighting</t>
+  </si>
+  <si>
+    <t>Fixed invisible items</t>
+  </si>
+  <si>
+    <t>Added biome modifiers</t>
   </si>
 </sst>
 </file>
@@ -962,7 +968,9 @@
       <c r="K9" s="8"/>
     </row>
     <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="8"/>
+      <c r="A10" s="8" t="s">
+        <v>68</v>
+      </c>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
@@ -984,7 +992,9 @@
       <c r="K10" s="8"/>
     </row>
     <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A11" s="8"/>
+      <c r="A11" s="8" t="s">
+        <v>69</v>
+      </c>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
@@ -2472,11 +2482,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2489,6 +2494,11 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Refactor shaders and assets for version 1.20.2
- Removed obsolete cloud shaders and configurations from 1.20.0.
- Added new rendertype_clouds shaders (vertex, fragment, and JSON) for 1.20.2.
- Introduced fog.glsl and flat_item.glsl includes for improved rendering.
- Updated shader versioning from 150 to 460 for compatibility with newer graphics features.
- Deleted unused moon and sun texture assets from the environment.
- Updated pack metadata to reflect the new shader directory structure.
- Cleaned up various shader files to enhance performance and maintainability.
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72E827B5-BA2A-42A2-BDFC-342BFDBD6ED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB4853A2-BAEC-4D73-A10E-E11B4E9A6163}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="421" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="64">
   <si>
     <t>Minecraft Version</t>
   </si>
@@ -216,40 +216,19 @@
     <t>Current version in development</t>
   </si>
   <si>
-    <t>Renamed resource pack folders</t>
-  </si>
-  <si>
-    <t>Fixed environmental fog for 1.21.6 and above</t>
-  </si>
-  <si>
     <t>1.20.0</t>
   </si>
   <si>
     <t>1.21.6 / 1.21.7</t>
   </si>
   <si>
-    <t>Added golden dandelion texture</t>
-  </si>
-  <si>
     <t>Better_Default_3.1</t>
   </si>
   <si>
-    <t>Re-added classic cat sound</t>
-  </si>
-  <si>
-    <t>Crackers0106 (golden dandelion texture)</t>
-  </si>
-  <si>
-    <t>Fixed entity lighting</t>
-  </si>
-  <si>
-    <t>Fixed invisible items</t>
-  </si>
-  <si>
-    <t>Added biome modifiers</t>
-  </si>
-  <si>
-    <t>Clamped cloud distance rendering between cloud render distance and terrain render distance</t>
+    <t>Reverted classic sun and moon</t>
+  </si>
+  <si>
+    <t>Raised GLSL version for 1.20.2 and 1.21</t>
   </si>
 </sst>
 </file>
@@ -811,13 +790,13 @@
     <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" s="27" t="str">
         <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-build-" &amp; D3</f>
-        <v>v10.0.11_1-build-5368-rt3</v>
+        <v>v10.0.11_1-build-5369-rt3</v>
       </c>
       <c r="B3" s="27"/>
       <c r="C3" s="27"/>
       <c r="D3" s="9" t="str">
-        <f>SUM(2601,637,2026,27,77) &amp; "-rt3"</f>
-        <v>5368-rt3</v>
+        <f>SUM(2601,637,2026,27,78) &amp; "-rt3"</f>
+        <v>5369-rt3</v>
       </c>
       <c r="E3" s="17">
         <f>K4</f>
@@ -862,7 +841,7 @@
       </c>
       <c r="J4" s="9" t="str">
         <f>D3</f>
-        <v>5368-rt3</v>
+        <v>5369-rt3</v>
       </c>
       <c r="K4" s="9">
         <v>26.1</v>
@@ -870,11 +849,9 @@
     </row>
     <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>66</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="B5" s="8"/>
       <c r="C5" s="23" t="s">
         <v>3</v>
       </c>
@@ -893,7 +870,7 @@
     </row>
     <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="8" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -912,9 +889,7 @@
       <c r="K6" s="14"/>
     </row>
     <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
-        <v>63</v>
-      </c>
+      <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
@@ -925,16 +900,14 @@
       </c>
       <c r="H7" s="11" t="str">
         <f>H6 &amp; "-build-" &amp; J4</f>
-        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5368-rt3</v>
+        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5369-rt3</v>
       </c>
       <c r="I7" s="12"/>
       <c r="J7" s="13"/>
       <c r="K7" s="8"/>
     </row>
     <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
-        <v>65</v>
-      </c>
+      <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
@@ -949,9 +922,7 @@
       <c r="K8" s="8"/>
     </row>
     <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
-        <v>67</v>
-      </c>
+      <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
@@ -972,9 +943,7 @@
       <c r="K9" s="8"/>
     </row>
     <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
-        <v>68</v>
-      </c>
+      <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
@@ -988,7 +957,7 @@
       </c>
       <c r="I10" s="9" t="str">
         <f>J4</f>
-        <v>5368-rt3</v>
+        <v>5369-rt3</v>
       </c>
       <c r="J10" s="9" t="s">
         <v>10</v>
@@ -996,9 +965,7 @@
       <c r="K10" s="8"/>
     </row>
     <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A11" s="8" t="s">
-        <v>69</v>
-      </c>
+      <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
       <c r="D11" s="8"/>
@@ -1016,9 +983,7 @@
       <c r="K11" s="8"/>
     </row>
     <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
-        <v>70</v>
-      </c>
+      <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
@@ -1047,7 +1012,7 @@
       </c>
       <c r="H13" s="15" t="str">
         <f>H12 &amp; "-build-" &amp; I10</f>
-        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5368-rt3</v>
+        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5369-rt3</v>
       </c>
       <c r="I13" s="16"/>
       <c r="J13" s="8"/>
@@ -1089,7 +1054,7 @@
       </c>
       <c r="I15" s="9" t="str">
         <f>I10</f>
-        <v>5368-rt3</v>
+        <v>5369-rt3</v>
       </c>
       <c r="J15" s="9" t="s">
         <v>11</v>
@@ -1144,7 +1109,7 @@
       </c>
       <c r="H18" s="15" t="str">
         <f>H17 &amp; "-build-" &amp; I15</f>
-        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5368-rt3</v>
+        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5369-rt3</v>
       </c>
       <c r="I18" s="16"/>
       <c r="J18" s="8"/>
@@ -1186,10 +1151,10 @@
       </c>
       <c r="I20" s="9" t="str">
         <f>I15</f>
-        <v>5368-rt3</v>
+        <v>5369-rt3</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K20" s="8"/>
     </row>
@@ -1241,7 +1206,7 @@
       </c>
       <c r="H23" s="15" t="str">
         <f>H22 &amp; "-build-" &amp; I20</f>
-        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5368-rt3</v>
+        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5369-rt3</v>
       </c>
       <c r="I23" s="16"/>
       <c r="J23" s="8"/>
@@ -1283,7 +1248,7 @@
       </c>
       <c r="I25" s="9" t="str">
         <f>I20</f>
-        <v>5368-rt3</v>
+        <v>5369-rt3</v>
       </c>
       <c r="J25" s="9" t="s">
         <v>12</v>
@@ -1338,7 +1303,7 @@
       </c>
       <c r="H28" s="15" t="str">
         <f>H27 &amp; "-build-" &amp; I25</f>
-        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5368-rt3</v>
+        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5369-rt3</v>
       </c>
       <c r="I28" s="16"/>
       <c r="J28" s="8"/>
@@ -1395,7 +1360,7 @@
       </c>
       <c r="I31" s="9" t="str">
         <f>I25</f>
-        <v>5368-rt3</v>
+        <v>5369-rt3</v>
       </c>
       <c r="J31" s="9" t="s">
         <v>14</v>
@@ -1450,7 +1415,7 @@
       </c>
       <c r="H34" s="15" t="str">
         <f>H33 &amp; "-build-" &amp; I31</f>
-        <v>v10.0.3-Classic_Reimagined_10_SE-build-5368-rt3</v>
+        <v>v10.0.3-Classic_Reimagined_10_SE-build-5369-rt3</v>
       </c>
       <c r="I34" s="16"/>
       <c r="J34" s="8"/>
@@ -1507,7 +1472,7 @@
       </c>
       <c r="I37" s="9" t="str">
         <f>I31</f>
-        <v>5368-rt3</v>
+        <v>5369-rt3</v>
       </c>
       <c r="J37" s="9" t="s">
         <v>17</v>
@@ -1561,7 +1526,7 @@
       </c>
       <c r="H40" s="15" t="str">
         <f>H39 &amp; "-build-" &amp; I37</f>
-        <v>v10.0.2-Classic_Reimagined_10s-build-5368-rt3</v>
+        <v>v10.0.2-Classic_Reimagined_10s-build-5369-rt3</v>
       </c>
       <c r="I40" s="16"/>
       <c r="J40" s="8"/>
@@ -1618,7 +1583,7 @@
       </c>
       <c r="I43" s="9" t="str">
         <f>I37</f>
-        <v>5368-rt3</v>
+        <v>5369-rt3</v>
       </c>
       <c r="J43" s="9" t="s">
         <v>18</v>
@@ -1672,7 +1637,7 @@
       </c>
       <c r="H46" s="15" t="str">
         <f>H45 &amp; "-build-" &amp; I43</f>
-        <v>v10.0.1-Classic_Reimagined_10-build-5368-rt3</v>
+        <v>v10.0.1-Classic_Reimagined_10-build-5369-rt3</v>
       </c>
       <c r="I46" s="16"/>
       <c r="J46" s="8"/>
@@ -1744,7 +1709,7 @@
       </c>
       <c r="I50" s="9" t="str">
         <f>I43</f>
-        <v>5368-rt3</v>
+        <v>5369-rt3</v>
       </c>
       <c r="J50" s="9" t="s">
         <v>30</v>
@@ -1798,7 +1763,7 @@
       </c>
       <c r="H53" s="15" t="str">
         <f>H52 &amp; "-build-" &amp; I50</f>
-        <v>v8.10.32-Classic_Reimagined_8-build-5368-rt3</v>
+        <v>v8.10.32-Classic_Reimagined_8-build-5369-rt3</v>
       </c>
       <c r="I53" s="16"/>
       <c r="J53" s="8"/>
@@ -1855,7 +1820,7 @@
       </c>
       <c r="I56" s="9" t="str">
         <f>I50</f>
-        <v>5368-rt3</v>
+        <v>5369-rt3</v>
       </c>
       <c r="J56" s="9" t="s">
         <v>31</v>
@@ -1909,7 +1874,7 @@
       </c>
       <c r="H59" s="15" t="str">
         <f>H58 &amp; "-build-" &amp; I56</f>
-        <v>v8.10.31-Classic_Reimagined_8-build-5368-rt3</v>
+        <v>v8.10.31-Classic_Reimagined_8-build-5369-rt3</v>
       </c>
       <c r="I59" s="16"/>
       <c r="J59" s="8"/>
@@ -1966,10 +1931,10 @@
       </c>
       <c r="I62" s="9" t="str">
         <f>I56</f>
-        <v>5368-rt3</v>
+        <v>5369-rt3</v>
       </c>
       <c r="J62" s="9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="K62" s="8"/>
     </row>
@@ -2020,7 +1985,7 @@
       </c>
       <c r="H65" s="15" t="str">
         <f>H64 &amp; "-build-" &amp; I62</f>
-        <v>v7.11.3-Better_Default_7-build-5368-rt3</v>
+        <v>v7.11.3-Better_Default_7-build-5369-rt3</v>
       </c>
       <c r="I65" s="16"/>
       <c r="J65" s="8"/>
@@ -2254,7 +2219,7 @@
         <v>8</v>
       </c>
       <c r="B20" s="28" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C20" s="29"/>
       <c r="D20" s="1"/>
@@ -2488,6 +2453,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2500,11 +2470,6 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Add is_nether.json for biome modifiers with fog settings
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE029E73-A8C0-45F5-9198-042E78DCA9C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E65C3CD-2664-4FAA-8DBB-8D6D7F850CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="421" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="66">
   <si>
     <t>Minecraft Version</t>
   </si>
@@ -232,6 +232,9 @@
   </si>
   <si>
     <t>Reimproved environmental fog</t>
+  </si>
+  <si>
+    <t>Fixed nether fog (1.21.6+)</t>
   </si>
 </sst>
 </file>
@@ -912,7 +915,9 @@
       <c r="K7" s="8"/>
     </row>
     <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="8"/>
+      <c r="A8" s="8" t="s">
+        <v>65</v>
+      </c>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
@@ -2458,11 +2463,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2475,6 +2475,11 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
undone 26.1 shader fix
lightmap sample got fixed in snaphot 7
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E8DE1B4-D41C-44D0-8E9B-8F10A57F91D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C305EB-6D67-4668-80E1-7B6AEC9C7698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="72">
   <si>
     <t>Current version in development</t>
   </si>
@@ -247,6 +247,9 @@
   </si>
   <si>
     <t>Updated GUI textures</t>
+  </si>
+  <si>
+    <t>Undone 26.1 shader fix</t>
   </si>
 </sst>
 </file>
@@ -703,13 +706,13 @@
     <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="str">
         <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-build-" &amp; D3</f>
-        <v>v10.0.11_1-build-5407-rt3</v>
+        <v>v10.0.11_1-build-5410-rt3</v>
       </c>
       <c r="B3" s="19"/>
       <c r="C3" s="19"/>
       <c r="D3" s="8" t="str">
-        <f>SUM(2601,664,2026,116) &amp; "-rt3"</f>
-        <v>5407-rt3</v>
+        <f>SUM(2601,664,2026,119) &amp; "-rt3"</f>
+        <v>5410-rt3</v>
       </c>
       <c r="E3" s="7">
         <f>K4</f>
@@ -754,7 +757,7 @@
       </c>
       <c r="J4" s="8" t="str">
         <f>D3</f>
-        <v>5407-rt3</v>
+        <v>5410-rt3</v>
       </c>
       <c r="K4" s="8">
         <v>26.1</v>
@@ -815,7 +818,7 @@
       </c>
       <c r="H7" s="11" t="str">
         <f>H6 &amp; "-build-" &amp; J4</f>
-        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5407-rt3</v>
+        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5410-rt3</v>
       </c>
       <c r="I7" s="12"/>
       <c r="J7" s="13"/>
@@ -878,7 +881,7 @@
       </c>
       <c r="I10" s="8" t="str">
         <f>J4</f>
-        <v>5407-rt3</v>
+        <v>5410-rt3</v>
       </c>
       <c r="J10" s="8" t="s">
         <v>24</v>
@@ -939,14 +942,16 @@
       </c>
       <c r="H13" s="15" t="str">
         <f>H12 &amp; "-build-" &amp; I10</f>
-        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5407-rt3</v>
+        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5410-rt3</v>
       </c>
       <c r="I13" s="16"/>
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
     </row>
     <row r="14" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A14" s="6"/>
+      <c r="A14" s="6" t="s">
+        <v>71</v>
+      </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
@@ -981,7 +986,7 @@
       </c>
       <c r="I15" s="8" t="str">
         <f>I10</f>
-        <v>5407-rt3</v>
+        <v>5410-rt3</v>
       </c>
       <c r="J15" s="8" t="s">
         <v>25</v>
@@ -1036,7 +1041,7 @@
       </c>
       <c r="H18" s="15" t="str">
         <f>H17 &amp; "-build-" &amp; I15</f>
-        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5407-rt3</v>
+        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5410-rt3</v>
       </c>
       <c r="I18" s="16"/>
       <c r="J18" s="6"/>
@@ -1078,7 +1083,7 @@
       </c>
       <c r="I20" s="8" t="str">
         <f>I15</f>
-        <v>5407-rt3</v>
+        <v>5410-rt3</v>
       </c>
       <c r="J20" s="8" t="s">
         <v>26</v>
@@ -1133,7 +1138,7 @@
       </c>
       <c r="H23" s="15" t="str">
         <f>H22 &amp; "-build-" &amp; I20</f>
-        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5407-rt3</v>
+        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5410-rt3</v>
       </c>
       <c r="I23" s="16"/>
       <c r="J23" s="6"/>
@@ -1175,7 +1180,7 @@
       </c>
       <c r="I25" s="8" t="str">
         <f>I20</f>
-        <v>5407-rt3</v>
+        <v>5410-rt3</v>
       </c>
       <c r="J25" s="8" t="s">
         <v>27</v>
@@ -1230,7 +1235,7 @@
       </c>
       <c r="H28" s="15" t="str">
         <f>H27 &amp; "-build-" &amp; I25</f>
-        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5407-rt3</v>
+        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5410-rt3</v>
       </c>
       <c r="I28" s="16"/>
       <c r="J28" s="6"/>
@@ -1287,7 +1292,7 @@
       </c>
       <c r="I31" s="8" t="str">
         <f>I25</f>
-        <v>5407-rt3</v>
+        <v>5410-rt3</v>
       </c>
       <c r="J31" s="8" t="s">
         <v>29</v>
@@ -1342,7 +1347,7 @@
       </c>
       <c r="H34" s="15" t="str">
         <f>H33 &amp; "-build-" &amp; I31</f>
-        <v>v10.0.3-Classic_Reimagined_10_SE-build-5407-rt3</v>
+        <v>v10.0.3-Classic_Reimagined_10_SE-build-5410-rt3</v>
       </c>
       <c r="I34" s="16"/>
       <c r="J34" s="6"/>
@@ -1399,7 +1404,7 @@
       </c>
       <c r="I37" s="8" t="str">
         <f>I31</f>
-        <v>5407-rt3</v>
+        <v>5410-rt3</v>
       </c>
       <c r="J37" s="8" t="s">
         <v>31</v>
@@ -1453,7 +1458,7 @@
       </c>
       <c r="H40" s="15" t="str">
         <f>H39 &amp; "-build-" &amp; I37</f>
-        <v>v10.0.2-Classic_Reimagined_10s-build-5407-rt3</v>
+        <v>v10.0.2-Classic_Reimagined_10s-build-5410-rt3</v>
       </c>
       <c r="I40" s="16"/>
       <c r="J40" s="6"/>
@@ -1510,7 +1515,7 @@
       </c>
       <c r="I43" s="8" t="str">
         <f>I37</f>
-        <v>5407-rt3</v>
+        <v>5410-rt3</v>
       </c>
       <c r="J43" s="8" t="s">
         <v>34</v>
@@ -1564,7 +1569,7 @@
       </c>
       <c r="H46" s="15" t="str">
         <f>H45 &amp; "-build-" &amp; I43</f>
-        <v>v10.0.1-Classic_Reimagined_10-build-5407-rt3</v>
+        <v>v10.0.1-Classic_Reimagined_10-build-5410-rt3</v>
       </c>
       <c r="I46" s="16"/>
       <c r="J46" s="6"/>
@@ -1636,7 +1641,7 @@
       </c>
       <c r="I50" s="8" t="str">
         <f>I43</f>
-        <v>5407-rt3</v>
+        <v>5410-rt3</v>
       </c>
       <c r="J50" s="8" t="s">
         <v>39</v>
@@ -1690,7 +1695,7 @@
       </c>
       <c r="H53" s="15" t="str">
         <f>H52 &amp; "-build-" &amp; I50</f>
-        <v>v8.10.32-Classic_Reimagined_8-build-5407-rt3</v>
+        <v>v8.10.32-Classic_Reimagined_8-build-5410-rt3</v>
       </c>
       <c r="I53" s="16"/>
       <c r="J53" s="6"/>
@@ -1747,7 +1752,7 @@
       </c>
       <c r="I56" s="8" t="str">
         <f>I50</f>
-        <v>5407-rt3</v>
+        <v>5410-rt3</v>
       </c>
       <c r="J56" s="8" t="s">
         <v>41</v>
@@ -1801,7 +1806,7 @@
       </c>
       <c r="H59" s="15" t="str">
         <f>H58 &amp; "-build-" &amp; I56</f>
-        <v>v8.10.31-Classic_Reimagined_8-build-5407-rt3</v>
+        <v>v8.10.31-Classic_Reimagined_8-build-5410-rt3</v>
       </c>
       <c r="I59" s="16"/>
       <c r="J59" s="6"/>
@@ -1858,7 +1863,7 @@
       </c>
       <c r="I62" s="8" t="str">
         <f>I56</f>
-        <v>5407-rt3</v>
+        <v>5410-rt3</v>
       </c>
       <c r="J62" s="8" t="s">
         <v>44</v>
@@ -1912,7 +1917,7 @@
       </c>
       <c r="H65" s="15" t="str">
         <f>H64 &amp; "-build-" &amp; I62</f>
-        <v>v7.11.3-Better_Default_7-build-5407-rt3</v>
+        <v>v7.11.3-Better_Default_7-build-5410-rt3</v>
       </c>
       <c r="I65" s="16"/>
       <c r="J65" s="6"/>
@@ -2380,11 +2385,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2397,6 +2397,11 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Adjust cloud fog color and alpha calculations
Refactor cloud shader fog blending: separate RGB and alpha calculations, add inline comments, and change fog distance parameters to hard-coded values (use 1024 and 64 for cloud distance blends and clamp FogRenderDistanceEnd comparisons to 1024). This updates how vertexColor is mixed with FogColor and how cloud alpha fades with vertexDistance to produce a different fog transition for environmental clouds. Also includes an updated version_guide.xlsx (binary metadata change).
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38C305EB-6D67-4668-80E1-7B6AEC9C7698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E03C683-591C-43F5-98C2-393D406ABDE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="73">
   <si>
     <t>Current version in development</t>
   </si>
@@ -250,6 +250,9 @@
   </si>
   <si>
     <t>Undone 26.1 shader fix</t>
+  </si>
+  <si>
+    <t>Improved cloud fog</t>
   </si>
 </sst>
 </file>
@@ -972,7 +975,9 @@
       <c r="K14" s="6"/>
     </row>
     <row r="15" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A15" s="6"/>
+      <c r="A15" s="6" t="s">
+        <v>72</v>
+      </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
       <c r="D15" s="6"/>
@@ -2385,6 +2390,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2397,11 +2407,6 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Add Classic-Reimagined-Lite assets (v1.1–v1.2.1)
Add a large collection of resource pack assets for Classic-Reimagined-Lite across v1.1.0, v1.1.1, v1.2.0 and v1.2.1. Files include polytone configs (biome modifiers, colormaps), block properties, dimension modifiers, blockstates and models, OptiFine CEMs, numerous textures (GUI, HUD, title panoramas, blocks, items, entities), GUI sprite sheets, and sounds.json. These additions populate the resource pack with visuals and audio required for the listed versions.
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32C381E3-9D83-4830-8B3D-525450BC188E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{439D96C4-95AA-456B-8109-D2786F3E5B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="68">
   <si>
     <t>Current version in development</t>
   </si>
@@ -232,6 +232,12 @@
   </si>
   <si>
     <t>1.21.6</t>
+  </si>
+  <si>
+    <t>Created Classic Reimagined Lite</t>
+  </si>
+  <si>
+    <t>Lite version</t>
   </si>
 </sst>
 </file>
@@ -388,7 +394,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -419,12 +425,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -443,6 +443,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -452,8 +455,19 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -667,20 +681,22 @@
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
-      <c r="M1" s="29" t="s">
+      <c r="M1" s="24" t="s">
         <v>62</v>
       </c>
-      <c r="N1" s="29"/>
-      <c r="O1" s="29"/>
-      <c r="P1" s="29"/>
-      <c r="Q1" s="29"/>
+      <c r="N1" s="24"/>
+      <c r="O1" s="24"/>
+      <c r="P1" s="24"/>
+      <c r="Q1" s="24"/>
     </row>
     <row r="2" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
+      <c r="B2" s="30" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" s="31"/>
       <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
@@ -711,15 +727,18 @@
       </c>
     </row>
     <row r="3" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A3" s="19" t="str">
+      <c r="A3" s="29" t="str">
         <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-build-" &amp; D3</f>
-        <v>v10.0.11_1-build-5418-rt4</v>
-      </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
+        <v>v10.0.11_1-build-5423-rt4</v>
+      </c>
+      <c r="B3" s="32" t="str">
+        <f>"v1.2.7_1-build-" &amp; D3 &amp; "-" &amp; E3</f>
+        <v>v1.2.7_1-build-5423-rt4-26.1</v>
+      </c>
+      <c r="C3" s="33"/>
       <c r="D3" s="8" t="str">
-        <f>SUM(2601,664,2026,127) &amp; "-rt4"</f>
-        <v>5418-rt4</v>
+        <f>SUM(2601,664,2026,132) &amp; "-rt4"</f>
+        <v>5423-rt4</v>
       </c>
       <c r="E3" s="7">
         <f>K4</f>
@@ -751,7 +770,7 @@
       </c>
       <c r="P3" s="8" t="str">
         <f>J4</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="Q3" s="8">
         <v>26.1</v>
@@ -764,11 +783,11 @@
       <c r="B4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="21"/>
-      <c r="E4" s="22"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="20"/>
       <c r="G4" s="8" t="s">
         <v>11</v>
       </c>
@@ -780,7 +799,7 @@
       </c>
       <c r="J4" s="8" t="str">
         <f>D3</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="K4" s="8">
         <v>26.1</v>
@@ -797,13 +816,15 @@
       <c r="Q4" s="14"/>
     </row>
     <row r="5" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A5" s="6"/>
+      <c r="A5" s="6" t="s">
+        <v>66</v>
+      </c>
       <c r="B5" s="6"/>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="24"/>
-      <c r="E5" s="25"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="23"/>
       <c r="G5" s="10" t="s">
         <v>13</v>
       </c>
@@ -847,7 +868,7 @@
       </c>
       <c r="N6" s="11" t="str">
         <f>N5 &amp; "-build-" &amp; P3</f>
-        <v>v1.2.7_1-Classic_Reimagined_Lite-build-5418-rt4</v>
+        <v>v1.2.7_1-Classic_Reimagined_Lite-build-5423-rt4</v>
       </c>
       <c r="O6" s="12"/>
       <c r="P6" s="13"/>
@@ -865,7 +886,7 @@
       </c>
       <c r="H7" s="11" t="str">
         <f>H6 &amp; "-build-" &amp; J4</f>
-        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5418-rt4</v>
+        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5423-rt4</v>
       </c>
       <c r="I7" s="12"/>
       <c r="J7" s="13"/>
@@ -905,7 +926,7 @@
       </c>
       <c r="O8" s="8" t="str">
         <f>P3</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="P8" s="8" t="s">
         <v>18</v>
@@ -956,7 +977,7 @@
       </c>
       <c r="I10" s="8" t="str">
         <f>J4</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="J10" s="8" t="s">
         <v>18</v>
@@ -994,7 +1015,7 @@
       </c>
       <c r="N11" s="15" t="str">
         <f>N10 &amp; "-build-" &amp; O8</f>
-        <v>v1.2.6-Classic_Reimagined_Lite-build-5418-rt4</v>
+        <v>v1.2.6-Classic_Reimagined_Lite-build-5423-rt4</v>
       </c>
       <c r="O11" s="16"/>
       <c r="P11" s="6"/>
@@ -1041,7 +1062,7 @@
       </c>
       <c r="H13" s="15" t="str">
         <f>H12 &amp; "-build-" &amp; I10</f>
-        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5418-rt4</v>
+        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5423-rt4</v>
       </c>
       <c r="I13" s="16"/>
       <c r="J13" s="6"/>
@@ -1054,7 +1075,7 @@
       </c>
       <c r="O13" s="8" t="str">
         <f>P3</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="P13" s="8" t="s">
         <v>19</v>
@@ -1105,7 +1126,7 @@
       </c>
       <c r="I15" s="8" t="str">
         <f>I10</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="J15" s="8" t="s">
         <v>19</v>
@@ -1143,7 +1164,7 @@
       </c>
       <c r="N16" s="15" t="str">
         <f>N15 &amp; "-build-" &amp; O13</f>
-        <v>v1.2.5-Classic_Reimagined_Lite-build-5418-rt4</v>
+        <v>v1.2.5-Classic_Reimagined_Lite-build-5423-rt4</v>
       </c>
       <c r="O16" s="16"/>
       <c r="P16" s="6"/>
@@ -1190,7 +1211,7 @@
       </c>
       <c r="H18" s="15" t="str">
         <f>H17 &amp; "-build-" &amp; I15</f>
-        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5418-rt4</v>
+        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5423-rt4</v>
       </c>
       <c r="I18" s="16"/>
       <c r="J18" s="6"/>
@@ -1203,7 +1224,7 @@
       </c>
       <c r="O18" s="8" t="str">
         <f>P3</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="P18" s="8" t="s">
         <v>65</v>
@@ -1254,7 +1275,7 @@
       </c>
       <c r="I20" s="8" t="str">
         <f>I15</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="J20" s="8" t="s">
         <v>20</v>
@@ -1292,7 +1313,7 @@
       </c>
       <c r="N21" s="15" t="str">
         <f>N20 &amp; "-build-" &amp; O18</f>
-        <v>v1.2.4-Classic_Reimagined_Lite-build-5418-rt4</v>
+        <v>v1.2.4-Classic_Reimagined_Lite-build-5423-rt4</v>
       </c>
       <c r="O21" s="16"/>
       <c r="P21" s="6"/>
@@ -1339,7 +1360,7 @@
       </c>
       <c r="H23" s="15" t="str">
         <f>H22 &amp; "-build-" &amp; I20</f>
-        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5418-rt4</v>
+        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5423-rt4</v>
       </c>
       <c r="I23" s="16"/>
       <c r="J23" s="6"/>
@@ -1352,7 +1373,7 @@
       </c>
       <c r="O23" s="8" t="str">
         <f>P3</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="P23" s="8" t="s">
         <v>21</v>
@@ -1403,7 +1424,7 @@
       </c>
       <c r="I25" s="8" t="str">
         <f>I20</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="J25" s="8" t="s">
         <v>21</v>
@@ -1441,7 +1462,7 @@
       </c>
       <c r="N26" s="15" t="str">
         <f>N25 &amp; "-build-" &amp; O23</f>
-        <v>v1.2.3-Classic_Reimagined_Lite-build-5418-rt4</v>
+        <v>v1.2.3-Classic_Reimagined_Lite-build-5423-rt4</v>
       </c>
       <c r="O26" s="16"/>
       <c r="P26" s="6"/>
@@ -1488,7 +1509,7 @@
       </c>
       <c r="H28" s="15" t="str">
         <f>H27 &amp; "-build-" &amp; I25</f>
-        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5418-rt4</v>
+        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5423-rt4</v>
       </c>
       <c r="I28" s="16"/>
       <c r="J28" s="6"/>
@@ -1501,7 +1522,7 @@
       </c>
       <c r="O28" s="8" t="str">
         <f>O23</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="P28" s="8" t="s">
         <v>23</v>
@@ -1576,7 +1597,7 @@
       </c>
       <c r="I31" s="8" t="str">
         <f>I25</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="J31" s="8" t="s">
         <v>23</v>
@@ -1587,7 +1608,7 @@
       </c>
       <c r="N31" s="15" t="str">
         <f>N30 &amp; "-build-" &amp; O28</f>
-        <v>v1.2.2-Classic_Reimagined_Lite-build-5418-rt4</v>
+        <v>v1.2.2-Classic_Reimagined_Lite-build-5423-rt4</v>
       </c>
       <c r="O31" s="16"/>
       <c r="P31" s="6"/>
@@ -1647,7 +1668,7 @@
       </c>
       <c r="O33" s="8" t="str">
         <f>O28</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="P33" s="8" t="s">
         <v>25</v>
@@ -1665,7 +1686,7 @@
       </c>
       <c r="H34" s="15" t="str">
         <f>H33 &amp; "-build-" &amp; I31</f>
-        <v>v10.0.3-Classic_Reimagined_10_SE-build-5418-rt4</v>
+        <v>v10.0.3-Classic_Reimagined_10_SE-build-5423-rt4</v>
       </c>
       <c r="I34" s="16"/>
       <c r="J34" s="6"/>
@@ -1729,7 +1750,7 @@
       </c>
       <c r="N36" s="15" t="str">
         <f>N35 &amp; "-build-" &amp; O33</f>
-        <v>v1.2.1-Classic_Reimagined_Lite-build-5418-rt4</v>
+        <v>v1.2.1-Classic_Reimagined_Lite-build-5423-rt4</v>
       </c>
       <c r="O36" s="16"/>
       <c r="P36" s="6"/>
@@ -1749,7 +1770,7 @@
       </c>
       <c r="I37" s="8" t="str">
         <f>I31</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="J37" s="8" t="s">
         <v>25</v>
@@ -1792,7 +1813,7 @@
       </c>
       <c r="O38" s="8" t="str">
         <f>O33</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="P38" s="8" t="s">
         <v>28</v>
@@ -1837,7 +1858,7 @@
       </c>
       <c r="H40" s="15" t="str">
         <f>H39 &amp; "-build-" &amp; I37</f>
-        <v>v10.0.2-Classic_Reimagined_10s-build-5418-rt4</v>
+        <v>v10.0.2-Classic_Reimagined_10s-build-5423-rt4</v>
       </c>
       <c r="I40" s="16"/>
       <c r="J40" s="6"/>
@@ -1871,7 +1892,7 @@
       </c>
       <c r="N41" s="15" t="str">
         <f>N40 &amp; "-build-" &amp; O38</f>
-        <v>v1.2.0-Classic_Reimagined_Lite-build-5418-rt4</v>
+        <v>v1.2.0-Classic_Reimagined_Lite-build-5423-rt4</v>
       </c>
       <c r="O41" s="16"/>
       <c r="P41" s="6"/>
@@ -1924,7 +1945,7 @@
       </c>
       <c r="I43" s="8" t="str">
         <f>I37</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="J43" s="8" t="s">
         <v>28</v>
@@ -1938,7 +1959,7 @@
       </c>
       <c r="O43" s="8" t="str">
         <f>O38</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="P43" s="8" t="s">
         <v>33</v>
@@ -2009,7 +2030,7 @@
       </c>
       <c r="H46" s="15" t="str">
         <f>H45 &amp; "-build-" &amp; I43</f>
-        <v>v10.0.1-Classic_Reimagined_10-build-5418-rt4</v>
+        <v>v10.0.1-Classic_Reimagined_10-build-5423-rt4</v>
       </c>
       <c r="I46" s="16"/>
       <c r="J46" s="6"/>
@@ -2019,7 +2040,7 @@
       </c>
       <c r="N46" s="15" t="str">
         <f>N45 &amp; "-build-" &amp; O43</f>
-        <v>v1.1.1-Classic_Reimagined_Lite-build-5418-rt4</v>
+        <v>v1.1.1-Classic_Reimagined_Lite-build-5423-rt4</v>
       </c>
       <c r="O46" s="16"/>
       <c r="P46" s="6"/>
@@ -2073,7 +2094,7 @@
       </c>
       <c r="O48" s="8" t="str">
         <f>O43</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="P48" s="8" t="s">
         <v>35</v>
@@ -2124,7 +2145,7 @@
       </c>
       <c r="I50" s="8" t="str">
         <f>I43</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="J50" s="8" t="s">
         <v>33</v>
@@ -2161,7 +2182,7 @@
       </c>
       <c r="N51" s="15" t="str">
         <f>N50 &amp; "-build-" &amp; O48</f>
-        <v>v1.1.0-Classic_Reimagined_Lite-build-5418-rt4</v>
+        <v>v1.1.0-Classic_Reimagined_Lite-build-5423-rt4</v>
       </c>
       <c r="O51" s="16"/>
       <c r="P51" s="6"/>
@@ -2196,7 +2217,7 @@
       </c>
       <c r="H53" s="15" t="str">
         <f>H52 &amp; "-build-" &amp; I50</f>
-        <v>v8.10.32-Classic_Reimagined_8-build-5418-rt4</v>
+        <v>v8.10.32-Classic_Reimagined_8-build-5423-rt4</v>
       </c>
       <c r="I53" s="16"/>
       <c r="J53" s="6"/>
@@ -2253,7 +2274,7 @@
       </c>
       <c r="I56" s="8" t="str">
         <f>I50</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="J56" s="8" t="s">
         <v>35</v>
@@ -2307,7 +2328,7 @@
       </c>
       <c r="H59" s="15" t="str">
         <f>H58 &amp; "-build-" &amp; I56</f>
-        <v>v8.10.31-Classic_Reimagined_8-build-5418-rt4</v>
+        <v>v8.10.31-Classic_Reimagined_8-build-5423-rt4</v>
       </c>
       <c r="I59" s="16"/>
       <c r="J59" s="6"/>
@@ -2364,7 +2385,7 @@
       </c>
       <c r="I62" s="8" t="str">
         <f>I56</f>
-        <v>5418-rt4</v>
+        <v>5423-rt4</v>
       </c>
       <c r="J62" s="8" t="s">
         <v>38</v>
@@ -2418,7 +2439,7 @@
       </c>
       <c r="H65" s="15" t="str">
         <f>H64 &amp; "-build-" &amp; I62</f>
-        <v>v7.11.3-Better_Default_7-build-5418-rt4</v>
+        <v>v7.11.3-Better_Default_7-build-5423-rt4</v>
       </c>
       <c r="I65" s="16"/>
       <c r="J65" s="6"/>
@@ -2426,11 +2447,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="C5:E5"/>
     <mergeCell ref="M1:Q1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -2446,12 +2467,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="27" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
     </row>
     <row r="2" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
@@ -2490,21 +2511,21 @@
       <c r="A5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="26" t="s">
+      <c r="B5" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="27"/>
+      <c r="C5" s="26"/>
       <c r="D5" s="14"/>
     </row>
     <row r="6" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="26" t="str">
+      <c r="B6" s="25" t="str">
         <f>A4 &amp; "." &amp; B4 &amp; "." &amp; C4 &amp; "-" &amp; B5</f>
         <v>v6.0.7-Better_Default_6</v>
       </c>
-      <c r="C6" s="27"/>
+      <c r="C6" s="26"/>
       <c r="D6" s="14"/>
     </row>
     <row r="7" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2544,21 +2565,21 @@
       <c r="A10" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="C10" s="27"/>
+      <c r="C10" s="26"/>
       <c r="D10" s="14"/>
     </row>
     <row r="11" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="26" t="str">
+      <c r="B11" s="25" t="str">
         <f>A9 &amp; "." &amp; B9 &amp; "." &amp; C9 &amp; "-" &amp; B10</f>
         <v>v1.4.0-Better_Default_5</v>
       </c>
-      <c r="C11" s="27"/>
+      <c r="C11" s="26"/>
       <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2598,21 +2619,21 @@
       <c r="A15" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="26" t="s">
+      <c r="B15" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="27"/>
+      <c r="C15" s="26"/>
       <c r="D15" s="14"/>
     </row>
     <row r="16" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="26" t="str">
+      <c r="B16" s="25" t="str">
         <f>A14 &amp; "." &amp; B14 &amp; "." &amp; C14 &amp; "-" &amp; B15</f>
         <v>v1.3.0-Better_Default_4</v>
       </c>
-      <c r="C16" s="27"/>
+      <c r="C16" s="26"/>
       <c r="D16" s="14"/>
     </row>
     <row r="17" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2652,21 +2673,21 @@
       <c r="A20" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="27"/>
+      <c r="C20" s="26"/>
       <c r="D20" s="14"/>
     </row>
     <row r="21" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="26" t="str">
+      <c r="B21" s="25" t="str">
         <f>A19 &amp; "." &amp; B19 &amp; "." &amp; C19 &amp; "-" &amp; B20</f>
         <v>v1.2.2-Better_Default_3.1</v>
       </c>
-      <c r="C21" s="27"/>
+      <c r="C21" s="26"/>
       <c r="D21" s="14"/>
     </row>
     <row r="22" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2706,21 +2727,21 @@
       <c r="A25" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="26" t="s">
+      <c r="B25" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="27"/>
+      <c r="C25" s="26"/>
       <c r="D25" s="14"/>
     </row>
     <row r="26" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B26" s="26" t="str">
+      <c r="B26" s="25" t="str">
         <f>A24 &amp; "." &amp; B24 &amp; "." &amp; C24 &amp; "-" &amp; B25</f>
         <v>v1.2.1-Better_Default_3</v>
       </c>
-      <c r="C26" s="27"/>
+      <c r="C26" s="26"/>
       <c r="D26" s="14"/>
     </row>
     <row r="27" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2760,21 +2781,21 @@
       <c r="A30" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="26" t="s">
+      <c r="B30" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="C30" s="27"/>
+      <c r="C30" s="26"/>
       <c r="D30" s="14"/>
     </row>
     <row r="31" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A31" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="26" t="str">
+      <c r="B31" s="25" t="str">
         <f>A29 &amp; "." &amp; B29 &amp; "." &amp; C29 &amp; "-" &amp; B30</f>
         <v>v1.2.0-Better_Default_2</v>
       </c>
-      <c r="C31" s="27"/>
+      <c r="C31" s="26"/>
       <c r="D31" s="14"/>
     </row>
     <row r="32" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2814,21 +2835,21 @@
       <c r="A35" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B35" s="26" t="s">
+      <c r="B35" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="C35" s="27"/>
+      <c r="C35" s="26"/>
       <c r="D35" s="14"/>
     </row>
     <row r="36" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A36" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B36" s="26" t="str">
+      <c r="B36" s="25" t="str">
         <f>A34 &amp; "." &amp; B34 &amp; "." &amp; C34 &amp; "-" &amp; B35</f>
         <v>v1.1.1-Better_Default</v>
       </c>
-      <c r="C36" s="27"/>
+      <c r="C36" s="26"/>
       <c r="D36" s="14"/>
     </row>
     <row r="37" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2868,25 +2889,30 @@
       <c r="A40" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="26" t="s">
+      <c r="B40" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="C40" s="27"/>
+      <c r="C40" s="26"/>
       <c r="D40" s="14"/>
     </row>
     <row r="41" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A41" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B41" s="26" t="str">
+      <c r="B41" s="25" t="str">
         <f>A39 &amp; "." &amp; B39 &amp; "." &amp; C39 &amp; "-" &amp; B40</f>
         <v>v1.1.0-Better_Default</v>
       </c>
-      <c r="C41" s="27"/>
+      <c r="C41" s="26"/>
       <c r="D41" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2899,11 +2925,6 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Update fog/discard behavior and lightmap sampling
Adjust shader fog and discard logic across multiple shader files and adapt lightmap sampling API.

- Classic-Reimagined-Modded/sodium/.../block_layer_opaque.fsh: apply linear fog earlier, discard fragments whose color equals the fog color, otherwise set fragColor to the computed color.
- Classic-Reimagined/*/terrain.fsh (1.21.11 and 26.1): replace previous fog mixing/apply_fog calls with an RGB mix using total_fog_value; discard fragments when linear_fog_value == 1.0, otherwise output the computed color.
- Classic-Reimagined/26.1_shaders/.../terrain.vsh: swap import from smooth_lighting.glsl to sample_lightmap.glsl and call sample_lightmap(...) instead of minecraft_sample_lightmap(...).

These changes modify fog/alpha handling to drop fully fogged pixels and update lightmap sampling to the new API.
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{439D96C4-95AA-456B-8109-D2786F3E5B03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A2E3A0F-1E4D-4BF0-99FF-E669000A48E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="69">
   <si>
     <t>Current version in development</t>
   </si>
@@ -238,6 +238,9 @@
   </si>
   <si>
     <t>Lite version</t>
+  </si>
+  <si>
+    <t>Update fog/discard behavior and lightmap sampling</t>
   </si>
 </sst>
 </file>
@@ -394,7 +397,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -425,6 +428,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -446,17 +450,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -467,6 +460,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -681,22 +683,22 @@
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
-      <c r="M1" s="24" t="s">
+      <c r="M1" s="25" t="s">
         <v>62</v>
       </c>
-      <c r="N1" s="24"/>
-      <c r="O1" s="24"/>
-      <c r="P1" s="24"/>
-      <c r="Q1" s="24"/>
+      <c r="N1" s="25"/>
+      <c r="O1" s="25"/>
+      <c r="P1" s="25"/>
+      <c r="Q1" s="25"/>
     </row>
     <row r="2" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="C2" s="31"/>
+      <c r="C2" s="27"/>
       <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
@@ -727,15 +729,15 @@
       </c>
     </row>
     <row r="3" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A3" s="29" t="str">
+      <c r="A3" s="18" t="str">
         <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-build-" &amp; D3</f>
         <v>v10.0.11_1-build-5423-rt4</v>
       </c>
-      <c r="B3" s="32" t="str">
+      <c r="B3" s="28" t="str">
         <f>"v1.2.7_1-build-" &amp; D3 &amp; "-" &amp; E3</f>
         <v>v1.2.7_1-build-5423-rt4-26.1</v>
       </c>
-      <c r="C3" s="33"/>
+      <c r="C3" s="29"/>
       <c r="D3" s="8" t="str">
         <f>SUM(2601,664,2026,132) &amp; "-rt4"</f>
         <v>5423-rt4</v>
@@ -783,11 +785,11 @@
       <c r="B4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="19"/>
-      <c r="E4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="21"/>
       <c r="G4" s="8" t="s">
         <v>11</v>
       </c>
@@ -820,11 +822,11 @@
         <v>66</v>
       </c>
       <c r="B5" s="6"/>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="23"/>
+      <c r="D5" s="23"/>
+      <c r="E5" s="24"/>
       <c r="G5" s="10" t="s">
         <v>13</v>
       </c>
@@ -847,7 +849,9 @@
       <c r="Q5" s="14"/>
     </row>
     <row r="6" spans="1:17" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A6" s="6"/>
+      <c r="A6" s="6" t="s">
+        <v>68</v>
+      </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
       <c r="D6" s="6"/>
@@ -2467,12 +2471,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
     </row>
     <row r="2" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
@@ -2511,21 +2515,21 @@
       <c r="A5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="30" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="26"/>
+      <c r="C5" s="31"/>
       <c r="D5" s="14"/>
     </row>
     <row r="6" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="25" t="str">
+      <c r="B6" s="30" t="str">
         <f>A4 &amp; "." &amp; B4 &amp; "." &amp; C4 &amp; "-" &amp; B5</f>
         <v>v6.0.7-Better_Default_6</v>
       </c>
-      <c r="C6" s="26"/>
+      <c r="C6" s="31"/>
       <c r="D6" s="14"/>
     </row>
     <row r="7" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2565,21 +2569,21 @@
       <c r="A10" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="30" t="s">
         <v>49</v>
       </c>
-      <c r="C10" s="26"/>
+      <c r="C10" s="31"/>
       <c r="D10" s="14"/>
     </row>
     <row r="11" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="25" t="str">
+      <c r="B11" s="30" t="str">
         <f>A9 &amp; "." &amp; B9 &amp; "." &amp; C9 &amp; "-" &amp; B10</f>
         <v>v1.4.0-Better_Default_5</v>
       </c>
-      <c r="C11" s="26"/>
+      <c r="C11" s="31"/>
       <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2619,21 +2623,21 @@
       <c r="A15" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="25" t="s">
+      <c r="B15" s="30" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="26"/>
+      <c r="C15" s="31"/>
       <c r="D15" s="14"/>
     </row>
     <row r="16" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="25" t="str">
+      <c r="B16" s="30" t="str">
         <f>A14 &amp; "." &amp; B14 &amp; "." &amp; C14 &amp; "-" &amp; B15</f>
         <v>v1.3.0-Better_Default_4</v>
       </c>
-      <c r="C16" s="26"/>
+      <c r="C16" s="31"/>
       <c r="D16" s="14"/>
     </row>
     <row r="17" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2673,21 +2677,21 @@
       <c r="A20" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="25" t="s">
+      <c r="B20" s="30" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="26"/>
+      <c r="C20" s="31"/>
       <c r="D20" s="14"/>
     </row>
     <row r="21" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="25" t="str">
+      <c r="B21" s="30" t="str">
         <f>A19 &amp; "." &amp; B19 &amp; "." &amp; C19 &amp; "-" &amp; B20</f>
         <v>v1.2.2-Better_Default_3.1</v>
       </c>
-      <c r="C21" s="26"/>
+      <c r="C21" s="31"/>
       <c r="D21" s="14"/>
     </row>
     <row r="22" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2727,21 +2731,21 @@
       <c r="A25" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="25" t="s">
+      <c r="B25" s="30" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="26"/>
+      <c r="C25" s="31"/>
       <c r="D25" s="14"/>
     </row>
     <row r="26" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B26" s="25" t="str">
+      <c r="B26" s="30" t="str">
         <f>A24 &amp; "." &amp; B24 &amp; "." &amp; C24 &amp; "-" &amp; B25</f>
         <v>v1.2.1-Better_Default_3</v>
       </c>
-      <c r="C26" s="26"/>
+      <c r="C26" s="31"/>
       <c r="D26" s="14"/>
     </row>
     <row r="27" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2781,21 +2785,21 @@
       <c r="A30" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="25" t="s">
+      <c r="B30" s="30" t="s">
         <v>58</v>
       </c>
-      <c r="C30" s="26"/>
+      <c r="C30" s="31"/>
       <c r="D30" s="14"/>
     </row>
     <row r="31" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A31" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="25" t="str">
+      <c r="B31" s="30" t="str">
         <f>A29 &amp; "." &amp; B29 &amp; "." &amp; C29 &amp; "-" &amp; B30</f>
         <v>v1.2.0-Better_Default_2</v>
       </c>
-      <c r="C31" s="26"/>
+      <c r="C31" s="31"/>
       <c r="D31" s="14"/>
     </row>
     <row r="32" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2835,21 +2839,21 @@
       <c r="A35" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B35" s="25" t="s">
+      <c r="B35" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="C35" s="26"/>
+      <c r="C35" s="31"/>
       <c r="D35" s="14"/>
     </row>
     <row r="36" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A36" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B36" s="25" t="str">
+      <c r="B36" s="30" t="str">
         <f>A34 &amp; "." &amp; B34 &amp; "." &amp; C34 &amp; "-" &amp; B35</f>
         <v>v1.1.1-Better_Default</v>
       </c>
-      <c r="C36" s="26"/>
+      <c r="C36" s="31"/>
       <c r="D36" s="14"/>
     </row>
     <row r="37" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2889,30 +2893,25 @@
       <c r="A40" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="25" t="s">
+      <c r="B40" s="30" t="s">
         <v>60</v>
       </c>
-      <c r="C40" s="26"/>
+      <c r="C40" s="31"/>
       <c r="D40" s="14"/>
     </row>
     <row r="41" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A41" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B41" s="25" t="str">
+      <c r="B41" s="30" t="str">
         <f>A39 &amp; "." &amp; B39 &amp; "." &amp; C39 &amp; "-" &amp; B40</f>
         <v>v1.1.0-Better_Default</v>
       </c>
-      <c r="C41" s="26"/>
+      <c r="C41" s="31"/>
       <c r="D41" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2925,6 +2924,11 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Use pow-based sky_factor in lightmap shaders
Replace clamp(spread(1.0 - SkyFactor, 15), 0, 11) with spread(pow(1 - SkyFactor, 1.25), 15) across multiple lightmap.fsh files (1.21.2, 1.21.6, 1.21.9, 1.21.11, 26.1). This updates the sky light attenuation to use an exponent (1.25) and removes the previous hard clamp, altering the sky light falloff behavior for the shaders.
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6127E2A9-A6EF-471A-A31E-66E577BDC242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9172E0FF-F816-40AD-B97D-D3C8A97B9314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -225,10 +225,10 @@
     <t>Created Classic Reimagined Lite</t>
   </si>
   <si>
-    <t>Lite version</t>
-  </si>
-  <si>
     <t>Update fog/discard behavior and lightmap sampling</t>
+  </si>
+  <si>
+    <t>Replaced clamped skyfactor with pow-based sky_factor in lightmap shaders</t>
   </si>
 </sst>
 </file>
@@ -385,7 +385,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -416,7 +416,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -454,6 +453,21 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -654,11 +668,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="35"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="G1" s="2" t="s">
@@ -670,13 +684,11 @@
       <c r="K1" s="2"/>
     </row>
     <row r="2" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="25" t="s">
-        <v>63</v>
-      </c>
-      <c r="C2" s="26"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="25"/>
       <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
@@ -692,15 +704,12 @@
       <c r="K2" s="6"/>
     </row>
     <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A3" s="18" t="str">
+      <c r="A3" s="26" t="str">
         <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-build-" &amp; D3</f>
         <v>v10.0.11_1-build-5436-rt4</v>
       </c>
-      <c r="B3" s="27" t="str">
-        <f>"v1.2.7_1-build-" &amp; D3 &amp; "-" &amp; E3</f>
-        <v>v1.2.7_1-build-5436-rt4-26.1</v>
-      </c>
-      <c r="C3" s="28"/>
+      <c r="B3" s="31"/>
+      <c r="C3" s="27"/>
       <c r="D3" s="8" t="str">
         <f>SUM(2601,664,2026,145) &amp; "-rt4"</f>
         <v>5436-rt4</v>
@@ -732,11 +741,11 @@
       <c r="B4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="C4" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="20"/>
-      <c r="E4" s="21"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="20"/>
       <c r="G4" s="8" t="s">
         <v>11</v>
       </c>
@@ -759,11 +768,11 @@
         <v>62</v>
       </c>
       <c r="B5" s="6"/>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="23"/>
-      <c r="E5" s="24"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="23"/>
       <c r="G5" s="10" t="s">
         <v>13</v>
       </c>
@@ -777,7 +786,7 @@
     </row>
     <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -796,7 +805,9 @@
       <c r="K6" s="14"/>
     </row>
     <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A7" s="6"/>
+      <c r="A7" s="6" t="s">
+        <v>64</v>
+      </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
@@ -1899,11 +1910,12 @@
       <c r="K65" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A1:C1"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="C5:E5"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -1919,12 +1931,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
     </row>
     <row r="2" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
@@ -1963,21 +1975,21 @@
       <c r="A5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="28" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="30"/>
+      <c r="C5" s="29"/>
       <c r="D5" s="14"/>
     </row>
     <row r="6" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="29" t="str">
+      <c r="B6" s="28" t="str">
         <f>A4 &amp; "." &amp; B4 &amp; "." &amp; C4 &amp; "-" &amp; B5</f>
         <v>v6.0.7-Better_Default_6</v>
       </c>
-      <c r="C6" s="30"/>
+      <c r="C6" s="29"/>
       <c r="D6" s="14"/>
     </row>
     <row r="7" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2017,21 +2029,21 @@
       <c r="A10" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="B10" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="C10" s="30"/>
+      <c r="C10" s="29"/>
       <c r="D10" s="14"/>
     </row>
     <row r="11" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="29" t="str">
+      <c r="B11" s="28" t="str">
         <f>A9 &amp; "." &amp; B9 &amp; "." &amp; C9 &amp; "-" &amp; B10</f>
         <v>v1.4.0-Better_Default_5</v>
       </c>
-      <c r="C11" s="30"/>
+      <c r="C11" s="29"/>
       <c r="D11" s="14"/>
     </row>
     <row r="12" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2071,21 +2083,21 @@
       <c r="A15" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="29" t="s">
+      <c r="B15" s="28" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="30"/>
+      <c r="C15" s="29"/>
       <c r="D15" s="14"/>
     </row>
     <row r="16" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="29" t="str">
+      <c r="B16" s="28" t="str">
         <f>A14 &amp; "." &amp; B14 &amp; "." &amp; C14 &amp; "-" &amp; B15</f>
         <v>v1.3.0-Better_Default_4</v>
       </c>
-      <c r="C16" s="30"/>
+      <c r="C16" s="29"/>
       <c r="D16" s="14"/>
     </row>
     <row r="17" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2125,21 +2137,21 @@
       <c r="A20" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="29" t="s">
+      <c r="B20" s="28" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="30"/>
+      <c r="C20" s="29"/>
       <c r="D20" s="14"/>
     </row>
     <row r="21" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="29" t="str">
+      <c r="B21" s="28" t="str">
         <f>A19 &amp; "." &amp; B19 &amp; "." &amp; C19 &amp; "-" &amp; B20</f>
         <v>v1.2.2-Better_Default_3.1</v>
       </c>
-      <c r="C21" s="30"/>
+      <c r="C21" s="29"/>
       <c r="D21" s="14"/>
     </row>
     <row r="22" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2179,21 +2191,21 @@
       <c r="A25" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="29" t="s">
+      <c r="B25" s="28" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="30"/>
+      <c r="C25" s="29"/>
       <c r="D25" s="14"/>
     </row>
     <row r="26" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B26" s="29" t="str">
+      <c r="B26" s="28" t="str">
         <f>A24 &amp; "." &amp; B24 &amp; "." &amp; C24 &amp; "-" &amp; B25</f>
         <v>v1.2.1-Better_Default_3</v>
       </c>
-      <c r="C26" s="30"/>
+      <c r="C26" s="29"/>
       <c r="D26" s="14"/>
     </row>
     <row r="27" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2233,21 +2245,21 @@
       <c r="A30" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="29" t="s">
+      <c r="B30" s="28" t="s">
         <v>58</v>
       </c>
-      <c r="C30" s="30"/>
+      <c r="C30" s="29"/>
       <c r="D30" s="14"/>
     </row>
     <row r="31" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A31" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="29" t="str">
+      <c r="B31" s="28" t="str">
         <f>A29 &amp; "." &amp; B29 &amp; "." &amp; C29 &amp; "-" &amp; B30</f>
         <v>v1.2.0-Better_Default_2</v>
       </c>
-      <c r="C31" s="30"/>
+      <c r="C31" s="29"/>
       <c r="D31" s="14"/>
     </row>
     <row r="32" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2287,21 +2299,21 @@
       <c r="A35" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B35" s="29" t="s">
+      <c r="B35" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="C35" s="30"/>
+      <c r="C35" s="29"/>
       <c r="D35" s="14"/>
     </row>
     <row r="36" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A36" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B36" s="29" t="str">
+      <c r="B36" s="28" t="str">
         <f>A34 &amp; "." &amp; B34 &amp; "." &amp; C34 &amp; "-" &amp; B35</f>
         <v>v1.1.1-Better_Default</v>
       </c>
-      <c r="C36" s="30"/>
+      <c r="C36" s="29"/>
       <c r="D36" s="14"/>
     </row>
     <row r="37" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2341,30 +2353,25 @@
       <c r="A40" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="29" t="s">
+      <c r="B40" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="C40" s="30"/>
+      <c r="C40" s="29"/>
       <c r="D40" s="14"/>
     </row>
     <row r="41" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A41" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B41" s="29" t="str">
+      <c r="B41" s="28" t="str">
         <f>A39 &amp; "." &amp; B39 &amp; "." &amp; C39 &amp; "-" &amp; B40</f>
         <v>v1.1.0-Better_Default</v>
       </c>
-      <c r="C41" s="30"/>
+      <c r="C41" s="29"/>
       <c r="D41" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2377,6 +2384,11 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Bump resource pack format to 84 in pack.mcmeta
Update pack.mcmeta to use format 84 (update formats and min_format from 76 to 84) for the entries for "26.1_shaders" and "v10.0.11_1-Classic_Reimagined_10_SE_2.1" so the pack targets the newer resource pack format. Also includes an updated version_guide.xlsx file (binary change) reflecting the version/metadata update.
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9172E0FF-F816-40AD-B97D-D3C8A97B9314}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42FB4EBC-6186-4885-8E29-45ED60F40503}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Active releases and Changelog" sheetId="1" r:id="rId1"/>
@@ -21,12 +21,7 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -34,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="68">
   <si>
     <t>Current version in development</t>
   </si>
@@ -229,13 +224,22 @@
   </si>
   <si>
     <t>Replaced clamped skyfactor with pow-based sky_factor in lightmap shaders</t>
+  </si>
+  <si>
+    <t>Added classic mob sounds</t>
+  </si>
+  <si>
+    <t>fixed cat sounds</t>
+  </si>
+  <si>
+    <t>Updated pack format (26.1)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -416,6 +420,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -434,16 +447,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -453,21 +472,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -661,18 +665,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K65"/>
-  <sheetFormatPr defaultColWidth="27.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="27.25" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="91.42578125" customWidth="1"/>
-    <col min="2" max="2" width="54.85546875" customWidth="1"/>
+    <col min="1" max="1" width="91.375" customWidth="1"/>
+    <col min="2" max="2" width="54.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
+    <row r="1" spans="1:11" ht="16.5">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="35"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="20"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
       <c r="G1" s="2" t="s">
@@ -683,12 +687,12 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A2" s="24" t="s">
+    <row r="2" spans="1:11" ht="16.5">
+      <c r="A2" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="32"/>
-      <c r="C2" s="25"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="32"/>
       <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
@@ -703,16 +707,16 @@
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
     </row>
-    <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A3" s="26" t="str">
+    <row r="3" spans="1:11" ht="16.5">
+      <c r="A3" s="27" t="str">
         <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-build-" &amp; D3</f>
-        <v>v10.0.11_1-build-5436-rt4</v>
-      </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="27"/>
+        <v>v10.0.11_1-build-5456-rt4</v>
+      </c>
+      <c r="B3" s="28"/>
+      <c r="C3" s="29"/>
       <c r="D3" s="8" t="str">
-        <f>SUM(2601,664,2026,145) &amp; "-rt4"</f>
-        <v>5436-rt4</v>
+        <f>SUM(2601,664,2026,165) &amp; "-rt4"</f>
+        <v>5456-rt4</v>
       </c>
       <c r="E3" s="7">
         <f>K4</f>
@@ -734,18 +738,18 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" ht="16.5">
       <c r="A4" s="9" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="19"/>
-      <c r="E4" s="20"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="23"/>
       <c r="G4" s="8" t="s">
         <v>11</v>
       </c>
@@ -757,22 +761,22 @@
       </c>
       <c r="J4" s="8" t="str">
         <f>D3</f>
-        <v>5436-rt4</v>
+        <v>5456-rt4</v>
       </c>
       <c r="K4" s="8">
         <v>26.1</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="16.5">
       <c r="A5" s="6" t="s">
         <v>62</v>
       </c>
       <c r="B5" s="6"/>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="23"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="26"/>
       <c r="G5" s="10" t="s">
         <v>13</v>
       </c>
@@ -784,7 +788,7 @@
       <c r="J5" s="13"/>
       <c r="K5" s="14"/>
     </row>
-    <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" ht="16.5">
       <c r="A6" s="6" t="s">
         <v>63</v>
       </c>
@@ -804,7 +808,7 @@
       <c r="J6" s="13"/>
       <c r="K6" s="14"/>
     </row>
-    <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="16.5">
       <c r="A7" s="6" t="s">
         <v>64</v>
       </c>
@@ -818,14 +822,16 @@
       </c>
       <c r="H7" s="11" t="str">
         <f>H6 &amp; "-build-" &amp; J4</f>
-        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5436-rt4</v>
+        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5456-rt4</v>
       </c>
       <c r="I7" s="12"/>
       <c r="J7" s="13"/>
       <c r="K7" s="6"/>
     </row>
-    <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A8" s="6"/>
+    <row r="8" spans="1:11" ht="16.5">
+      <c r="A8" s="6" t="s">
+        <v>65</v>
+      </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
       <c r="D8" s="6"/>
@@ -839,8 +845,10 @@
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
     </row>
-    <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="6"/>
+    <row r="9" spans="1:11" ht="16.5">
+      <c r="A9" s="6" t="s">
+        <v>66</v>
+      </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
@@ -860,8 +868,10 @@
       </c>
       <c r="K9" s="6"/>
     </row>
-    <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="6"/>
+    <row r="10" spans="1:11" ht="16.5">
+      <c r="A10" s="6" t="s">
+        <v>67</v>
+      </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
@@ -875,14 +885,14 @@
       </c>
       <c r="I10" s="8" t="str">
         <f>J4</f>
-        <v>5436-rt4</v>
+        <v>5456-rt4</v>
       </c>
       <c r="J10" s="8" t="s">
         <v>18</v>
       </c>
       <c r="K10" s="6"/>
     </row>
-    <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" ht="16.5">
       <c r="A11" s="6"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -900,7 +910,7 @@
       <c r="J11" s="14"/>
       <c r="K11" s="6"/>
     </row>
-    <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" ht="16.5">
       <c r="A12" s="6"/>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -918,7 +928,7 @@
       <c r="J12" s="14"/>
       <c r="K12" s="6"/>
     </row>
-    <row r="13" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="16.5">
       <c r="A13" s="6"/>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
@@ -930,13 +940,13 @@
       </c>
       <c r="H13" s="15" t="str">
         <f>H12 &amp; "-build-" &amp; I10</f>
-        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5436-rt4</v>
+        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5456-rt4</v>
       </c>
       <c r="I13" s="16"/>
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
     </row>
-    <row r="14" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" ht="16.5">
       <c r="A14" s="6"/>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -957,7 +967,7 @@
       </c>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="16.5">
       <c r="A15" s="6"/>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -972,14 +982,14 @@
       </c>
       <c r="I15" s="8" t="str">
         <f>I10</f>
-        <v>5436-rt4</v>
+        <v>5456-rt4</v>
       </c>
       <c r="J15" s="8" t="s">
         <v>19</v>
       </c>
       <c r="K15" s="6"/>
     </row>
-    <row r="16" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="16.5">
       <c r="A16" s="6"/>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -997,7 +1007,7 @@
       <c r="J16" s="14"/>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="16.5">
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -1015,7 +1025,7 @@
       <c r="J17" s="14"/>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" ht="16.5">
       <c r="A18" s="6"/>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -1027,13 +1037,13 @@
       </c>
       <c r="H18" s="15" t="str">
         <f>H17 &amp; "-build-" &amp; I15</f>
-        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5436-rt4</v>
+        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5456-rt4</v>
       </c>
       <c r="I18" s="16"/>
       <c r="J18" s="6"/>
       <c r="K18" s="6"/>
     </row>
-    <row r="19" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="16.5">
       <c r="A19" s="6"/>
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
@@ -1054,7 +1064,7 @@
       </c>
       <c r="K19" s="6"/>
     </row>
-    <row r="20" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" ht="16.5">
       <c r="A20" s="6"/>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
@@ -1069,14 +1079,14 @@
       </c>
       <c r="I20" s="8" t="str">
         <f>I15</f>
-        <v>5436-rt4</v>
+        <v>5456-rt4</v>
       </c>
       <c r="J20" s="8" t="s">
         <v>20</v>
       </c>
       <c r="K20" s="6"/>
     </row>
-    <row r="21" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" ht="16.5">
       <c r="A21" s="6"/>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -1094,7 +1104,7 @@
       <c r="J21" s="14"/>
       <c r="K21" s="6"/>
     </row>
-    <row r="22" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" ht="16.5">
       <c r="A22" s="6"/>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
@@ -1112,7 +1122,7 @@
       <c r="J22" s="14"/>
       <c r="K22" s="6"/>
     </row>
-    <row r="23" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" ht="16.5">
       <c r="A23" s="6"/>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
@@ -1124,13 +1134,13 @@
       </c>
       <c r="H23" s="15" t="str">
         <f>H22 &amp; "-build-" &amp; I20</f>
-        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5436-rt4</v>
+        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5456-rt4</v>
       </c>
       <c r="I23" s="16"/>
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
     </row>
-    <row r="24" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" ht="16.5">
       <c r="A24" s="6"/>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -1151,7 +1161,7 @@
       </c>
       <c r="K24" s="6"/>
     </row>
-    <row r="25" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" ht="16.5">
       <c r="A25" s="6"/>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -1166,14 +1176,14 @@
       </c>
       <c r="I25" s="8" t="str">
         <f>I20</f>
-        <v>5436-rt4</v>
+        <v>5456-rt4</v>
       </c>
       <c r="J25" s="8" t="s">
         <v>21</v>
       </c>
       <c r="K25" s="6"/>
     </row>
-    <row r="26" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" ht="16.5">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -1191,7 +1201,7 @@
       <c r="J26" s="14"/>
       <c r="K26" s="6"/>
     </row>
-    <row r="27" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" ht="16.5">
       <c r="A27" s="6"/>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -1209,7 +1219,7 @@
       <c r="J27" s="14"/>
       <c r="K27" s="6"/>
     </row>
-    <row r="28" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" ht="16.5">
       <c r="A28" s="6"/>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
@@ -1221,13 +1231,13 @@
       </c>
       <c r="H28" s="15" t="str">
         <f>H27 &amp; "-build-" &amp; I25</f>
-        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5436-rt4</v>
+        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5456-rt4</v>
       </c>
       <c r="I28" s="16"/>
       <c r="J28" s="6"/>
       <c r="K28" s="6"/>
     </row>
-    <row r="29" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" ht="16.5">
       <c r="A29" s="6"/>
       <c r="B29" s="6"/>
       <c r="C29" s="6"/>
@@ -1242,7 +1252,7 @@
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
     </row>
-    <row r="30" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" ht="16.5">
       <c r="A30" s="6"/>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
@@ -1263,7 +1273,7 @@
       </c>
       <c r="K30" s="6"/>
     </row>
-    <row r="31" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" ht="16.5">
       <c r="A31" s="6"/>
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
@@ -1278,14 +1288,14 @@
       </c>
       <c r="I31" s="8" t="str">
         <f>I25</f>
-        <v>5436-rt4</v>
+        <v>5456-rt4</v>
       </c>
       <c r="J31" s="8" t="s">
         <v>23</v>
       </c>
       <c r="K31" s="6"/>
     </row>
-    <row r="32" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" ht="16.5">
       <c r="A32" s="6"/>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
@@ -1303,7 +1313,7 @@
       <c r="J32" s="14"/>
       <c r="K32" s="6"/>
     </row>
-    <row r="33" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" ht="16.5">
       <c r="A33" s="6"/>
       <c r="B33" s="6"/>
       <c r="C33" s="6"/>
@@ -1321,7 +1331,7 @@
       <c r="J33" s="14"/>
       <c r="K33" s="6"/>
     </row>
-    <row r="34" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" ht="16.5">
       <c r="A34" s="6"/>
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
@@ -1333,13 +1343,13 @@
       </c>
       <c r="H34" s="15" t="str">
         <f>H33 &amp; "-build-" &amp; I31</f>
-        <v>v10.0.3-Classic_Reimagined_10_SE-build-5436-rt4</v>
+        <v>v10.0.3-Classic_Reimagined_10_SE-build-5456-rt4</v>
       </c>
       <c r="I34" s="16"/>
       <c r="J34" s="6"/>
       <c r="K34" s="6"/>
     </row>
-    <row r="35" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" ht="16.5">
       <c r="A35" s="6"/>
       <c r="B35" s="6"/>
       <c r="C35" s="6"/>
@@ -1354,7 +1364,7 @@
       <c r="J35" s="6"/>
       <c r="K35" s="6"/>
     </row>
-    <row r="36" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" ht="16.5">
       <c r="A36" s="6"/>
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
@@ -1375,7 +1385,7 @@
       </c>
       <c r="K36" s="6"/>
     </row>
-    <row r="37" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" ht="16.5">
       <c r="A37" s="6"/>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -1390,14 +1400,14 @@
       </c>
       <c r="I37" s="8" t="str">
         <f>I31</f>
-        <v>5436-rt4</v>
+        <v>5456-rt4</v>
       </c>
       <c r="J37" s="8" t="s">
         <v>25</v>
       </c>
       <c r="K37" s="6"/>
     </row>
-    <row r="38" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" ht="16.5">
       <c r="A38" s="6"/>
       <c r="B38" s="6"/>
       <c r="C38" s="6"/>
@@ -1414,7 +1424,7 @@
       <c r="J38" s="14"/>
       <c r="K38" s="6"/>
     </row>
-    <row r="39" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" ht="16.5">
       <c r="A39" s="6"/>
       <c r="B39" s="6"/>
       <c r="C39" s="6"/>
@@ -1432,7 +1442,7 @@
       <c r="J39" s="14"/>
       <c r="K39" s="6"/>
     </row>
-    <row r="40" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" ht="16.5">
       <c r="A40" s="6"/>
       <c r="B40" s="6"/>
       <c r="C40" s="6"/>
@@ -1444,13 +1454,13 @@
       </c>
       <c r="H40" s="15" t="str">
         <f>H39 &amp; "-build-" &amp; I37</f>
-        <v>v10.0.2-Classic_Reimagined_10s-build-5436-rt4</v>
+        <v>v10.0.2-Classic_Reimagined_10s-build-5456-rt4</v>
       </c>
       <c r="I40" s="16"/>
       <c r="J40" s="6"/>
       <c r="K40" s="6"/>
     </row>
-    <row r="41" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" ht="16.5">
       <c r="A41" s="6"/>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
@@ -1465,7 +1475,7 @@
       <c r="J41" s="6"/>
       <c r="K41" s="6"/>
     </row>
-    <row r="42" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" ht="16.5">
       <c r="A42" s="6"/>
       <c r="B42" s="6"/>
       <c r="C42" s="6"/>
@@ -1486,7 +1496,7 @@
       </c>
       <c r="K42" s="6"/>
     </row>
-    <row r="43" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" ht="16.5">
       <c r="A43" s="6"/>
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
@@ -1501,14 +1511,14 @@
       </c>
       <c r="I43" s="8" t="str">
         <f>I37</f>
-        <v>5436-rt4</v>
+        <v>5456-rt4</v>
       </c>
       <c r="J43" s="8" t="s">
         <v>28</v>
       </c>
       <c r="K43" s="6"/>
     </row>
-    <row r="44" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" ht="16.5">
       <c r="A44" s="6"/>
       <c r="B44" s="6"/>
       <c r="C44" s="6"/>
@@ -1525,7 +1535,7 @@
       <c r="J44" s="14"/>
       <c r="K44" s="6"/>
     </row>
-    <row r="45" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" ht="16.5">
       <c r="A45" s="6"/>
       <c r="B45" s="6"/>
       <c r="C45" s="6"/>
@@ -1543,7 +1553,7 @@
       <c r="J45" s="14"/>
       <c r="K45" s="6"/>
     </row>
-    <row r="46" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" ht="16.5">
       <c r="A46" s="6"/>
       <c r="B46" s="6"/>
       <c r="C46" s="6"/>
@@ -1555,13 +1565,13 @@
       </c>
       <c r="H46" s="15" t="str">
         <f>H45 &amp; "-build-" &amp; I43</f>
-        <v>v10.0.1-Classic_Reimagined_10-build-5436-rt4</v>
+        <v>v10.0.1-Classic_Reimagined_10-build-5456-rt4</v>
       </c>
       <c r="I46" s="16"/>
       <c r="J46" s="6"/>
       <c r="K46" s="6"/>
     </row>
-    <row r="47" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" ht="16.5">
       <c r="A47" s="6"/>
       <c r="B47" s="6"/>
       <c r="C47" s="6"/>
@@ -1576,7 +1586,7 @@
       <c r="J47" s="2"/>
       <c r="K47" s="6"/>
     </row>
-    <row r="48" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" ht="16.5">
       <c r="A48" s="6"/>
       <c r="B48" s="6"/>
       <c r="C48" s="6"/>
@@ -1591,7 +1601,7 @@
       <c r="J48" s="6"/>
       <c r="K48" s="6"/>
     </row>
-    <row r="49" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" ht="16.5">
       <c r="A49" s="6"/>
       <c r="B49" s="6"/>
       <c r="C49" s="6"/>
@@ -1612,7 +1622,7 @@
       </c>
       <c r="K49" s="6"/>
     </row>
-    <row r="50" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" ht="16.5">
       <c r="A50" s="6"/>
       <c r="B50" s="6"/>
       <c r="C50" s="6"/>
@@ -1627,14 +1637,14 @@
       </c>
       <c r="I50" s="8" t="str">
         <f>I43</f>
-        <v>5436-rt4</v>
+        <v>5456-rt4</v>
       </c>
       <c r="J50" s="8" t="s">
         <v>33</v>
       </c>
       <c r="K50" s="6"/>
     </row>
-    <row r="51" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" ht="16.5">
       <c r="A51" s="6"/>
       <c r="B51" s="6"/>
       <c r="C51" s="6"/>
@@ -1651,7 +1661,7 @@
       <c r="J51" s="14"/>
       <c r="K51" s="6"/>
     </row>
-    <row r="52" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" ht="16.5">
       <c r="A52" s="6"/>
       <c r="B52" s="6"/>
       <c r="C52" s="6"/>
@@ -1669,7 +1679,7 @@
       <c r="J52" s="14"/>
       <c r="K52" s="6"/>
     </row>
-    <row r="53" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" ht="16.5">
       <c r="A53" s="6"/>
       <c r="B53" s="6"/>
       <c r="C53" s="6"/>
@@ -1681,13 +1691,13 @@
       </c>
       <c r="H53" s="15" t="str">
         <f>H52 &amp; "-build-" &amp; I50</f>
-        <v>v8.10.32-Classic_Reimagined_8-build-5436-rt4</v>
+        <v>v8.10.32-Classic_Reimagined_8-build-5456-rt4</v>
       </c>
       <c r="I53" s="16"/>
       <c r="J53" s="6"/>
       <c r="K53" s="6"/>
     </row>
-    <row r="54" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" ht="16.5">
       <c r="A54" s="6"/>
       <c r="B54" s="6"/>
       <c r="C54" s="6"/>
@@ -1702,7 +1712,7 @@
       <c r="J54" s="6"/>
       <c r="K54" s="6"/>
     </row>
-    <row r="55" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" ht="16.5">
       <c r="A55" s="6"/>
       <c r="B55" s="6"/>
       <c r="C55" s="6"/>
@@ -1723,7 +1733,7 @@
       </c>
       <c r="K55" s="6"/>
     </row>
-    <row r="56" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" ht="16.5">
       <c r="A56" s="6"/>
       <c r="B56" s="6"/>
       <c r="C56" s="6"/>
@@ -1738,14 +1748,14 @@
       </c>
       <c r="I56" s="8" t="str">
         <f>I50</f>
-        <v>5436-rt4</v>
+        <v>5456-rt4</v>
       </c>
       <c r="J56" s="8" t="s">
         <v>35</v>
       </c>
       <c r="K56" s="6"/>
     </row>
-    <row r="57" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" ht="16.5">
       <c r="A57" s="6"/>
       <c r="B57" s="6"/>
       <c r="C57" s="6"/>
@@ -1762,7 +1772,7 @@
       <c r="J57" s="14"/>
       <c r="K57" s="6"/>
     </row>
-    <row r="58" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" ht="16.5">
       <c r="A58" s="6"/>
       <c r="B58" s="6"/>
       <c r="C58" s="6"/>
@@ -1780,7 +1790,7 @@
       <c r="J58" s="14"/>
       <c r="K58" s="6"/>
     </row>
-    <row r="59" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" ht="16.5">
       <c r="A59" s="6"/>
       <c r="B59" s="6"/>
       <c r="C59" s="6"/>
@@ -1792,13 +1802,13 @@
       </c>
       <c r="H59" s="15" t="str">
         <f>H58 &amp; "-build-" &amp; I56</f>
-        <v>v8.10.31-Classic_Reimagined_8-build-5436-rt4</v>
+        <v>v8.10.31-Classic_Reimagined_8-build-5456-rt4</v>
       </c>
       <c r="I59" s="16"/>
       <c r="J59" s="6"/>
       <c r="K59" s="6"/>
     </row>
-    <row r="60" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" ht="16.5">
       <c r="A60" s="6"/>
       <c r="B60" s="6"/>
       <c r="C60" s="6"/>
@@ -1813,7 +1823,7 @@
       <c r="J60" s="17"/>
       <c r="K60" s="6"/>
     </row>
-    <row r="61" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" ht="16.5">
       <c r="A61" s="6"/>
       <c r="B61" s="6"/>
       <c r="C61" s="6"/>
@@ -1834,7 +1844,7 @@
       </c>
       <c r="K61" s="6"/>
     </row>
-    <row r="62" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" ht="16.5">
       <c r="A62" s="6"/>
       <c r="B62" s="6"/>
       <c r="C62" s="6"/>
@@ -1849,14 +1859,14 @@
       </c>
       <c r="I62" s="8" t="str">
         <f>I56</f>
-        <v>5436-rt4</v>
+        <v>5456-rt4</v>
       </c>
       <c r="J62" s="8" t="s">
         <v>38</v>
       </c>
       <c r="K62" s="6"/>
     </row>
-    <row r="63" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" ht="16.5">
       <c r="A63" s="6"/>
       <c r="B63" s="6"/>
       <c r="C63" s="6"/>
@@ -1873,7 +1883,7 @@
       <c r="J63" s="14"/>
       <c r="K63" s="6"/>
     </row>
-    <row r="64" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" ht="16.5">
       <c r="A64" s="6"/>
       <c r="B64" s="6"/>
       <c r="C64" s="6"/>
@@ -1891,7 +1901,7 @@
       <c r="J64" s="14"/>
       <c r="K64" s="6"/>
     </row>
-    <row r="65" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:11" ht="16.5">
       <c r="A65" s="6"/>
       <c r="B65" s="6"/>
       <c r="C65" s="6"/>
@@ -1903,7 +1913,7 @@
       </c>
       <c r="H65" s="15" t="str">
         <f>H64 &amp; "-build-" &amp; I62</f>
-        <v>v7.11.3-Better_Default_7-build-5436-rt4</v>
+        <v>v7.11.3-Better_Default_7-build-5456-rt4</v>
       </c>
       <c r="I65" s="16"/>
       <c r="J65" s="6"/>
@@ -1925,25 +1935,25 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D41"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="4" width="27.42578125" customWidth="1"/>
+    <col min="1" max="4" width="27.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+    <row r="1" spans="1:4" ht="16.5">
+      <c r="A1" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-    </row>
-    <row r="2" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+    </row>
+    <row r="2" spans="1:4" ht="16.5">
       <c r="A2" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="16.5">
       <c r="A3" s="4" t="s">
         <v>17</v>
       </c>
@@ -1957,7 +1967,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="16.5">
       <c r="A4" s="8" t="s">
         <v>43</v>
       </c>
@@ -1971,33 +1981,33 @@
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="16.5">
       <c r="A5" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="28" t="s">
+      <c r="B5" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="29"/>
+      <c r="C5" s="34"/>
       <c r="D5" s="14"/>
     </row>
-    <row r="6" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="16.5">
       <c r="A6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="28" t="str">
+      <c r="B6" s="33" t="str">
         <f>A4 &amp; "." &amp; B4 &amp; "." &amp; C4 &amp; "-" &amp; B5</f>
         <v>v6.0.7-Better_Default_6</v>
       </c>
-      <c r="C6" s="29"/>
+      <c r="C6" s="34"/>
       <c r="D6" s="14"/>
     </row>
-    <row r="7" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="16.5">
       <c r="A7" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" ht="16.5">
       <c r="A8" s="4" t="s">
         <v>17</v>
       </c>
@@ -2011,7 +2021,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="16.5">
       <c r="A9" s="8" t="s">
         <v>47</v>
       </c>
@@ -2025,33 +2035,33 @@
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="16.5">
       <c r="A10" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="33" t="s">
         <v>49</v>
       </c>
-      <c r="C10" s="29"/>
+      <c r="C10" s="34"/>
       <c r="D10" s="14"/>
     </row>
-    <row r="11" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="16.5">
       <c r="A11" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="28" t="str">
+      <c r="B11" s="33" t="str">
         <f>A9 &amp; "." &amp; B9 &amp; "." &amp; C9 &amp; "-" &amp; B10</f>
         <v>v1.4.0-Better_Default_5</v>
       </c>
-      <c r="C11" s="29"/>
+      <c r="C11" s="34"/>
       <c r="D11" s="14"/>
     </row>
-    <row r="12" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" ht="16.5">
       <c r="A12" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" ht="16.5">
       <c r="A13" s="4" t="s">
         <v>17</v>
       </c>
@@ -2065,7 +2075,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="16.5">
       <c r="A14" s="8" t="s">
         <v>47</v>
       </c>
@@ -2079,33 +2089,33 @@
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" ht="16.5">
       <c r="A15" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="28" t="s">
+      <c r="B15" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="29"/>
+      <c r="C15" s="34"/>
       <c r="D15" s="14"/>
     </row>
-    <row r="16" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" ht="16.5">
       <c r="A16" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="28" t="str">
+      <c r="B16" s="33" t="str">
         <f>A14 &amp; "." &amp; B14 &amp; "." &amp; C14 &amp; "-" &amp; B15</f>
         <v>v1.3.0-Better_Default_4</v>
       </c>
-      <c r="C16" s="29"/>
+      <c r="C16" s="34"/>
       <c r="D16" s="14"/>
     </row>
-    <row r="17" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" ht="16.5">
       <c r="A17" s="5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" ht="16.5">
       <c r="A18" s="4" t="s">
         <v>17</v>
       </c>
@@ -2119,7 +2129,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" ht="16.5">
       <c r="A19" s="8" t="s">
         <v>47</v>
       </c>
@@ -2133,33 +2143,33 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" ht="16.5">
       <c r="A20" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="29"/>
+      <c r="C20" s="34"/>
       <c r="D20" s="14"/>
     </row>
-    <row r="21" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" ht="16.5">
       <c r="A21" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="28" t="str">
+      <c r="B21" s="33" t="str">
         <f>A19 &amp; "." &amp; B19 &amp; "." &amp; C19 &amp; "-" &amp; B20</f>
         <v>v1.2.2-Better_Default_3.1</v>
       </c>
-      <c r="C21" s="29"/>
+      <c r="C21" s="34"/>
       <c r="D21" s="14"/>
     </row>
-    <row r="22" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" ht="16.5">
       <c r="A22" s="5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" ht="16.5">
       <c r="A23" s="4" t="s">
         <v>17</v>
       </c>
@@ -2173,7 +2183,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" ht="16.5">
       <c r="A24" s="8" t="s">
         <v>47</v>
       </c>
@@ -2187,33 +2197,33 @@
         <v>1.1599999999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" ht="16.5">
       <c r="A25" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="28" t="s">
+      <c r="B25" s="33" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="29"/>
+      <c r="C25" s="34"/>
       <c r="D25" s="14"/>
     </row>
-    <row r="26" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" ht="16.5">
       <c r="A26" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B26" s="28" t="str">
+      <c r="B26" s="33" t="str">
         <f>A24 &amp; "." &amp; B24 &amp; "." &amp; C24 &amp; "-" &amp; B25</f>
         <v>v1.2.1-Better_Default_3</v>
       </c>
-      <c r="C26" s="29"/>
+      <c r="C26" s="34"/>
       <c r="D26" s="14"/>
     </row>
-    <row r="27" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" ht="16.5">
       <c r="A27" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" ht="16.5">
       <c r="A28" s="4" t="s">
         <v>17</v>
       </c>
@@ -2227,7 +2237,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" ht="16.5">
       <c r="A29" s="8" t="s">
         <v>47</v>
       </c>
@@ -2241,33 +2251,33 @@
         <v>1.1499999999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" ht="16.5">
       <c r="A30" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="28" t="s">
+      <c r="B30" s="33" t="s">
         <v>58</v>
       </c>
-      <c r="C30" s="29"/>
+      <c r="C30" s="34"/>
       <c r="D30" s="14"/>
     </row>
-    <row r="31" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" ht="16.5">
       <c r="A31" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="28" t="str">
+      <c r="B31" s="33" t="str">
         <f>A29 &amp; "." &amp; B29 &amp; "." &amp; C29 &amp; "-" &amp; B30</f>
         <v>v1.2.0-Better_Default_2</v>
       </c>
-      <c r="C31" s="29"/>
+      <c r="C31" s="34"/>
       <c r="D31" s="14"/>
     </row>
-    <row r="32" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" ht="16.5">
       <c r="A32" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" ht="16.5">
       <c r="A33" s="4" t="s">
         <v>17</v>
       </c>
@@ -2281,7 +2291,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" ht="16.5">
       <c r="A34" s="8" t="s">
         <v>47</v>
       </c>
@@ -2295,33 +2305,33 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" ht="16.5">
       <c r="A35" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B35" s="28" t="s">
+      <c r="B35" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="C35" s="29"/>
+      <c r="C35" s="34"/>
       <c r="D35" s="14"/>
     </row>
-    <row r="36" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" ht="16.5">
       <c r="A36" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B36" s="28" t="str">
+      <c r="B36" s="33" t="str">
         <f>A34 &amp; "." &amp; B34 &amp; "." &amp; C34 &amp; "-" &amp; B35</f>
         <v>v1.1.1-Better_Default</v>
       </c>
-      <c r="C36" s="29"/>
+      <c r="C36" s="34"/>
       <c r="D36" s="14"/>
     </row>
-    <row r="37" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" ht="16.5">
       <c r="A37" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" ht="16.5">
       <c r="A38" s="4" t="s">
         <v>17</v>
       </c>
@@ -2335,7 +2345,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" ht="16.5">
       <c r="A39" s="8" t="s">
         <v>47</v>
       </c>
@@ -2349,25 +2359,25 @@
         <v>1.1299999999999999</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" ht="16.5">
       <c r="A40" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="28" t="s">
+      <c r="B40" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="C40" s="29"/>
+      <c r="C40" s="34"/>
       <c r="D40" s="14"/>
     </row>
-    <row r="41" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" ht="16.5">
       <c r="A41" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B41" s="28" t="str">
+      <c r="B41" s="33" t="str">
         <f>A39 &amp; "." &amp; B39 &amp; "." &amp; C39 &amp; "-" &amp; B40</f>
         <v>v1.1.0-Better_Default</v>
       </c>
-      <c r="C41" s="29"/>
+      <c r="C41" s="34"/>
       <c r="D41" s="14"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update grass textures; add baby entity textures
Replace and modify grass textures (grass.png, grass_0.png, grass_1.png) and add .mcmeta files setting "mipmap_strategy": "strict_cutout". Remove older .mcmeta entries in the v10.0.10 release that used the "mean" strategy. Add a large set of new baby/variant entity textures under v10.0.11_1-Classic_Reimagined_10_SE_2.1 (animals, horses, villagers, zombies, equipment overlays, etc.) to support the new release assets.
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42FB4EBC-6186-4885-8E29-45ED60F40503}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{209B862D-2829-40BE-B36E-88771061853A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,12 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -29,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="70">
   <si>
     <t>Current version in development</t>
   </si>
@@ -233,6 +238,12 @@
   </si>
   <si>
     <t>Updated pack format (26.1)</t>
+  </si>
+  <si>
+    <t>Fixed grass rendering</t>
+  </si>
+  <si>
+    <t>Added baby mob textures</t>
   </si>
 </sst>
 </file>
@@ -769,7 +780,7 @@
     </row>
     <row r="5" spans="1:11" ht="16.5">
       <c r="A5" s="6" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="24" t="s">
@@ -790,7 +801,7 @@
     </row>
     <row r="6" spans="1:11" ht="16.5">
       <c r="A6" s="6" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -810,7 +821,7 @@
     </row>
     <row r="7" spans="1:11" ht="16.5">
       <c r="A7" s="6" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -830,7 +841,7 @@
     </row>
     <row r="8" spans="1:11" ht="16.5">
       <c r="A8" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -847,7 +858,7 @@
     </row>
     <row r="9" spans="1:11" ht="16.5">
       <c r="A9" s="6" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -870,7 +881,7 @@
     </row>
     <row r="10" spans="1:11" ht="16.5">
       <c r="A10" s="6" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -893,7 +904,9 @@
       <c r="K10" s="6"/>
     </row>
     <row r="11" spans="1:11" ht="16.5">
-      <c r="A11" s="6"/>
+      <c r="A11" s="6" t="s">
+        <v>63</v>
+      </c>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
       <c r="D11" s="6"/>
@@ -911,7 +924,9 @@
       <c r="K11" s="6"/>
     </row>
     <row r="12" spans="1:11" ht="16.5">
-      <c r="A12" s="6"/>
+      <c r="A12" s="6" t="s">
+        <v>67</v>
+      </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
@@ -1920,6 +1935,9 @@
       <c r="K65" s="6"/>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:A12">
+    <sortCondition ref="A12"/>
+  </sortState>
   <mergeCells count="5">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="C4:E4"/>
@@ -2382,6 +2400,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2394,11 +2417,6 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Remove fire/water textures, update metadata
Delete legacy block textures and their .mcmeta files (campfire_fire, fire_0, fire_1, soul_campfire_fire, soul_fire_0, soul_fire_1, and water.png). Update water_flow.png (binary changed) and simplify its .mcmeta animation settings to only include width and height (removed interpolate and frametime).
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18EEB19B-E37D-49D9-BAEB-1A46457EB369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6F12E9D-D1A4-4E9D-8B99-F7171A8B5DB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="67">
   <si>
     <t>Current version in development</t>
   </si>
@@ -222,38 +222,26 @@
     <t>Better Default 1.1</t>
   </si>
   <si>
-    <t>Created Classic Reimagined Lite</t>
-  </si>
-  <si>
-    <t>Update fog/discard behavior and lightmap sampling</t>
-  </si>
-  <si>
-    <t>Replaced clamped skyfactor with pow-based sky_factor in lightmap shaders</t>
-  </si>
-  <si>
-    <t>Added classic mob sounds</t>
-  </si>
-  <si>
-    <t>fixed cat sounds</t>
-  </si>
-  <si>
-    <t>Updated pack format (26.1)</t>
-  </si>
-  <si>
-    <t>Fixed grass rendering</t>
-  </si>
-  <si>
-    <t>Added baby mob textures</t>
-  </si>
-  <si>
-    <t>Fixed compatibility issue with 26.1</t>
+    <t>Optimized textures for Vulkan's memory buffer</t>
+  </si>
+  <si>
+    <t>Improved shaders</t>
+  </si>
+  <si>
+    <t>Added 26.2 compatibility</t>
+  </si>
+  <si>
+    <t>Simplified animated textures to less sprites</t>
+  </si>
+  <si>
+    <t>Optimized VRAM usage by 17%</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -679,13 +667,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K65"/>
-  <sheetFormatPr defaultColWidth="27.25" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="27.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="91.375" customWidth="1"/>
-    <col min="2" max="2" width="54.875" customWidth="1"/>
+    <col min="1" max="1" width="91.42578125" customWidth="1"/>
+    <col min="2" max="2" width="54.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="16.5">
+    <row r="1" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
@@ -701,7 +689,7 @@
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:11" ht="16.5">
+    <row r="2" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2" s="30" t="s">
         <v>2</v>
       </c>
@@ -721,16 +709,16 @@
       <c r="J2" s="6"/>
       <c r="K2" s="6"/>
     </row>
-    <row r="3" spans="1:11" ht="16.5">
+    <row r="3" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" s="27" t="str">
         <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-build-" &amp; D3</f>
-        <v>v10.0.11_1-build-5459-rt4</v>
+        <v>v10.0.11_1-build-5460-rt4</v>
       </c>
       <c r="B3" s="28"/>
       <c r="C3" s="29"/>
       <c r="D3" s="8" t="str">
-        <f>SUM(2601,664,2026,168) &amp; "-rt4"</f>
-        <v>5459-rt4</v>
+        <f>SUM(2601,664,2026,169) &amp; "-rt4"</f>
+        <v>5460-rt4</v>
       </c>
       <c r="E3" s="7">
         <f>K4</f>
@@ -752,7 +740,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="16.5">
+    <row r="4" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>8</v>
       </c>
@@ -775,15 +763,15 @@
       </c>
       <c r="J4" s="8" t="str">
         <f>D3</f>
-        <v>5459-rt4</v>
+        <v>5460-rt4</v>
       </c>
       <c r="K4" s="8">
         <v>26.1</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="16.5">
+    <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="24" t="s">
@@ -802,9 +790,9 @@
       <c r="J5" s="13"/>
       <c r="K5" s="14"/>
     </row>
-    <row r="6" spans="1:11" ht="16.5">
+    <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -822,7 +810,7 @@
       <c r="J6" s="13"/>
       <c r="K6" s="14"/>
     </row>
-    <row r="7" spans="1:11" ht="16.5">
+    <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>62</v>
       </c>
@@ -836,13 +824,13 @@
       </c>
       <c r="H7" s="11" t="str">
         <f>H6 &amp; "-build-" &amp; J4</f>
-        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5459-rt4</v>
+        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5460-rt4</v>
       </c>
       <c r="I7" s="12"/>
       <c r="J7" s="13"/>
       <c r="K7" s="6"/>
     </row>
-    <row r="8" spans="1:11" ht="16.5">
+    <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>66</v>
       </c>
@@ -859,9 +847,9 @@
       <c r="J8" s="6"/>
       <c r="K8" s="6"/>
     </row>
-    <row r="9" spans="1:11" ht="16.5">
+    <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -882,10 +870,8 @@
       </c>
       <c r="K9" s="6"/>
     </row>
-    <row r="10" spans="1:11" ht="16.5">
-      <c r="A10" s="6" t="s">
-        <v>68</v>
-      </c>
+    <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A10" s="6"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
@@ -899,17 +885,15 @@
       </c>
       <c r="I10" s="8" t="str">
         <f>J4</f>
-        <v>5459-rt4</v>
+        <v>5460-rt4</v>
       </c>
       <c r="J10" s="8" t="s">
         <v>18</v>
       </c>
       <c r="K10" s="6"/>
     </row>
-    <row r="11" spans="1:11" ht="16.5">
-      <c r="A11" s="6" t="s">
-        <v>64</v>
-      </c>
+    <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A11" s="6"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
       <c r="D11" s="6"/>
@@ -926,10 +910,8 @@
       <c r="J11" s="14"/>
       <c r="K11" s="6"/>
     </row>
-    <row r="12" spans="1:11" ht="16.5">
-      <c r="A12" s="6" t="s">
-        <v>63</v>
-      </c>
+    <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A12" s="6"/>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
@@ -946,10 +928,8 @@
       <c r="J12" s="14"/>
       <c r="K12" s="6"/>
     </row>
-    <row r="13" spans="1:11" ht="16.5">
-      <c r="A13" s="6" t="s">
-        <v>67</v>
-      </c>
+    <row r="13" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
+      <c r="A13" s="6"/>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
       <c r="D13" s="6"/>
@@ -960,13 +940,13 @@
       </c>
       <c r="H13" s="15" t="str">
         <f>H12 &amp; "-build-" &amp; I10</f>
-        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5459-rt4</v>
+        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5460-rt4</v>
       </c>
       <c r="I13" s="16"/>
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
     </row>
-    <row r="14" spans="1:11" ht="16.5">
+    <row r="14" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A14" s="6"/>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -987,7 +967,7 @@
       </c>
       <c r="K14" s="6"/>
     </row>
-    <row r="15" spans="1:11" ht="16.5">
+    <row r="15" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A15" s="6"/>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -1002,14 +982,14 @@
       </c>
       <c r="I15" s="8" t="str">
         <f>I10</f>
-        <v>5459-rt4</v>
+        <v>5460-rt4</v>
       </c>
       <c r="J15" s="8" t="s">
         <v>19</v>
       </c>
       <c r="K15" s="6"/>
     </row>
-    <row r="16" spans="1:11" ht="16.5">
+    <row r="16" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A16" s="6"/>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -1027,7 +1007,7 @@
       <c r="J16" s="14"/>
       <c r="K16" s="6"/>
     </row>
-    <row r="17" spans="1:11" ht="16.5">
+    <row r="17" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
@@ -1045,7 +1025,7 @@
       <c r="J17" s="14"/>
       <c r="K17" s="6"/>
     </row>
-    <row r="18" spans="1:11" ht="16.5">
+    <row r="18" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A18" s="6"/>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -1057,13 +1037,13 @@
       </c>
       <c r="H18" s="15" t="str">
         <f>H17 &amp; "-build-" &amp; I15</f>
-        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5459-rt4</v>
+        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5460-rt4</v>
       </c>
       <c r="I18" s="16"/>
       <c r="J18" s="6"/>
       <c r="K18" s="6"/>
     </row>
-    <row r="19" spans="1:11" ht="16.5">
+    <row r="19" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A19" s="6"/>
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
@@ -1084,7 +1064,7 @@
       </c>
       <c r="K19" s="6"/>
     </row>
-    <row r="20" spans="1:11" ht="16.5">
+    <row r="20" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A20" s="6"/>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
@@ -1099,14 +1079,14 @@
       </c>
       <c r="I20" s="8" t="str">
         <f>I15</f>
-        <v>5459-rt4</v>
+        <v>5460-rt4</v>
       </c>
       <c r="J20" s="8" t="s">
         <v>20</v>
       </c>
       <c r="K20" s="6"/>
     </row>
-    <row r="21" spans="1:11" ht="16.5">
+    <row r="21" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A21" s="6"/>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -1124,7 +1104,7 @@
       <c r="J21" s="14"/>
       <c r="K21" s="6"/>
     </row>
-    <row r="22" spans="1:11" ht="16.5">
+    <row r="22" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A22" s="6"/>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
@@ -1142,7 +1122,7 @@
       <c r="J22" s="14"/>
       <c r="K22" s="6"/>
     </row>
-    <row r="23" spans="1:11" ht="16.5">
+    <row r="23" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A23" s="6"/>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
@@ -1154,13 +1134,13 @@
       </c>
       <c r="H23" s="15" t="str">
         <f>H22 &amp; "-build-" &amp; I20</f>
-        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5459-rt4</v>
+        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5460-rt4</v>
       </c>
       <c r="I23" s="16"/>
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
     </row>
-    <row r="24" spans="1:11" ht="16.5">
+    <row r="24" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A24" s="6"/>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -1181,7 +1161,7 @@
       </c>
       <c r="K24" s="6"/>
     </row>
-    <row r="25" spans="1:11" ht="16.5">
+    <row r="25" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A25" s="6"/>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -1196,14 +1176,14 @@
       </c>
       <c r="I25" s="8" t="str">
         <f>I20</f>
-        <v>5459-rt4</v>
+        <v>5460-rt4</v>
       </c>
       <c r="J25" s="8" t="s">
         <v>21</v>
       </c>
       <c r="K25" s="6"/>
     </row>
-    <row r="26" spans="1:11" ht="16.5">
+    <row r="26" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A26" s="6"/>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -1221,7 +1201,7 @@
       <c r="J26" s="14"/>
       <c r="K26" s="6"/>
     </row>
-    <row r="27" spans="1:11" ht="16.5">
+    <row r="27" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A27" s="6"/>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -1239,7 +1219,7 @@
       <c r="J27" s="14"/>
       <c r="K27" s="6"/>
     </row>
-    <row r="28" spans="1:11" ht="16.5">
+    <row r="28" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A28" s="6"/>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
@@ -1251,13 +1231,13 @@
       </c>
       <c r="H28" s="15" t="str">
         <f>H27 &amp; "-build-" &amp; I25</f>
-        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5459-rt4</v>
+        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5460-rt4</v>
       </c>
       <c r="I28" s="16"/>
       <c r="J28" s="6"/>
       <c r="K28" s="6"/>
     </row>
-    <row r="29" spans="1:11" ht="16.5">
+    <row r="29" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A29" s="6"/>
       <c r="B29" s="6"/>
       <c r="C29" s="6"/>
@@ -1272,7 +1252,7 @@
       <c r="J29" s="6"/>
       <c r="K29" s="6"/>
     </row>
-    <row r="30" spans="1:11" ht="16.5">
+    <row r="30" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A30" s="6"/>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
@@ -1293,7 +1273,7 @@
       </c>
       <c r="K30" s="6"/>
     </row>
-    <row r="31" spans="1:11" ht="16.5">
+    <row r="31" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A31" s="6"/>
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
@@ -1308,14 +1288,14 @@
       </c>
       <c r="I31" s="8" t="str">
         <f>I25</f>
-        <v>5459-rt4</v>
+        <v>5460-rt4</v>
       </c>
       <c r="J31" s="8" t="s">
         <v>23</v>
       </c>
       <c r="K31" s="6"/>
     </row>
-    <row r="32" spans="1:11" ht="16.5">
+    <row r="32" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A32" s="6"/>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
@@ -1333,7 +1313,7 @@
       <c r="J32" s="14"/>
       <c r="K32" s="6"/>
     </row>
-    <row r="33" spans="1:11" ht="16.5">
+    <row r="33" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A33" s="6"/>
       <c r="B33" s="6"/>
       <c r="C33" s="6"/>
@@ -1351,7 +1331,7 @@
       <c r="J33" s="14"/>
       <c r="K33" s="6"/>
     </row>
-    <row r="34" spans="1:11" ht="16.5">
+    <row r="34" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A34" s="6"/>
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
@@ -1363,13 +1343,13 @@
       </c>
       <c r="H34" s="15" t="str">
         <f>H33 &amp; "-build-" &amp; I31</f>
-        <v>v10.0.3-Classic_Reimagined_10_SE-build-5459-rt4</v>
+        <v>v10.0.3-Classic_Reimagined_10_SE-build-5460-rt4</v>
       </c>
       <c r="I34" s="16"/>
       <c r="J34" s="6"/>
       <c r="K34" s="6"/>
     </row>
-    <row r="35" spans="1:11" ht="16.5">
+    <row r="35" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A35" s="6"/>
       <c r="B35" s="6"/>
       <c r="C35" s="6"/>
@@ -1384,7 +1364,7 @@
       <c r="J35" s="6"/>
       <c r="K35" s="6"/>
     </row>
-    <row r="36" spans="1:11" ht="16.5">
+    <row r="36" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A36" s="6"/>
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
@@ -1405,7 +1385,7 @@
       </c>
       <c r="K36" s="6"/>
     </row>
-    <row r="37" spans="1:11" ht="16.5">
+    <row r="37" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A37" s="6"/>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -1420,14 +1400,14 @@
       </c>
       <c r="I37" s="8" t="str">
         <f>I31</f>
-        <v>5459-rt4</v>
+        <v>5460-rt4</v>
       </c>
       <c r="J37" s="8" t="s">
         <v>25</v>
       </c>
       <c r="K37" s="6"/>
     </row>
-    <row r="38" spans="1:11" ht="16.5">
+    <row r="38" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A38" s="6"/>
       <c r="B38" s="6"/>
       <c r="C38" s="6"/>
@@ -1444,7 +1424,7 @@
       <c r="J38" s="14"/>
       <c r="K38" s="6"/>
     </row>
-    <row r="39" spans="1:11" ht="16.5">
+    <row r="39" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A39" s="6"/>
       <c r="B39" s="6"/>
       <c r="C39" s="6"/>
@@ -1462,7 +1442,7 @@
       <c r="J39" s="14"/>
       <c r="K39" s="6"/>
     </row>
-    <row r="40" spans="1:11" ht="16.5">
+    <row r="40" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A40" s="6"/>
       <c r="B40" s="6"/>
       <c r="C40" s="6"/>
@@ -1474,13 +1454,13 @@
       </c>
       <c r="H40" s="15" t="str">
         <f>H39 &amp; "-build-" &amp; I37</f>
-        <v>v10.0.2-Classic_Reimagined_10s-build-5459-rt4</v>
+        <v>v10.0.2-Classic_Reimagined_10s-build-5460-rt4</v>
       </c>
       <c r="I40" s="16"/>
       <c r="J40" s="6"/>
       <c r="K40" s="6"/>
     </row>
-    <row r="41" spans="1:11" ht="16.5">
+    <row r="41" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A41" s="6"/>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
@@ -1495,7 +1475,7 @@
       <c r="J41" s="6"/>
       <c r="K41" s="6"/>
     </row>
-    <row r="42" spans="1:11" ht="16.5">
+    <row r="42" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A42" s="6"/>
       <c r="B42" s="6"/>
       <c r="C42" s="6"/>
@@ -1516,7 +1496,7 @@
       </c>
       <c r="K42" s="6"/>
     </row>
-    <row r="43" spans="1:11" ht="16.5">
+    <row r="43" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A43" s="6"/>
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
@@ -1531,14 +1511,14 @@
       </c>
       <c r="I43" s="8" t="str">
         <f>I37</f>
-        <v>5459-rt4</v>
+        <v>5460-rt4</v>
       </c>
       <c r="J43" s="8" t="s">
         <v>28</v>
       </c>
       <c r="K43" s="6"/>
     </row>
-    <row r="44" spans="1:11" ht="16.5">
+    <row r="44" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A44" s="6"/>
       <c r="B44" s="6"/>
       <c r="C44" s="6"/>
@@ -1555,7 +1535,7 @@
       <c r="J44" s="14"/>
       <c r="K44" s="6"/>
     </row>
-    <row r="45" spans="1:11" ht="16.5">
+    <row r="45" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A45" s="6"/>
       <c r="B45" s="6"/>
       <c r="C45" s="6"/>
@@ -1573,7 +1553,7 @@
       <c r="J45" s="14"/>
       <c r="K45" s="6"/>
     </row>
-    <row r="46" spans="1:11" ht="16.5">
+    <row r="46" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A46" s="6"/>
       <c r="B46" s="6"/>
       <c r="C46" s="6"/>
@@ -1585,13 +1565,13 @@
       </c>
       <c r="H46" s="15" t="str">
         <f>H45 &amp; "-build-" &amp; I43</f>
-        <v>v10.0.1-Classic_Reimagined_10-build-5459-rt4</v>
+        <v>v10.0.1-Classic_Reimagined_10-build-5460-rt4</v>
       </c>
       <c r="I46" s="16"/>
       <c r="J46" s="6"/>
       <c r="K46" s="6"/>
     </row>
-    <row r="47" spans="1:11" ht="16.5">
+    <row r="47" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A47" s="6"/>
       <c r="B47" s="6"/>
       <c r="C47" s="6"/>
@@ -1606,7 +1586,7 @@
       <c r="J47" s="2"/>
       <c r="K47" s="6"/>
     </row>
-    <row r="48" spans="1:11" ht="16.5">
+    <row r="48" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A48" s="6"/>
       <c r="B48" s="6"/>
       <c r="C48" s="6"/>
@@ -1621,7 +1601,7 @@
       <c r="J48" s="6"/>
       <c r="K48" s="6"/>
     </row>
-    <row r="49" spans="1:11" ht="16.5">
+    <row r="49" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A49" s="6"/>
       <c r="B49" s="6"/>
       <c r="C49" s="6"/>
@@ -1642,7 +1622,7 @@
       </c>
       <c r="K49" s="6"/>
     </row>
-    <row r="50" spans="1:11" ht="16.5">
+    <row r="50" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A50" s="6"/>
       <c r="B50" s="6"/>
       <c r="C50" s="6"/>
@@ -1657,14 +1637,14 @@
       </c>
       <c r="I50" s="8" t="str">
         <f>I43</f>
-        <v>5459-rt4</v>
+        <v>5460-rt4</v>
       </c>
       <c r="J50" s="8" t="s">
         <v>33</v>
       </c>
       <c r="K50" s="6"/>
     </row>
-    <row r="51" spans="1:11" ht="16.5">
+    <row r="51" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A51" s="6"/>
       <c r="B51" s="6"/>
       <c r="C51" s="6"/>
@@ -1681,7 +1661,7 @@
       <c r="J51" s="14"/>
       <c r="K51" s="6"/>
     </row>
-    <row r="52" spans="1:11" ht="16.5">
+    <row r="52" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A52" s="6"/>
       <c r="B52" s="6"/>
       <c r="C52" s="6"/>
@@ -1699,7 +1679,7 @@
       <c r="J52" s="14"/>
       <c r="K52" s="6"/>
     </row>
-    <row r="53" spans="1:11" ht="16.5">
+    <row r="53" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A53" s="6"/>
       <c r="B53" s="6"/>
       <c r="C53" s="6"/>
@@ -1711,13 +1691,13 @@
       </c>
       <c r="H53" s="15" t="str">
         <f>H52 &amp; "-build-" &amp; I50</f>
-        <v>v8.10.32-Classic_Reimagined_8-build-5459-rt4</v>
+        <v>v8.10.32-Classic_Reimagined_8-build-5460-rt4</v>
       </c>
       <c r="I53" s="16"/>
       <c r="J53" s="6"/>
       <c r="K53" s="6"/>
     </row>
-    <row r="54" spans="1:11" ht="16.5">
+    <row r="54" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A54" s="6"/>
       <c r="B54" s="6"/>
       <c r="C54" s="6"/>
@@ -1732,7 +1712,7 @@
       <c r="J54" s="6"/>
       <c r="K54" s="6"/>
     </row>
-    <row r="55" spans="1:11" ht="16.5">
+    <row r="55" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A55" s="6"/>
       <c r="B55" s="6"/>
       <c r="C55" s="6"/>
@@ -1753,7 +1733,7 @@
       </c>
       <c r="K55" s="6"/>
     </row>
-    <row r="56" spans="1:11" ht="16.5">
+    <row r="56" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A56" s="6"/>
       <c r="B56" s="6"/>
       <c r="C56" s="6"/>
@@ -1768,14 +1748,14 @@
       </c>
       <c r="I56" s="8" t="str">
         <f>I50</f>
-        <v>5459-rt4</v>
+        <v>5460-rt4</v>
       </c>
       <c r="J56" s="8" t="s">
         <v>35</v>
       </c>
       <c r="K56" s="6"/>
     </row>
-    <row r="57" spans="1:11" ht="16.5">
+    <row r="57" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A57" s="6"/>
       <c r="B57" s="6"/>
       <c r="C57" s="6"/>
@@ -1792,7 +1772,7 @@
       <c r="J57" s="14"/>
       <c r="K57" s="6"/>
     </row>
-    <row r="58" spans="1:11" ht="16.5">
+    <row r="58" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A58" s="6"/>
       <c r="B58" s="6"/>
       <c r="C58" s="6"/>
@@ -1810,7 +1790,7 @@
       <c r="J58" s="14"/>
       <c r="K58" s="6"/>
     </row>
-    <row r="59" spans="1:11" ht="16.5">
+    <row r="59" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A59" s="6"/>
       <c r="B59" s="6"/>
       <c r="C59" s="6"/>
@@ -1822,13 +1802,13 @@
       </c>
       <c r="H59" s="15" t="str">
         <f>H58 &amp; "-build-" &amp; I56</f>
-        <v>v8.10.31-Classic_Reimagined_8-build-5459-rt4</v>
+        <v>v8.10.31-Classic_Reimagined_8-build-5460-rt4</v>
       </c>
       <c r="I59" s="16"/>
       <c r="J59" s="6"/>
       <c r="K59" s="6"/>
     </row>
-    <row r="60" spans="1:11" ht="16.5">
+    <row r="60" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A60" s="6"/>
       <c r="B60" s="6"/>
       <c r="C60" s="6"/>
@@ -1843,7 +1823,7 @@
       <c r="J60" s="17"/>
       <c r="K60" s="6"/>
     </row>
-    <row r="61" spans="1:11" ht="16.5">
+    <row r="61" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A61" s="6"/>
       <c r="B61" s="6"/>
       <c r="C61" s="6"/>
@@ -1864,7 +1844,7 @@
       </c>
       <c r="K61" s="6"/>
     </row>
-    <row r="62" spans="1:11" ht="16.5">
+    <row r="62" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A62" s="6"/>
       <c r="B62" s="6"/>
       <c r="C62" s="6"/>
@@ -1879,14 +1859,14 @@
       </c>
       <c r="I62" s="8" t="str">
         <f>I56</f>
-        <v>5459-rt4</v>
+        <v>5460-rt4</v>
       </c>
       <c r="J62" s="8" t="s">
         <v>38</v>
       </c>
       <c r="K62" s="6"/>
     </row>
-    <row r="63" spans="1:11" ht="16.5">
+    <row r="63" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A63" s="6"/>
       <c r="B63" s="6"/>
       <c r="C63" s="6"/>
@@ -1903,7 +1883,7 @@
       <c r="J63" s="14"/>
       <c r="K63" s="6"/>
     </row>
-    <row r="64" spans="1:11" ht="16.5">
+    <row r="64" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A64" s="6"/>
       <c r="B64" s="6"/>
       <c r="C64" s="6"/>
@@ -1921,7 +1901,7 @@
       <c r="J64" s="14"/>
       <c r="K64" s="6"/>
     </row>
-    <row r="65" spans="1:11" ht="16.5">
+    <row r="65" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A65" s="6"/>
       <c r="B65" s="6"/>
       <c r="C65" s="6"/>
@@ -1933,15 +1913,15 @@
       </c>
       <c r="H65" s="15" t="str">
         <f>H64 &amp; "-build-" &amp; I62</f>
-        <v>v7.11.3-Better_Default_7-build-5459-rt4</v>
+        <v>v7.11.3-Better_Default_7-build-5460-rt4</v>
       </c>
       <c r="I65" s="16"/>
       <c r="J65" s="6"/>
       <c r="K65" s="6"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:A13">
-    <sortCondition ref="A13"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:A9">
+    <sortCondition ref="A9"/>
   </sortState>
   <mergeCells count="5">
     <mergeCell ref="A1:C1"/>
@@ -1958,12 +1938,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D41"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="27.375" customWidth="1"/>
+    <col min="1" max="4" width="27.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="16.5">
+    <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A1" s="35" t="s">
         <v>40</v>
       </c>
@@ -1971,12 +1951,12 @@
       <c r="C1" s="35"/>
       <c r="D1" s="35"/>
     </row>
-    <row r="2" spans="1:4" ht="16.5">
+    <row r="2" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="16.5">
+    <row r="3" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>17</v>
       </c>
@@ -1990,7 +1970,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="16.5">
+    <row r="4" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
         <v>43</v>
       </c>
@@ -2004,7 +1984,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="16.5">
+    <row r="5" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
         <v>13</v>
       </c>
@@ -2014,7 +1994,7 @@
       <c r="C5" s="34"/>
       <c r="D5" s="14"/>
     </row>
-    <row r="6" spans="1:4" ht="16.5">
+    <row r="6" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
         <v>15</v>
       </c>
@@ -2025,12 +2005,12 @@
       <c r="C6" s="34"/>
       <c r="D6" s="14"/>
     </row>
-    <row r="7" spans="1:4" ht="16.5">
+    <row r="7" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="16.5">
+    <row r="8" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>17</v>
       </c>
@@ -2044,7 +2024,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="16.5">
+    <row r="9" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A9" s="8" t="s">
         <v>47</v>
       </c>
@@ -2058,7 +2038,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="16.5">
+    <row r="10" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
         <v>13</v>
       </c>
@@ -2068,7 +2048,7 @@
       <c r="C10" s="34"/>
       <c r="D10" s="14"/>
     </row>
-    <row r="11" spans="1:4" ht="16.5">
+    <row r="11" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A11" s="10" t="s">
         <v>15</v>
       </c>
@@ -2079,12 +2059,12 @@
       <c r="C11" s="34"/>
       <c r="D11" s="14"/>
     </row>
-    <row r="12" spans="1:4" ht="16.5">
+    <row r="12" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="16.5">
+    <row r="13" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
         <v>17</v>
       </c>
@@ -2098,7 +2078,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="16.5">
+    <row r="14" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A14" s="8" t="s">
         <v>47</v>
       </c>
@@ -2112,7 +2092,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="16.5">
+    <row r="15" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A15" s="10" t="s">
         <v>13</v>
       </c>
@@ -2122,7 +2102,7 @@
       <c r="C15" s="34"/>
       <c r="D15" s="14"/>
     </row>
-    <row r="16" spans="1:4" ht="16.5">
+    <row r="16" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
         <v>15</v>
       </c>
@@ -2133,12 +2113,12 @@
       <c r="C16" s="34"/>
       <c r="D16" s="14"/>
     </row>
-    <row r="17" spans="1:4" ht="16.5">
+    <row r="17" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="16.5">
+    <row r="18" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
         <v>17</v>
       </c>
@@ -2152,7 +2132,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="16.5">
+    <row r="19" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>47</v>
       </c>
@@ -2166,7 +2146,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="16.5">
+    <row r="20" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
         <v>13</v>
       </c>
@@ -2176,7 +2156,7 @@
       <c r="C20" s="34"/>
       <c r="D20" s="14"/>
     </row>
-    <row r="21" spans="1:4" ht="16.5">
+    <row r="21" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A21" s="10" t="s">
         <v>15</v>
       </c>
@@ -2187,12 +2167,12 @@
       <c r="C21" s="34"/>
       <c r="D21" s="14"/>
     </row>
-    <row r="22" spans="1:4" ht="16.5">
+    <row r="22" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="16.5">
+    <row r="23" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
         <v>17</v>
       </c>
@@ -2206,7 +2186,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="16.5">
+    <row r="24" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A24" s="8" t="s">
         <v>47</v>
       </c>
@@ -2220,7 +2200,7 @@
         <v>1.1599999999999999</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="16.5">
+    <row r="25" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A25" s="10" t="s">
         <v>13</v>
       </c>
@@ -2230,7 +2210,7 @@
       <c r="C25" s="34"/>
       <c r="D25" s="14"/>
     </row>
-    <row r="26" spans="1:4" ht="16.5">
+    <row r="26" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="s">
         <v>15</v>
       </c>
@@ -2241,12 +2221,12 @@
       <c r="C26" s="34"/>
       <c r="D26" s="14"/>
     </row>
-    <row r="27" spans="1:4" ht="16.5">
+    <row r="27" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="16.5">
+    <row r="28" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
         <v>17</v>
       </c>
@@ -2260,7 +2240,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="16.5">
+    <row r="29" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A29" s="8" t="s">
         <v>47</v>
       </c>
@@ -2274,7 +2254,7 @@
         <v>1.1499999999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="16.5">
+    <row r="30" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A30" s="10" t="s">
         <v>13</v>
       </c>
@@ -2284,7 +2264,7 @@
       <c r="C30" s="34"/>
       <c r="D30" s="14"/>
     </row>
-    <row r="31" spans="1:4" ht="16.5">
+    <row r="31" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A31" s="10" t="s">
         <v>15</v>
       </c>
@@ -2295,12 +2275,12 @@
       <c r="C31" s="34"/>
       <c r="D31" s="14"/>
     </row>
-    <row r="32" spans="1:4" ht="16.5">
+    <row r="32" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="16.5">
+    <row r="33" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
         <v>17</v>
       </c>
@@ -2314,7 +2294,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="16.5">
+    <row r="34" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A34" s="8" t="s">
         <v>47</v>
       </c>
@@ -2328,7 +2308,7 @@
         <v>1.1399999999999999</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="16.5">
+    <row r="35" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A35" s="10" t="s">
         <v>13</v>
       </c>
@@ -2338,7 +2318,7 @@
       <c r="C35" s="34"/>
       <c r="D35" s="14"/>
     </row>
-    <row r="36" spans="1:4" ht="16.5">
+    <row r="36" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A36" s="10" t="s">
         <v>15</v>
       </c>
@@ -2349,12 +2329,12 @@
       <c r="C36" s="34"/>
       <c r="D36" s="14"/>
     </row>
-    <row r="37" spans="1:4" ht="16.5">
+    <row r="37" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="16.5">
+    <row r="38" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
         <v>17</v>
       </c>
@@ -2368,7 +2348,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="16.5">
+    <row r="39" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A39" s="8" t="s">
         <v>47</v>
       </c>
@@ -2382,7 +2362,7 @@
         <v>1.1299999999999999</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="16.5">
+    <row r="40" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A40" s="10" t="s">
         <v>13</v>
       </c>
@@ -2392,7 +2372,7 @@
       <c r="C40" s="34"/>
       <c r="D40" s="14"/>
     </row>
-    <row r="41" spans="1:4" ht="16.5">
+    <row r="41" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A41" s="10" t="s">
         <v>15</v>
       </c>
@@ -2405,6 +2385,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2417,11 +2402,6 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Added sulfur cube textures
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6F12E9D-D1A4-4E9D-8B99-F7171A8B5DB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5C22CAD-C5D0-4910-A1F1-809956548B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="68">
   <si>
     <t>Current version in development</t>
   </si>
@@ -235,6 +235,9 @@
   </si>
   <si>
     <t>Optimized VRAM usage by 17%</t>
+  </si>
+  <si>
+    <t>Added sulfur cube textures</t>
   </si>
 </sst>
 </file>
@@ -871,7 +874,9 @@
       <c r="K9" s="6"/>
     </row>
     <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="6"/>
+      <c r="A10" s="6" t="s">
+        <v>67</v>
+      </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
@@ -2385,11 +2390,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2402,6 +2402,11 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Update night vision shader and sulfur cube assets
Refine Night Vision blending in shaders/core/lightmap.fsh to use an ambient-based brightening formula and adjusted sqrt mixing to correct color calculations. Update sulfur_cube inner/outer textures, add a new particle texture (sulfur_cube_goo.png), and update version_guide.xlsx.
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5C22CAD-C5D0-4910-A1F1-809956548B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BDF8E16-96B6-416D-AFAA-4CD3AB472076}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="70">
   <si>
     <t>Current version in development</t>
   </si>
@@ -238,6 +238,12 @@
   </si>
   <si>
     <t>Added sulfur cube textures</t>
+  </si>
+  <si>
+    <t>Added sulfur cube goo particle texture</t>
+  </si>
+  <si>
+    <t>Fixed lightmap shader</t>
   </si>
 </sst>
 </file>
@@ -898,7 +904,9 @@
       <c r="K10" s="6"/>
     </row>
     <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A11" s="6"/>
+      <c r="A11" s="6" t="s">
+        <v>68</v>
+      </c>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
       <c r="D11" s="6"/>
@@ -916,7 +924,9 @@
       <c r="K11" s="6"/>
     </row>
     <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A12" s="6"/>
+      <c r="A12" s="6" t="s">
+        <v>69</v>
+      </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
@@ -2390,6 +2400,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2402,11 +2417,6 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Remove lantern/chain; add cinnabar & sulfur assets
Delete vanilla block textures (chain.png, lantern.png, soul_lantern.png, soul_fire_lantern.png) and their lantern .mcmeta animation files. Add Classic_Reimagined v10.0.11_2 assets: cinnabar.png, sulfur.png and a set of sulfur_spike_* textures (up/down base, frustum, middle, tip, and merged tip variants). This replaces the removed assets with the new resourcepack/mod textures for the Classic_Reimagined update.
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D64E119C-E36A-4ACC-B384-8866CD77C744}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1834179F-CF21-44A0-9CF3-A103183CD1BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="76">
   <si>
     <t>Current version in development</t>
   </si>
@@ -253,6 +253,15 @@
   </si>
   <si>
     <t>Added sulfur cube spawn egg item definition</t>
+  </si>
+  <si>
+    <t>Added cinnabar block textures</t>
+  </si>
+  <si>
+    <t>Added sulfur block textures</t>
+  </si>
+  <si>
+    <t>Removed chain/old lantern textures</t>
   </si>
 </sst>
 </file>
@@ -1020,7 +1029,9 @@
       <c r="K15" s="6"/>
     </row>
     <row r="16" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A16" s="6"/>
+      <c r="A16" s="6" t="s">
+        <v>73</v>
+      </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
@@ -1038,7 +1049,9 @@
       <c r="K16" s="6"/>
     </row>
     <row r="17" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A17" s="6"/>
+      <c r="A17" s="6" t="s">
+        <v>74</v>
+      </c>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
@@ -1056,7 +1069,9 @@
       <c r="K17" s="6"/>
     </row>
     <row r="18" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="6"/>
+      <c r="A18" s="6" t="s">
+        <v>75</v>
+      </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
@@ -2415,6 +2430,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2427,11 +2447,6 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Add sign assets & chicken sounds; update textures
Modify two cooked item textures and add new versioned assets for Classic_Reimagined v10.0.11.

Changes:
- Updated assets/minecraft/textures/item/cooked_beef.png and cooked_porkchop.png.
- Added numerous chicken sound files (baby_chicken, picky, say/plop/step variants) under v10.0.11_1.
- Added sign models (sign_rot_0..3, wall_sign), particle definition (geyser_poof), and a set of sign textures and hanging-sign textures under v10.0.11_2.
- Updated version_guide.xlsx.
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB704AFE-8F6B-4830-B493-BAC87DC715FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A31AFB5B-423E-4A38-8000-8877D7BAA7B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="66">
   <si>
     <t>Current version in development</t>
   </si>
@@ -222,46 +222,16 @@
     <t>Better Default 1.1</t>
   </si>
   <si>
-    <t>Optimized textures for Vulkan's memory buffer</t>
-  </si>
-  <si>
-    <t>Improved shaders</t>
-  </si>
-  <si>
-    <t>Added 26.2 compatibility</t>
-  </si>
-  <si>
-    <t>Simplified animated textures to less sprites</t>
-  </si>
-  <si>
-    <t>Optimized VRAM usage by 17%</t>
-  </si>
-  <si>
-    <t>Added sulfur cube textures</t>
-  </si>
-  <si>
-    <t>Added sulfur cube goo particle texture</t>
-  </si>
-  <si>
-    <t>Fixed lightmap shader</t>
-  </si>
-  <si>
-    <t>Added noxious gas particle textures</t>
-  </si>
-  <si>
-    <t>Added sulfur cube bucket texture</t>
-  </si>
-  <si>
-    <t>Added sulfur cube spawn egg item definition</t>
-  </si>
-  <si>
-    <t>Added cinnabar block textures</t>
-  </si>
-  <si>
-    <t>Added sulfur block textures</t>
-  </si>
-  <si>
-    <t>Removed chain/old lantern textures</t>
+    <t>Added sign block models</t>
+  </si>
+  <si>
+    <t>Fixed chicken sound effects</t>
+  </si>
+  <si>
+    <t>Fixed cooked cooked_beef texture</t>
+  </si>
+  <si>
+    <t>Fixed cooked cooked_porkchop texture</t>
   </si>
 </sst>
 </file>
@@ -798,7 +768,7 @@
     </row>
     <row r="5" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="24" t="s">
@@ -819,7 +789,7 @@
     </row>
     <row r="6" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -839,7 +809,7 @@
     </row>
     <row r="7" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -859,7 +829,7 @@
     </row>
     <row r="8" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -875,9 +845,7 @@
       <c r="K8" s="6"/>
     </row>
     <row r="9" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A9" s="6" t="s">
-        <v>71</v>
-      </c>
+      <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
       <c r="D9" s="6"/>
@@ -898,9 +866,7 @@
       <c r="K9" s="6"/>
     </row>
     <row r="10" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A10" s="6" t="s">
-        <v>68</v>
-      </c>
+      <c r="A10" s="6"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
       <c r="D10" s="6"/>
@@ -922,9 +888,7 @@
       <c r="K10" s="6"/>
     </row>
     <row r="11" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A11" s="6" t="s">
-        <v>72</v>
-      </c>
+      <c r="A11" s="6"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
       <c r="D11" s="6"/>
@@ -942,9 +906,7 @@
       <c r="K11" s="6"/>
     </row>
     <row r="12" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
-        <v>67</v>
-      </c>
+      <c r="A12" s="6"/>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
       <c r="D12" s="6"/>
@@ -962,9 +924,7 @@
       <c r="K12" s="6"/>
     </row>
     <row r="13" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A13" s="6" t="s">
-        <v>69</v>
-      </c>
+      <c r="A13" s="6"/>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
       <c r="D13" s="6"/>
@@ -982,9 +942,7 @@
       <c r="K13" s="6"/>
     </row>
     <row r="14" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A14" s="6" t="s">
-        <v>63</v>
-      </c>
+      <c r="A14" s="6"/>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
       <c r="D14" s="6"/>
@@ -1005,9 +963,7 @@
       <c r="K14" s="6"/>
     </row>
     <row r="15" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
-        <v>62</v>
-      </c>
+      <c r="A15" s="6"/>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
       <c r="D15" s="6"/>
@@ -1029,9 +985,7 @@
       <c r="K15" s="6"/>
     </row>
     <row r="16" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A16" s="6" t="s">
-        <v>66</v>
-      </c>
+      <c r="A16" s="6"/>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>
@@ -1049,9 +1003,7 @@
       <c r="K16" s="6"/>
     </row>
     <row r="17" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A17" s="6" t="s">
-        <v>75</v>
-      </c>
+      <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
@@ -1069,9 +1021,7 @@
       <c r="K17" s="6"/>
     </row>
     <row r="18" spans="1:11" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A18" s="6" t="s">
-        <v>65</v>
-      </c>
+      <c r="A18" s="6"/>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
@@ -2430,6 +2380,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2442,11 +2397,6 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Fixed bed models and textures (26.2+)
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hexy\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BD3B178-1635-447C-BBFB-45D6FF627C6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDEDD18E-E420-4BC3-9D65-12BCC1CB0413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="74">
   <si>
     <t>Current version in development</t>
   </si>
@@ -253,6 +253,9 @@
   </si>
   <si>
     <t>Base build</t>
+  </si>
+  <si>
+    <t>Fixed bed models and textures (26.2+)</t>
   </si>
 </sst>
 </file>
@@ -952,6 +955,9 @@
       <c r="J12" s="16"/>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="7" t="s">
+        <v>73</v>
+      </c>
       <c r="G13" s="12" t="s">
         <v>15</v>
       </c>
@@ -2008,11 +2014,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2025,6 +2026,11 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Rename sign models and add textures
Rename sign model files to use a template_ prefix (sign_rot_0..3 -> template_sign_rot_0..3, wall_sign -> template_wall_sign) for asset reorganization. Add new block textures purpur_pillar_side.png and quartz_pillar_side.png. Add small sulfur cube textures (sulfur_cube_inner_small.png, sulfur_cube_outer_small.png) and update sulfur_cube_outer.png. Update version_guide.xlsx to reflect these changes.

Co-Authored-By: Arc360 <155182753+arc360alt@users.noreply.github.com>
Co-Authored-By: Katsumi_Neko <63895016+katsumi-neko@users.noreply.github.com>
Co-Authored-By: shmoobalizer <53633630+shmoobalizer@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDEDD18E-E420-4BC3-9D65-12BCC1CB0413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2951B5A-E510-42D4-9491-E71B202CB42B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="77">
   <si>
     <t>Current version in development</t>
   </si>
@@ -256,6 +256,15 @@
   </si>
   <si>
     <t>Fixed bed models and textures (26.2+)</t>
+  </si>
+  <si>
+    <t>Added purpur pillar and quartz pillar side textures</t>
+  </si>
+  <si>
+    <t>Added small sulfur cube texture</t>
+  </si>
+  <si>
+    <t>Updated pack format to 88</t>
   </si>
 </sst>
 </file>
@@ -968,6 +977,9 @@
       <c r="I13" s="18"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" s="7" t="s">
+        <v>74</v>
+      </c>
       <c r="G14" s="10" t="s">
         <v>17</v>
       </c>
@@ -982,6 +994,9 @@
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="7" t="s">
+        <v>75</v>
+      </c>
       <c r="G15" s="11" t="s">
         <v>11</v>
       </c>
@@ -997,6 +1012,9 @@
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="7" t="s">
+        <v>76</v>
+      </c>
       <c r="G16" s="12" t="s">
         <v>13</v>
       </c>
@@ -2014,6 +2032,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2026,11 +2049,6 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Updated pack format to 88
Co-Authored-By: Katsumi_Neko <63895016+katsumi-neko@users.noreply.github.com>
Co-Authored-By: Arc360 <155182753+arc360alt@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96D723D6-FCC1-4EE2-A3C5-11971B6E70D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A620B0CB-DE8B-45D5-82F3-5ADA58F69C5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="73">
   <si>
     <t>Current version in development</t>
   </si>
@@ -225,21 +225,12 @@
     <t>Branch</t>
   </si>
   <si>
-    <t>5</t>
-  </si>
-  <si>
     <t>Month</t>
   </si>
   <si>
-    <t>05</t>
-  </si>
-  <si>
     <t>Seasonal drop</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>Base build</t>
   </si>
   <si>
@@ -256,6 +247,12 @@
   </si>
   <si>
     <t>Updated small sulfur cube texture</t>
+  </si>
+  <si>
+    <t>Updated pack format to 88</t>
+  </si>
+  <si>
+    <t>Classic Reimagined 11 version history</t>
   </si>
 </sst>
 </file>
@@ -317,7 +314,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -367,6 +364,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0070C0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -444,7 +447,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -455,7 +458,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -476,8 +478,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -500,8 +500,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="7" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -522,6 +520,23 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -713,854 +728,934 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K65"/>
+  <dimension ref="A1:K72"/>
   <sheetFormatPr defaultColWidth="27.28515625" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="36.5703125" style="7" customWidth="1"/>
-    <col min="2" max="2" width="36.7109375" style="7" customWidth="1"/>
-    <col min="3" max="16384" width="27.28515625" style="7"/>
+    <col min="1" max="1" width="36.5703125" style="6" customWidth="1"/>
+    <col min="2" max="2" width="36.7109375" style="6" customWidth="1"/>
+    <col min="3" max="16384" width="27.28515625" style="6"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="40"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="G1" s="8" t="s">
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="35"/>
+      <c r="G1" s="42" t="s">
+        <v>72</v>
+      </c>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" s="32" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" s="44">
+        <v>5</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" s="32" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" s="44">
+        <v>2</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="K3" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" s="32" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" s="44">
+        <v>6</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="10">
+        <v>11</v>
+      </c>
+      <c r="I4" s="10">
+        <v>2</v>
+      </c>
+      <c r="J4" s="10" t="str">
+        <f>D7</f>
+        <v>5206-rt5</v>
+      </c>
+      <c r="K4" s="10">
+        <v>26.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="32" t="s">
+        <v>65</v>
+      </c>
+      <c r="B5" s="45" t="str">
+        <f>B2&amp;B3&amp;0&amp;0+B4</f>
+        <v>5206</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="12" t="str">
+        <f>"Classic_Reimagined_11" &amp; G2</f>
+        <v>Classic_Reimagined_11_SE_2.1</v>
+      </c>
+      <c r="I5" s="13"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="15"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="39" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="40"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="E6" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" s="12" t="str">
+        <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-" &amp; H5</f>
+        <v>v10.0.11_2-Classic_Reimagined_11_SE_2.1</v>
+      </c>
+      <c r="I6" s="13"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="15"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="19" t="str">
+        <f>G11 &amp; "." &amp; H11 &amp; "_" &amp; I11 &amp; "-build-" &amp; D7</f>
+        <v>v10.0.11_1-build-5206-rt5</v>
+      </c>
+      <c r="B7" s="30"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="10" t="str">
+        <f>B5&amp;"-rt"&amp;B2</f>
+        <v>5206-rt5</v>
+      </c>
+      <c r="E7" s="21">
+        <f>K11</f>
+        <v>26.1</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H7" s="12" t="str">
+        <f>H6 &amp; "-build-" &amp; J4</f>
+        <v>v10.0.11_2-Classic_Reimagined_11_SE_2.1-build-5206-rt5</v>
+      </c>
+      <c r="I7" s="13"/>
+      <c r="J7" s="14"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" s="24"/>
+      <c r="E8" s="25"/>
+      <c r="G8" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="8"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="37" t="s">
-        <v>62</v>
-      </c>
-      <c r="B2" s="33" t="s">
-        <v>63</v>
-      </c>
-      <c r="C2"/>
-      <c r="D2"/>
-      <c r="G2" s="9" t="s">
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
+      <c r="J8" s="7"/>
+      <c r="K8" s="7"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="27"/>
+      <c r="E9" s="28"/>
+      <c r="G9" s="8" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="37" t="s">
-        <v>64</v>
-      </c>
-      <c r="B3" s="33" t="s">
-        <v>65</v>
-      </c>
-      <c r="C3"/>
-      <c r="D3"/>
-      <c r="G3" s="10" t="s">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="G10" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="H10" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="I10" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="J3" s="10" t="s">
+      <c r="J10" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="K3" s="10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="37" t="s">
-        <v>66</v>
-      </c>
-      <c r="B4" s="33" t="s">
-        <v>67</v>
-      </c>
-      <c r="C4"/>
-      <c r="D4"/>
-      <c r="G4" s="11" t="s">
+      <c r="K10" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="H4" s="11">
+      <c r="H11" s="10">
         <v>11</v>
       </c>
-      <c r="I4" s="11">
+      <c r="I11" s="10">
         <v>1</v>
       </c>
-      <c r="J4" s="11" t="str">
-        <f>D7</f>
-        <v>5052-rt5</v>
-      </c>
-      <c r="K4" s="11">
+      <c r="J11" s="10" t="str">
+        <f>J4</f>
+        <v>5206-rt5</v>
+      </c>
+      <c r="K11" s="10">
         <v>26.1</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="37" t="s">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="B5" s="33" t="str">
-        <f>B2&amp;B3&amp;B4</f>
-        <v>5052</v>
-      </c>
-      <c r="C5"/>
-      <c r="D5"/>
-      <c r="G5" s="12" t="s">
+      <c r="G12" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="13" t="str">
-        <f>"Classic_Reimagined_10" &amp; G2</f>
+      <c r="H12" s="12" t="str">
+        <f>"Classic_Reimagined_10" &amp; G9</f>
         <v>Classic_Reimagined_10_SE_2.1</v>
       </c>
-      <c r="I5" s="14"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="16"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="19" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="34"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="10" t="s">
+      <c r="I12" s="13"/>
+      <c r="J12" s="14"/>
+      <c r="K12" s="15"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H13" s="12" t="str">
+        <f>G11 &amp; "." &amp; H11 &amp; "_" &amp; I11 &amp; "-" &amp; H12</f>
+        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1</v>
+      </c>
+      <c r="I13" s="13"/>
+      <c r="J13" s="14"/>
+      <c r="K13" s="15"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H14" s="12" t="str">
+        <f>H13 &amp; "-build-" &amp; J11</f>
+        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5206-rt5</v>
+      </c>
+      <c r="I14" s="13"/>
+      <c r="J14" s="14"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G15" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G16" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="I16" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="21" t="s">
-        <v>4</v>
-      </c>
-      <c r="G6" s="12" t="s">
+      <c r="J16" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G17" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="H17" s="10">
+        <v>10</v>
+      </c>
+      <c r="I17" s="10" t="str">
+        <f>J11</f>
+        <v>5206-rt5</v>
+      </c>
+      <c r="J17" s="10" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G18" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H18" s="16" t="str">
+        <f>"Classic_Reimagined_10" &amp; G15</f>
+        <v>Classic_Reimagined_10_SE_2</v>
+      </c>
+      <c r="I18" s="17"/>
+      <c r="J18" s="15"/>
+    </row>
+    <row r="19" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G19" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="13" t="str">
-        <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-" &amp; H5</f>
-        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1</v>
-      </c>
-      <c r="I6" s="14"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="16"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="22" t="str">
-        <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-build-" &amp; D7</f>
-        <v>v10.0.11_1-build-5052-rt5</v>
-      </c>
-      <c r="B7" s="35"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="11" t="str">
-        <f>B5&amp;"-rt"&amp;B2</f>
-        <v>5052-rt5</v>
-      </c>
-      <c r="E7" s="24">
-        <f>K4</f>
-        <v>26.1</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="H7" s="13" t="str">
-        <f>H6 &amp; "-build-" &amp; J4</f>
-        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5052-rt5</v>
-      </c>
-      <c r="I7" s="14"/>
-      <c r="J7" s="15"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="25" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="36" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="27"/>
-      <c r="E8" s="28"/>
-      <c r="G8" s="9" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
-        <v>70</v>
-      </c>
-      <c r="C9" s="29" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="30"/>
-      <c r="E9" s="31"/>
-      <c r="G9" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="I9" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="J9" s="10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="7" t="s">
-        <v>69</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="H10" s="11">
-        <v>10</v>
-      </c>
-      <c r="I10" s="11" t="str">
-        <f>J4</f>
-        <v>5052-rt5</v>
-      </c>
-      <c r="J10" s="11" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H11" s="17" t="str">
-        <f>"Classic_Reimagined_10" &amp; G8</f>
-        <v>Classic_Reimagined_10_SE_2</v>
-      </c>
-      <c r="I11" s="18"/>
-      <c r="J11" s="16"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="G12" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="H12" s="17" t="str">
-        <f>G10 &amp; "." &amp; H10 &amp; "-" &amp; H11</f>
+      <c r="H19" s="16" t="str">
+        <f>G17 &amp; "." &amp; H17 &amp; "-" &amp; H18</f>
         <v>v10.0.10-Classic_Reimagined_10_SE_2</v>
       </c>
-      <c r="I12" s="18"/>
-      <c r="J12" s="16"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="G13" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="H13" s="17" t="str">
-        <f>H12 &amp; "-build-" &amp; I10</f>
-        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5052-rt5</v>
-      </c>
-      <c r="I13" s="18"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G14" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="H14" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="I14" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="J14" s="10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G15" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="H15" s="11">
-        <v>9</v>
-      </c>
-      <c r="I15" s="11" t="str">
-        <f>I10</f>
-        <v>5052-rt5</v>
-      </c>
-      <c r="J15" s="11" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G16" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="H16" s="17" t="str">
-        <f>H11</f>
-        <v>Classic_Reimagined_10_SE_2</v>
-      </c>
-      <c r="I16" s="18"/>
-      <c r="J16" s="16"/>
-    </row>
-    <row r="17" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G17" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="H17" s="17" t="str">
-        <f>G15 &amp; "." &amp; H15 &amp; "-" &amp; H16</f>
-        <v>v10.0.9-Classic_Reimagined_10_SE_2</v>
-      </c>
-      <c r="I17" s="18"/>
-      <c r="J17" s="16"/>
-    </row>
-    <row r="18" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G18" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="H18" s="17" t="str">
-        <f>H17 &amp; "-build-" &amp; I15</f>
-        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5052-rt5</v>
-      </c>
-      <c r="I18" s="18"/>
-    </row>
-    <row r="19" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G19" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="I19" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="J19" s="10" t="s">
-        <v>4</v>
-      </c>
+      <c r="I19" s="17"/>
+      <c r="J19" s="15"/>
     </row>
     <row r="20" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G20" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H20" s="16" t="str">
+        <f>H19 &amp; "-build-" &amp; I17</f>
+        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5206-rt5</v>
+      </c>
+      <c r="I20" s="17"/>
+    </row>
+    <row r="21" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G21" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="I21" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G22" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="H20" s="11">
-        <v>7</v>
-      </c>
-      <c r="I20" s="11" t="str">
-        <f>I15</f>
-        <v>5052-rt5</v>
-      </c>
-      <c r="J20" s="11" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="21" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G21" s="12" t="s">
+      <c r="H22" s="10">
+        <v>9</v>
+      </c>
+      <c r="I22" s="10" t="str">
+        <f>I17</f>
+        <v>5206-rt5</v>
+      </c>
+      <c r="J22" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G23" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="H21" s="17" t="str">
-        <f>H16</f>
+      <c r="H23" s="16" t="str">
+        <f>H18</f>
         <v>Classic_Reimagined_10_SE_2</v>
       </c>
-      <c r="I21" s="18"/>
-      <c r="J21" s="16"/>
-    </row>
-    <row r="22" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G22" s="12" t="s">
+      <c r="I23" s="17"/>
+      <c r="J23" s="15"/>
+    </row>
+    <row r="24" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G24" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H22" s="17" t="str">
-        <f>G20 &amp; "." &amp; H20 &amp; "-" &amp; H21</f>
-        <v>v10.0.7-Classic_Reimagined_10_SE_2</v>
-      </c>
-      <c r="I22" s="18"/>
-      <c r="J22" s="16"/>
-    </row>
-    <row r="23" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G23" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="H23" s="17" t="str">
-        <f>H22 &amp; "-build-" &amp; I20</f>
-        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5052-rt5</v>
-      </c>
-      <c r="I23" s="18"/>
-    </row>
-    <row r="24" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G24" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="H24" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="I24" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="J24" s="10" t="s">
-        <v>4</v>
-      </c>
+      <c r="H24" s="16" t="str">
+        <f>G22 &amp; "." &amp; H22 &amp; "-" &amp; H23</f>
+        <v>v10.0.9-Classic_Reimagined_10_SE_2</v>
+      </c>
+      <c r="I24" s="17"/>
+      <c r="J24" s="15"/>
     </row>
     <row r="25" spans="7:10" x14ac:dyDescent="0.3">
       <c r="G25" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H25" s="16" t="str">
+        <f>H24 &amp; "-build-" &amp; I22</f>
+        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5206-rt5</v>
+      </c>
+      <c r="I25" s="17"/>
+    </row>
+    <row r="26" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G26" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H26" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="I26" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="J26" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G27" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="H25" s="11">
-        <v>4</v>
-      </c>
-      <c r="I25" s="11" t="str">
-        <f>I20</f>
-        <v>5052-rt5</v>
-      </c>
-      <c r="J25" s="11" t="s">
+      <c r="H27" s="10">
+        <v>7</v>
+      </c>
+      <c r="I27" s="10" t="str">
+        <f>I22</f>
+        <v>5206-rt5</v>
+      </c>
+      <c r="J27" s="10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G28" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H28" s="16" t="str">
+        <f>H23</f>
+        <v>Classic_Reimagined_10_SE_2</v>
+      </c>
+      <c r="I28" s="17"/>
+      <c r="J28" s="15"/>
+    </row>
+    <row r="29" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G29" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="H29" s="16" t="str">
+        <f>G27 &amp; "." &amp; H27 &amp; "-" &amp; H28</f>
+        <v>v10.0.7-Classic_Reimagined_10_SE_2</v>
+      </c>
+      <c r="I29" s="17"/>
+      <c r="J29" s="15"/>
+    </row>
+    <row r="30" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G30" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" s="16" t="str">
+        <f>H29 &amp; "-build-" &amp; I27</f>
+        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5206-rt5</v>
+      </c>
+      <c r="I30" s="17"/>
+    </row>
+    <row r="31" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G31" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="I31" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="J31" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G32" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="H32" s="10">
+        <v>4</v>
+      </c>
+      <c r="I32" s="10" t="str">
+        <f>I27</f>
+        <v>5206-rt5</v>
+      </c>
+      <c r="J32" s="10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G26" s="12" t="s">
+    <row r="33" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G33" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="H26" s="17" t="str">
-        <f>H21</f>
+      <c r="H33" s="16" t="str">
+        <f>H28</f>
         <v>Classic_Reimagined_10_SE_2</v>
       </c>
-      <c r="I26" s="18"/>
-      <c r="J26" s="16"/>
-    </row>
-    <row r="27" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G27" s="12" t="s">
+      <c r="I33" s="17"/>
+      <c r="J33" s="15"/>
+    </row>
+    <row r="34" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G34" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H27" s="17" t="str">
-        <f>G25 &amp; "." &amp; H25 &amp; "-" &amp; H26</f>
+      <c r="H34" s="16" t="str">
+        <f>G32 &amp; "." &amp; H32 &amp; "-" &amp; H33</f>
         <v>v10.0.4-Classic_Reimagined_10_SE_2</v>
       </c>
-      <c r="I27" s="18"/>
-      <c r="J27" s="16"/>
-    </row>
-    <row r="28" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G28" s="12" t="s">
+      <c r="I34" s="17"/>
+      <c r="J34" s="15"/>
+    </row>
+    <row r="35" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G35" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H28" s="17" t="str">
-        <f>H27 &amp; "-build-" &amp; I25</f>
-        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5052-rt5</v>
-      </c>
-      <c r="I28" s="18"/>
-    </row>
-    <row r="29" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G29" s="9" t="s">
+      <c r="H35" s="16" t="str">
+        <f>H34 &amp; "-build-" &amp; I32</f>
+        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5206-rt5</v>
+      </c>
+      <c r="I35" s="17"/>
+    </row>
+    <row r="36" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G36" s="8" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G30" s="10" t="s">
+    <row r="37" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G37" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H30" s="10" t="s">
+      <c r="H37" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I30" s="10" t="s">
+      <c r="I37" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="J30" s="10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G31" s="11" t="s">
+      <c r="J37" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G38" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="H31" s="11">
+      <c r="H38" s="10">
         <v>3</v>
       </c>
-      <c r="I31" s="11" t="str">
-        <f>I25</f>
-        <v>5052-rt5</v>
-      </c>
-      <c r="J31" s="11" t="s">
+      <c r="I38" s="10" t="str">
+        <f>I32</f>
+        <v>5206-rt5</v>
+      </c>
+      <c r="J38" s="10" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G32" s="12" t="s">
+    <row r="39" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G39" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="H32" s="17" t="str">
-        <f>"Classic_Reimagined_10" &amp; G29</f>
+      <c r="H39" s="16" t="str">
+        <f>"Classic_Reimagined_10" &amp; G36</f>
         <v>Classic_Reimagined_10_SE</v>
       </c>
-      <c r="I32" s="18"/>
-      <c r="J32" s="16"/>
-    </row>
-    <row r="33" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G33" s="12" t="s">
+      <c r="I39" s="17"/>
+      <c r="J39" s="15"/>
+    </row>
+    <row r="40" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G40" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H33" s="17" t="str">
-        <f>G31 &amp; "." &amp; H31 &amp; "-" &amp; H32</f>
+      <c r="H40" s="16" t="str">
+        <f>G38 &amp; "." &amp; H38 &amp; "-" &amp; H39</f>
         <v>v10.0.3-Classic_Reimagined_10_SE</v>
       </c>
-      <c r="I33" s="18"/>
-      <c r="J33" s="16"/>
-    </row>
-    <row r="34" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G34" s="12" t="s">
+      <c r="I40" s="17"/>
+      <c r="J40" s="15"/>
+    </row>
+    <row r="41" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G41" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H34" s="17" t="str">
-        <f>H33 &amp; "-build-" &amp; I31</f>
-        <v>v10.0.3-Classic_Reimagined_10_SE-build-5052-rt5</v>
-      </c>
-      <c r="I34" s="18"/>
-    </row>
-    <row r="35" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G35" s="9" t="s">
+      <c r="H41" s="16" t="str">
+        <f>H40 &amp; "-build-" &amp; I38</f>
+        <v>v10.0.3-Classic_Reimagined_10_SE-build-5206-rt5</v>
+      </c>
+      <c r="I41" s="17"/>
+    </row>
+    <row r="42" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G42" s="8" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="36" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G36" s="10" t="s">
+    <row r="43" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G43" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H36" s="10" t="s">
+      <c r="H43" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I36" s="10" t="s">
+      <c r="I43" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="J36" s="10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="37" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G37" s="11" t="s">
+      <c r="J43" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G44" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="H37" s="11">
+      <c r="H44" s="10">
         <v>2</v>
       </c>
-      <c r="I37" s="11" t="str">
-        <f>I31</f>
-        <v>5052-rt5</v>
-      </c>
-      <c r="J37" s="11" t="s">
+      <c r="I44" s="10" t="str">
+        <f>I38</f>
+        <v>5206-rt5</v>
+      </c>
+      <c r="J44" s="10" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G38" s="12" t="s">
+    <row r="45" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G45" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="H38" s="17" t="s">
+      <c r="H45" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="I38" s="18"/>
-      <c r="J38" s="16"/>
-    </row>
-    <row r="39" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G39" s="12" t="s">
+      <c r="I45" s="17"/>
+      <c r="J45" s="15"/>
+    </row>
+    <row r="46" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G46" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H39" s="17" t="str">
-        <f>G37 &amp; "." &amp; H37 &amp; "-" &amp; H38</f>
+      <c r="H46" s="16" t="str">
+        <f>G44 &amp; "." &amp; H44 &amp; "-" &amp; H45</f>
         <v>v10.0.2-Classic_Reimagined_10s</v>
       </c>
-      <c r="I39" s="18"/>
-      <c r="J39" s="16"/>
-    </row>
-    <row r="40" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G40" s="12" t="s">
+      <c r="I46" s="17"/>
+      <c r="J46" s="15"/>
+    </row>
+    <row r="47" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G47" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H40" s="17" t="str">
-        <f>H39 &amp; "-build-" &amp; I37</f>
-        <v>v10.0.2-Classic_Reimagined_10s-build-5052-rt5</v>
-      </c>
-      <c r="I40" s="18"/>
-    </row>
-    <row r="41" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G41" s="9" t="s">
+      <c r="H47" s="16" t="str">
+        <f>H46 &amp; "-build-" &amp; I44</f>
+        <v>v10.0.2-Classic_Reimagined_10s-build-5206-rt5</v>
+      </c>
+      <c r="I47" s="17"/>
+    </row>
+    <row r="48" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G48" s="8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="42" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G42" s="10" t="s">
+    <row r="49" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G49" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H42" s="10" t="s">
+      <c r="H49" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I42" s="10" t="s">
+      <c r="I49" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="J42" s="10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="43" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G43" s="11" t="s">
+      <c r="J49" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G50" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="H43" s="11">
+      <c r="H50" s="10">
         <v>1</v>
       </c>
-      <c r="I43" s="11" t="str">
-        <f>I37</f>
-        <v>5052-rt5</v>
-      </c>
-      <c r="J43" s="11" t="s">
+      <c r="I50" s="10" t="str">
+        <f>I44</f>
+        <v>5206-rt5</v>
+      </c>
+      <c r="J50" s="10" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="44" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G44" s="12" t="s">
+    <row r="51" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G51" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="H44" s="17" t="s">
+      <c r="H51" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="I44" s="18"/>
-      <c r="J44" s="16"/>
-    </row>
-    <row r="45" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G45" s="12" t="s">
+      <c r="I51" s="17"/>
+      <c r="J51" s="15"/>
+    </row>
+    <row r="52" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G52" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H45" s="17" t="str">
-        <f>G43 &amp; "." &amp; H43 &amp; "-" &amp; H44</f>
+      <c r="H52" s="16" t="str">
+        <f>G50 &amp; "." &amp; H50 &amp; "-" &amp; H51</f>
         <v>v10.0.1-Classic_Reimagined_10</v>
       </c>
-      <c r="I45" s="18"/>
-      <c r="J45" s="16"/>
-    </row>
-    <row r="46" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G46" s="12" t="s">
+      <c r="I52" s="17"/>
+      <c r="J52" s="15"/>
+    </row>
+    <row r="53" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G53" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H46" s="17" t="str">
-        <f>H45 &amp; "-build-" &amp; I43</f>
-        <v>v10.0.1-Classic_Reimagined_10-build-5052-rt5</v>
-      </c>
-      <c r="I46" s="18"/>
-    </row>
-    <row r="47" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G47" s="8" t="s">
+      <c r="H53" s="16" t="str">
+        <f>H52 &amp; "-build-" &amp; I50</f>
+        <v>v10.0.1-Classic_Reimagined_10-build-5206-rt5</v>
+      </c>
+      <c r="I53" s="17"/>
+    </row>
+    <row r="54" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G54" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="H47" s="8"/>
-      <c r="I47" s="8"/>
-      <c r="J47" s="8"/>
-    </row>
-    <row r="48" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G48" s="9" t="s">
+      <c r="H54" s="7"/>
+      <c r="I54" s="7"/>
+      <c r="J54" s="7"/>
+    </row>
+    <row r="55" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G55" s="8" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="49" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G49" s="10" t="s">
+    <row r="56" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G56" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H49" s="10" t="s">
+      <c r="H56" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I49" s="10" t="s">
+      <c r="I56" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="J49" s="10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="50" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G50" s="11" t="s">
+      <c r="J56" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G57" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H50" s="11">
+      <c r="H57" s="10">
         <v>32</v>
       </c>
-      <c r="I50" s="11" t="str">
-        <f>I43</f>
-        <v>5052-rt5</v>
-      </c>
-      <c r="J50" s="11" t="s">
+      <c r="I57" s="10" t="str">
+        <f>I50</f>
+        <v>5206-rt5</v>
+      </c>
+      <c r="J57" s="10" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="51" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G51" s="12" t="s">
+    <row r="58" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G58" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="H51" s="17" t="s">
+      <c r="H58" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="I51" s="18"/>
-      <c r="J51" s="16"/>
-    </row>
-    <row r="52" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G52" s="12" t="s">
+      <c r="I58" s="17"/>
+      <c r="J58" s="15"/>
+    </row>
+    <row r="59" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G59" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H52" s="17" t="str">
-        <f>G50 &amp; "." &amp; H50 &amp; "-" &amp; H51</f>
+      <c r="H59" s="16" t="str">
+        <f>G57 &amp; "." &amp; H57 &amp; "-" &amp; H58</f>
         <v>v8.10.32-Classic_Reimagined_8</v>
       </c>
-      <c r="I52" s="18"/>
-      <c r="J52" s="16"/>
-    </row>
-    <row r="53" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G53" s="12" t="s">
+      <c r="I59" s="17"/>
+      <c r="J59" s="15"/>
+    </row>
+    <row r="60" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G60" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H53" s="17" t="str">
-        <f>H52 &amp; "-build-" &amp; I50</f>
-        <v>v8.10.32-Classic_Reimagined_8-build-5052-rt5</v>
-      </c>
-      <c r="I53" s="18"/>
-    </row>
-    <row r="54" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G54" s="9" t="s">
+      <c r="H60" s="16" t="str">
+        <f>H59 &amp; "-build-" &amp; I57</f>
+        <v>v8.10.32-Classic_Reimagined_8-build-5206-rt5</v>
+      </c>
+      <c r="I60" s="17"/>
+    </row>
+    <row r="61" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G61" s="8" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="55" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G55" s="10" t="s">
+    <row r="62" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G62" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H55" s="10" t="s">
+      <c r="H62" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I55" s="10" t="s">
+      <c r="I62" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="J55" s="10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="56" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G56" s="11" t="s">
+      <c r="J62" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="63" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G63" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="H56" s="11">
+      <c r="H63" s="10">
         <v>31</v>
       </c>
-      <c r="I56" s="11" t="str">
-        <f>I50</f>
-        <v>5052-rt5</v>
-      </c>
-      <c r="J56" s="11" t="s">
+      <c r="I63" s="10" t="str">
+        <f>I57</f>
+        <v>5206-rt5</v>
+      </c>
+      <c r="J63" s="10" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="57" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G57" s="12" t="s">
+    <row r="64" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G64" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="H57" s="17" t="s">
+      <c r="H64" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="I57" s="18"/>
-      <c r="J57" s="16"/>
-    </row>
-    <row r="58" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G58" s="12" t="s">
+      <c r="I64" s="17"/>
+      <c r="J64" s="15"/>
+    </row>
+    <row r="65" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G65" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H58" s="17" t="str">
-        <f>G56 &amp; "." &amp; H56 &amp; "-" &amp; H57</f>
+      <c r="H65" s="16" t="str">
+        <f>G63 &amp; "." &amp; H63 &amp; "-" &amp; H64</f>
         <v>v8.10.31-Classic_Reimagined_8</v>
       </c>
-      <c r="I58" s="18"/>
-      <c r="J58" s="16"/>
-    </row>
-    <row r="59" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G59" s="12" t="s">
+      <c r="I65" s="17"/>
+      <c r="J65" s="15"/>
+    </row>
+    <row r="66" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G66" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H59" s="17" t="str">
-        <f>H58 &amp; "-build-" &amp; I56</f>
-        <v>v8.10.31-Classic_Reimagined_8-build-5052-rt5</v>
-      </c>
-      <c r="I59" s="18"/>
-    </row>
-    <row r="60" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G60" s="32" t="s">
+      <c r="H66" s="16" t="str">
+        <f>H65 &amp; "-build-" &amp; I63</f>
+        <v>v8.10.31-Classic_Reimagined_8-build-5206-rt5</v>
+      </c>
+      <c r="I66" s="17"/>
+    </row>
+    <row r="67" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G67" s="29" t="s">
         <v>36</v>
       </c>
-      <c r="H60" s="32"/>
-      <c r="I60" s="32"/>
-      <c r="J60" s="32"/>
-    </row>
-    <row r="61" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G61" s="10" t="s">
+      <c r="H67" s="29"/>
+      <c r="I67" s="29"/>
+      <c r="J67" s="29"/>
+    </row>
+    <row r="68" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G68" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H61" s="10" t="s">
+      <c r="H68" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="I61" s="10" t="s">
+      <c r="I68" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="J61" s="10" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="62" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G62" s="11" t="s">
+      <c r="J68" s="9" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="69" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G69" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="H62" s="11">
+      <c r="H69" s="10">
         <v>3</v>
       </c>
-      <c r="I62" s="11" t="str">
-        <f>I56</f>
-        <v>5052-rt5</v>
-      </c>
-      <c r="J62" s="11" t="s">
+      <c r="I69" s="10" t="str">
+        <f>I63</f>
+        <v>5206-rt5</v>
+      </c>
+      <c r="J69" s="10" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="63" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G63" s="12" t="s">
+    <row r="70" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G70" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="H63" s="17" t="s">
+      <c r="H70" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="I63" s="18"/>
-      <c r="J63" s="16"/>
-    </row>
-    <row r="64" spans="7:10" x14ac:dyDescent="0.3">
-      <c r="G64" s="12" t="s">
+      <c r="I70" s="17"/>
+      <c r="J70" s="15"/>
+    </row>
+    <row r="71" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G71" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="H64" s="17" t="str">
-        <f>G62 &amp; "." &amp; H62 &amp; "-" &amp; H63</f>
+      <c r="H71" s="16" t="str">
+        <f>G69 &amp; "." &amp; H69 &amp; "-" &amp; H70</f>
         <v>v7.11.3-Better_Default_7</v>
       </c>
-      <c r="I64" s="18"/>
-      <c r="J64" s="16"/>
-    </row>
-    <row r="65" spans="7:9" x14ac:dyDescent="0.3">
-      <c r="G65" s="12" t="s">
+      <c r="I71" s="17"/>
+      <c r="J71" s="15"/>
+    </row>
+    <row r="72" spans="7:10" x14ac:dyDescent="0.3">
+      <c r="G72" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="H65" s="17" t="str">
-        <f>H64 &amp; "-build-" &amp; I62</f>
-        <v>v7.11.3-Better_Default_7-build-5052-rt5</v>
-      </c>
-      <c r="I65" s="18"/>
+      <c r="H72" s="16" t="str">
+        <f>H71 &amp; "-build-" &amp; I69</f>
+        <v>v7.11.3-Better_Default_7-build-5206-rt5</v>
+      </c>
+      <c r="I72" s="17"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A9:A12">
-    <sortCondition ref="A12"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:B4">
+    <sortCondition descending="1" ref="A3:A4"/>
   </sortState>
-  <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A6:C6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1573,12 +1668,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="38" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="43"/>
-      <c r="C1" s="43"/>
-      <c r="D1" s="43"/>
+      <c r="B1" s="38"/>
+      <c r="C1" s="38"/>
+      <c r="D1" s="38"/>
     </row>
     <row r="2" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -1617,21 +1712,21 @@
       <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="41" t="s">
+      <c r="B5" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="42"/>
+      <c r="C5" s="37"/>
       <c r="D5" s="5"/>
     </row>
     <row r="6" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="41" t="str">
+      <c r="B6" s="36" t="str">
         <f>A4 &amp; "." &amp; B4 &amp; "." &amp; C4 &amp; "-" &amp; B5</f>
         <v>v6.0.7-Better_Default_6</v>
       </c>
-      <c r="C6" s="42"/>
+      <c r="C6" s="37"/>
       <c r="D6" s="5"/>
     </row>
     <row r="7" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -1671,21 +1766,21 @@
       <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="41" t="s">
+      <c r="B10" s="36" t="s">
         <v>49</v>
       </c>
-      <c r="C10" s="42"/>
+      <c r="C10" s="37"/>
       <c r="D10" s="5"/>
     </row>
     <row r="11" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="41" t="str">
+      <c r="B11" s="36" t="str">
         <f>A9 &amp; "." &amp; B9 &amp; "." &amp; C9 &amp; "-" &amp; B10</f>
         <v>v1.4.0-Better_Default_5</v>
       </c>
-      <c r="C11" s="42"/>
+      <c r="C11" s="37"/>
       <c r="D11" s="5"/>
     </row>
     <row r="12" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -1725,21 +1820,21 @@
       <c r="A15" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="41" t="s">
+      <c r="B15" s="36" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="42"/>
+      <c r="C15" s="37"/>
       <c r="D15" s="5"/>
     </row>
     <row r="16" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="41" t="str">
+      <c r="B16" s="36" t="str">
         <f>A14 &amp; "." &amp; B14 &amp; "." &amp; C14 &amp; "-" &amp; B15</f>
         <v>v1.3.0-Better_Default_4</v>
       </c>
-      <c r="C16" s="42"/>
+      <c r="C16" s="37"/>
       <c r="D16" s="5"/>
     </row>
     <row r="17" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -1779,21 +1874,21 @@
       <c r="A20" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="41" t="s">
+      <c r="B20" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="42"/>
+      <c r="C20" s="37"/>
       <c r="D20" s="5"/>
     </row>
     <row r="21" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="41" t="str">
+      <c r="B21" s="36" t="str">
         <f>A19 &amp; "." &amp; B19 &amp; "." &amp; C19 &amp; "-" &amp; B20</f>
         <v>v1.2.2-Better_Default_3.1</v>
       </c>
-      <c r="C21" s="42"/>
+      <c r="C21" s="37"/>
       <c r="D21" s="5"/>
     </row>
     <row r="22" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -1833,21 +1928,21 @@
       <c r="A25" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="41" t="s">
+      <c r="B25" s="36" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="42"/>
+      <c r="C25" s="37"/>
       <c r="D25" s="5"/>
     </row>
     <row r="26" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B26" s="41" t="str">
+      <c r="B26" s="36" t="str">
         <f>A24 &amp; "." &amp; B24 &amp; "." &amp; C24 &amp; "-" &amp; B25</f>
         <v>v1.2.1-Better_Default_3</v>
       </c>
-      <c r="C26" s="42"/>
+      <c r="C26" s="37"/>
       <c r="D26" s="5"/>
     </row>
     <row r="27" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -1887,21 +1982,21 @@
       <c r="A30" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="41" t="s">
+      <c r="B30" s="36" t="s">
         <v>58</v>
       </c>
-      <c r="C30" s="42"/>
+      <c r="C30" s="37"/>
       <c r="D30" s="5"/>
     </row>
     <row r="31" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="41" t="str">
+      <c r="B31" s="36" t="str">
         <f>A29 &amp; "." &amp; B29 &amp; "." &amp; C29 &amp; "-" &amp; B30</f>
         <v>v1.2.0-Better_Default_2</v>
       </c>
-      <c r="C31" s="42"/>
+      <c r="C31" s="37"/>
       <c r="D31" s="5"/>
     </row>
     <row r="32" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -1941,21 +2036,21 @@
       <c r="A35" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B35" s="41" t="s">
+      <c r="B35" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="C35" s="42"/>
+      <c r="C35" s="37"/>
       <c r="D35" s="5"/>
     </row>
     <row r="36" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B36" s="41" t="str">
+      <c r="B36" s="36" t="str">
         <f>A34 &amp; "." &amp; B34 &amp; "." &amp; C34 &amp; "-" &amp; B35</f>
         <v>v1.1.1-Better_Default</v>
       </c>
-      <c r="C36" s="42"/>
+      <c r="C36" s="37"/>
       <c r="D36" s="5"/>
     </row>
     <row r="37" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -1995,30 +2090,25 @@
       <c r="A40" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="41" t="s">
+      <c r="B40" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="C40" s="42"/>
+      <c r="C40" s="37"/>
       <c r="D40" s="5"/>
     </row>
     <row r="41" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B41" s="41" t="str">
+      <c r="B41" s="36" t="str">
         <f>A39 &amp; "." &amp; B39 &amp; "." &amp; C39 &amp; "-" &amp; B40</f>
         <v>v1.1.0-Better_Default</v>
       </c>
-      <c r="C41" s="42"/>
+      <c r="C41" s="37"/>
       <c r="D41" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2031,6 +2121,11 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Add celestial textures and OptiFine sky configs
Add new celestial assets and sky configurations to improve sun/moon visuals. Includes new OptiFine sky image (overworld.png) and sky0.properties, a rotation axis fix in sky1.properties (axis set to 1.0 0.0 0.0), moon_phases.png and sun.png textures, and a set of separate moon phase images under v10.0.10-Classic_Reimagined_10_SE_2. Also update version_guide.xlsx to reflect these changes.
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E846C9D-5065-44FA-9308-1356FE1A3AFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CEBF46A-71EE-4671-8B8E-B523365BC759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="76">
   <si>
     <t>Current version in development</t>
   </si>
@@ -256,6 +256,12 @@
   </si>
   <si>
     <t>Updated bat model</t>
+  </si>
+  <si>
+    <t>Changed rabbit model</t>
+  </si>
+  <si>
+    <t>Changed sky orientation</t>
   </si>
 </sst>
 </file>
@@ -1013,6 +1019,9 @@
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>74</v>
+      </c>
       <c r="G16" s="9" t="s">
         <v>17</v>
       </c>
@@ -1026,7 +1035,10 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
+        <v>75</v>
+      </c>
       <c r="G17" s="10" t="s">
         <v>11</v>
       </c>
@@ -1041,7 +1053,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="18" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G18" s="11" t="s">
         <v>13</v>
       </c>
@@ -1052,7 +1064,7 @@
       <c r="I18" s="17"/>
       <c r="J18" s="15"/>
     </row>
-    <row r="19" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G19" s="11" t="s">
         <v>14</v>
       </c>
@@ -1063,7 +1075,7 @@
       <c r="I19" s="17"/>
       <c r="J19" s="15"/>
     </row>
-    <row r="20" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G20" s="11" t="s">
         <v>15</v>
       </c>
@@ -1073,7 +1085,7 @@
       </c>
       <c r="I20" s="17"/>
     </row>
-    <row r="21" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G21" s="9" t="s">
         <v>17</v>
       </c>
@@ -1087,7 +1099,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="22" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G22" s="10" t="s">
         <v>11</v>
       </c>
@@ -1102,7 +1114,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G23" s="11" t="s">
         <v>13</v>
       </c>
@@ -1113,7 +1125,7 @@
       <c r="I23" s="17"/>
       <c r="J23" s="15"/>
     </row>
-    <row r="24" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G24" s="11" t="s">
         <v>14</v>
       </c>
@@ -1124,7 +1136,7 @@
       <c r="I24" s="17"/>
       <c r="J24" s="15"/>
     </row>
-    <row r="25" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G25" s="11" t="s">
         <v>15</v>
       </c>
@@ -1134,7 +1146,7 @@
       </c>
       <c r="I25" s="17"/>
     </row>
-    <row r="26" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G26" s="9" t="s">
         <v>17</v>
       </c>
@@ -1148,7 +1160,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G27" s="10" t="s">
         <v>11</v>
       </c>
@@ -1163,7 +1175,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G28" s="11" t="s">
         <v>13</v>
       </c>
@@ -1174,7 +1186,7 @@
       <c r="I28" s="17"/>
       <c r="J28" s="15"/>
     </row>
-    <row r="29" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G29" s="11" t="s">
         <v>14</v>
       </c>
@@ -1185,7 +1197,7 @@
       <c r="I29" s="17"/>
       <c r="J29" s="15"/>
     </row>
-    <row r="30" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G30" s="11" t="s">
         <v>15</v>
       </c>
@@ -1195,7 +1207,7 @@
       </c>
       <c r="I30" s="17"/>
     </row>
-    <row r="31" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G31" s="9" t="s">
         <v>17</v>
       </c>
@@ -1209,7 +1221,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="7:10" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="G32" s="10" t="s">
         <v>11</v>
       </c>
@@ -2122,6 +2134,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2134,11 +2151,6 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Add 1.20.3+ shader support and leaf textures
Adds new shader files (clouds.fsh, clouds.vsh, lightmap.fsh, fog.glsl) for format 90 (1.20.3+). Includes new leaf textures (azalea, cherry, classic, flowering_azalea, jungle, mangrove, pale_oak, spruce) with mipmap metadata. Updates pack.mcmeta to support format 90 and adjusts shader directory version constraints.
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BFB7825-6E3F-42F8-B5DB-2B7950B9E675}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ADCB976-D1E5-413F-BBF9-843976E1AED6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="70">
   <si>
     <t>Current version in development</t>
   </si>
@@ -238,6 +238,12 @@
   </si>
   <si>
     <t>Release year</t>
+  </si>
+  <si>
+    <t>Added 26.3+ shader support</t>
+  </si>
+  <si>
+    <t>Added leaf textures for Classic Reimagined 11</t>
   </si>
 </sst>
 </file>
@@ -481,9 +487,6 @@
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -527,6 +530,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -728,13 +740,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="33"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="30"/>
       <c r="G1" s="24" t="s">
         <v>66</v>
       </c>
@@ -748,7 +760,7 @@
         <v>62</v>
       </c>
       <c r="B2" s="26">
-        <v>5</v>
+        <v>5.4</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>5</v>
@@ -795,7 +807,7 @@
       </c>
       <c r="J4" s="10" t="str">
         <f>D8</f>
-        <v>5308-rt5</v>
+        <v>5708-rt5.4</v>
       </c>
       <c r="K4" s="10">
         <v>26.3</v>
@@ -825,7 +837,7 @@
       </c>
       <c r="B6" s="27">
         <f>(B2*1000)+(B3*100)+B4+((B5-2026)*1000)</f>
-        <v>5308</v>
+        <v>5708</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>14</v>
@@ -839,11 +851,11 @@
       <c r="K6" s="15"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="40" t="s">
+      <c r="A7" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="41"/>
-      <c r="C7" s="42"/>
+      <c r="B7" s="38"/>
+      <c r="C7" s="39"/>
       <c r="D7" s="9" t="s">
         <v>3</v>
       </c>
@@ -855,21 +867,21 @@
       </c>
       <c r="H7" s="12" t="str">
         <f>H6 &amp; "-build-" &amp; J4</f>
-        <v>v10.0.11_3-Classic_Reimagined_11_SE_2.1-build-5308-rt5</v>
+        <v>v10.0.11_3-Classic_Reimagined_11_SE_2.1-build-5708-rt5.4</v>
       </c>
       <c r="I7" s="13"/>
       <c r="J7" s="14"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="28" t="str">
+      <c r="A8" s="43" t="str">
         <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-build-" &amp; D8</f>
-        <v>v10.0.11_3-build-5308-rt5</v>
-      </c>
-      <c r="B8" s="29"/>
-      <c r="C8" s="30"/>
+        <v>v10.0.11_3-build-5708-rt5.4</v>
+      </c>
+      <c r="B8" s="44"/>
+      <c r="C8" s="45"/>
       <c r="D8" s="10" t="str">
         <f>B6&amp;"-rt"&amp;B2</f>
-        <v>5308-rt5</v>
+        <v>5708-rt5.4</v>
       </c>
       <c r="E8" s="19">
         <f>K10</f>
@@ -886,11 +898,11 @@
       <c r="B9" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="34" t="s">
+      <c r="C9" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="35"/>
-      <c r="E9" s="36"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="33"/>
       <c r="G9" s="9" t="s">
         <v>2</v>
       </c>
@@ -908,11 +920,14 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="C10" s="37" t="s">
+      <c r="A10" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="C10" s="34" t="s">
         <v>12</v>
       </c>
-      <c r="D10" s="38"/>
-      <c r="E10" s="39"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="36"/>
       <c r="G10" s="10" t="s">
         <v>11</v>
       </c>
@@ -924,13 +939,16 @@
       </c>
       <c r="J10" s="10" t="str">
         <f>J4</f>
-        <v>5308-rt5</v>
+        <v>5708-rt5.4</v>
       </c>
       <c r="K10" s="10">
         <v>26.2</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>69</v>
+      </c>
       <c r="G11" s="11" t="s">
         <v>13</v>
       </c>
@@ -960,7 +978,7 @@
       </c>
       <c r="H13" s="12" t="str">
         <f>H12 &amp; "-build-" &amp; J10</f>
-        <v>v10.0.11_2-Classic_Reimagined_11_SE_2.1-build-5308-rt5</v>
+        <v>v10.0.11_2-Classic_Reimagined_11_SE_2.1-build-5708-rt5.4</v>
       </c>
       <c r="I13" s="13"/>
       <c r="J13" s="14"/>
@@ -1008,7 +1026,7 @@
       </c>
       <c r="J17" s="10" t="str">
         <f>J10</f>
-        <v>5308-rt5</v>
+        <v>5708-rt5.4</v>
       </c>
       <c r="K17" s="10">
         <v>26.1</v>
@@ -1044,7 +1062,7 @@
       </c>
       <c r="H20" s="12" t="str">
         <f>H19 &amp; "-build-" &amp; J17</f>
-        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5308-rt5</v>
+        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5708-rt5.4</v>
       </c>
       <c r="I20" s="13"/>
       <c r="J20" s="14"/>
@@ -1077,7 +1095,7 @@
       </c>
       <c r="I23" s="10" t="str">
         <f>J17</f>
-        <v>5308-rt5</v>
+        <v>5708-rt5.4</v>
       </c>
       <c r="J23" s="10" t="s">
         <v>18</v>
@@ -1111,7 +1129,7 @@
       </c>
       <c r="H26" s="16" t="str">
         <f>H25 &amp; "-build-" &amp; I23</f>
-        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5308-rt5</v>
+        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5708-rt5.4</v>
       </c>
       <c r="I26" s="17"/>
     </row>
@@ -1138,7 +1156,7 @@
       </c>
       <c r="I28" s="10" t="str">
         <f>I23</f>
-        <v>5308-rt5</v>
+        <v>5708-rt5.4</v>
       </c>
       <c r="J28" s="10" t="s">
         <v>19</v>
@@ -1172,7 +1190,7 @@
       </c>
       <c r="H31" s="16" t="str">
         <f>H30 &amp; "-build-" &amp; I28</f>
-        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5308-rt5</v>
+        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5708-rt5.4</v>
       </c>
       <c r="I31" s="17"/>
     </row>
@@ -1199,7 +1217,7 @@
       </c>
       <c r="I33" s="10" t="str">
         <f>I28</f>
-        <v>5308-rt5</v>
+        <v>5708-rt5.4</v>
       </c>
       <c r="J33" s="10" t="s">
         <v>20</v>
@@ -1233,7 +1251,7 @@
       </c>
       <c r="H36" s="16" t="str">
         <f>H35 &amp; "-build-" &amp; I33</f>
-        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5308-rt5</v>
+        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5708-rt5.4</v>
       </c>
       <c r="I36" s="17"/>
     </row>
@@ -1260,7 +1278,7 @@
       </c>
       <c r="I38" s="10" t="str">
         <f>I33</f>
-        <v>5308-rt5</v>
+        <v>5708-rt5.4</v>
       </c>
       <c r="J38" s="10" t="s">
         <v>21</v>
@@ -1294,7 +1312,7 @@
       </c>
       <c r="H41" s="16" t="str">
         <f>H40 &amp; "-build-" &amp; I38</f>
-        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5308-rt5</v>
+        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5708-rt5.4</v>
       </c>
       <c r="I41" s="17"/>
     </row>
@@ -1326,7 +1344,7 @@
       </c>
       <c r="I44" s="10" t="str">
         <f>I38</f>
-        <v>5308-rt5</v>
+        <v>5708-rt5.4</v>
       </c>
       <c r="J44" s="10" t="s">
         <v>23</v>
@@ -1360,7 +1378,7 @@
       </c>
       <c r="H47" s="16" t="str">
         <f>H46 &amp; "-build-" &amp; I44</f>
-        <v>v10.0.3-Classic_Reimagined_10_SE-build-5308-rt5</v>
+        <v>v10.0.3-Classic_Reimagined_10_SE-build-5708-rt5.4</v>
       </c>
       <c r="I47" s="17"/>
     </row>
@@ -1392,7 +1410,7 @@
       </c>
       <c r="I50" s="10" t="str">
         <f>I44</f>
-        <v>5308-rt5</v>
+        <v>5708-rt5.4</v>
       </c>
       <c r="J50" s="10" t="s">
         <v>25</v>
@@ -1425,7 +1443,7 @@
       </c>
       <c r="H53" s="16" t="str">
         <f>H52 &amp; "-build-" &amp; I50</f>
-        <v>v10.0.2-Classic_Reimagined_10s-build-5308-rt5</v>
+        <v>v10.0.2-Classic_Reimagined_10s-build-5708-rt5.4</v>
       </c>
       <c r="I53" s="17"/>
     </row>
@@ -1457,7 +1475,7 @@
       </c>
       <c r="I56" s="10" t="str">
         <f>I50</f>
-        <v>5308-rt5</v>
+        <v>5708-rt5.4</v>
       </c>
       <c r="J56" s="10" t="s">
         <v>28</v>
@@ -1490,7 +1508,7 @@
       </c>
       <c r="H59" s="16" t="str">
         <f>H58 &amp; "-build-" &amp; I56</f>
-        <v>v10.0.1-Classic_Reimagined_10-build-5308-rt5</v>
+        <v>v10.0.1-Classic_Reimagined_10-build-5708-rt5.4</v>
       </c>
       <c r="I59" s="17"/>
     </row>
@@ -1530,7 +1548,7 @@
       </c>
       <c r="I63" s="10" t="str">
         <f>I56</f>
-        <v>5308-rt5</v>
+        <v>5708-rt5.4</v>
       </c>
       <c r="J63" s="10" t="s">
         <v>33</v>
@@ -1563,7 +1581,7 @@
       </c>
       <c r="H66" s="16" t="str">
         <f>H65 &amp; "-build-" &amp; I63</f>
-        <v>v8.10.32-Classic_Reimagined_8-build-5308-rt5</v>
+        <v>v8.10.32-Classic_Reimagined_8-build-5708-rt5.4</v>
       </c>
       <c r="I66" s="17"/>
     </row>
@@ -1595,7 +1613,7 @@
       </c>
       <c r="I69" s="10" t="str">
         <f>I63</f>
-        <v>5308-rt5</v>
+        <v>5708-rt5.4</v>
       </c>
       <c r="J69" s="10" t="s">
         <v>35</v>
@@ -1628,7 +1646,7 @@
       </c>
       <c r="H72" s="16" t="str">
         <f>H71 &amp; "-build-" &amp; I69</f>
-        <v>v8.10.31-Classic_Reimagined_8-build-5308-rt5</v>
+        <v>v8.10.31-Classic_Reimagined_8-build-5708-rt5.4</v>
       </c>
       <c r="I72" s="17"/>
     </row>
@@ -1663,7 +1681,7 @@
       </c>
       <c r="I75" s="10" t="str">
         <f>I69</f>
-        <v>5308-rt5</v>
+        <v>5708-rt5.4</v>
       </c>
       <c r="J75" s="10" t="s">
         <v>38</v>
@@ -1696,7 +1714,7 @@
       </c>
       <c r="H78" s="16" t="str">
         <f>H77 &amp; "-build-" &amp; I75</f>
-        <v>v7.11.3-Better_Default_7-build-5308-rt5</v>
+        <v>v7.11.3-Better_Default_7-build-5708-rt5.4</v>
       </c>
       <c r="I78" s="17"/>
     </row>
@@ -1704,11 +1722,12 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:B4">
     <sortCondition descending="1" ref="A3:A4"/>
   </sortState>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C9:E9"/>
     <mergeCell ref="C10:E10"/>
     <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A8:C8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1724,12 +1743,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="42" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="45"/>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
     </row>
     <row r="2" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
@@ -1768,21 +1787,21 @@
       <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="43" t="s">
+      <c r="B5" s="40" t="s">
         <v>45</v>
       </c>
-      <c r="C5" s="44"/>
+      <c r="C5" s="41"/>
       <c r="D5" s="5"/>
     </row>
     <row r="6" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="43" t="str">
+      <c r="B6" s="40" t="str">
         <f>A4 &amp; "." &amp; B4 &amp; "." &amp; C4 &amp; "-" &amp; B5</f>
         <v>v6.0.7-Better_Default_6</v>
       </c>
-      <c r="C6" s="44"/>
+      <c r="C6" s="41"/>
       <c r="D6" s="5"/>
     </row>
     <row r="7" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -1822,21 +1841,21 @@
       <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="43" t="s">
+      <c r="B10" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="C10" s="44"/>
+      <c r="C10" s="41"/>
       <c r="D10" s="5"/>
     </row>
     <row r="11" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="43" t="str">
+      <c r="B11" s="40" t="str">
         <f>A9 &amp; "." &amp; B9 &amp; "." &amp; C9 &amp; "-" &amp; B10</f>
         <v>v1.4.0-Better_Default_5</v>
       </c>
-      <c r="C11" s="44"/>
+      <c r="C11" s="41"/>
       <c r="D11" s="5"/>
     </row>
     <row r="12" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -1876,21 +1895,21 @@
       <c r="A15" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="43" t="s">
+      <c r="B15" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="44"/>
+      <c r="C15" s="41"/>
       <c r="D15" s="5"/>
     </row>
     <row r="16" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="43" t="str">
+      <c r="B16" s="40" t="str">
         <f>A14 &amp; "." &amp; B14 &amp; "." &amp; C14 &amp; "-" &amp; B15</f>
         <v>v1.3.0-Better_Default_4</v>
       </c>
-      <c r="C16" s="44"/>
+      <c r="C16" s="41"/>
       <c r="D16" s="5"/>
     </row>
     <row r="17" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -1930,21 +1949,21 @@
       <c r="A20" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="43" t="s">
+      <c r="B20" s="40" t="s">
         <v>55</v>
       </c>
-      <c r="C20" s="44"/>
+      <c r="C20" s="41"/>
       <c r="D20" s="5"/>
     </row>
     <row r="21" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B21" s="43" t="str">
+      <c r="B21" s="40" t="str">
         <f>A19 &amp; "." &amp; B19 &amp; "." &amp; C19 &amp; "-" &amp; B20</f>
         <v>v1.2.2-Better_Default_3.1</v>
       </c>
-      <c r="C21" s="44"/>
+      <c r="C21" s="41"/>
       <c r="D21" s="5"/>
     </row>
     <row r="22" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -1984,21 +2003,21 @@
       <c r="A25" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="43" t="s">
+      <c r="B25" s="40" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="44"/>
+      <c r="C25" s="41"/>
       <c r="D25" s="5"/>
     </row>
     <row r="26" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B26" s="43" t="str">
+      <c r="B26" s="40" t="str">
         <f>A24 &amp; "." &amp; B24 &amp; "." &amp; C24 &amp; "-" &amp; B25</f>
         <v>v1.2.1-Better_Default_3</v>
       </c>
-      <c r="C26" s="44"/>
+      <c r="C26" s="41"/>
       <c r="D26" s="5"/>
     </row>
     <row r="27" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2038,21 +2057,21 @@
       <c r="A30" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B30" s="43" t="s">
+      <c r="B30" s="40" t="s">
         <v>58</v>
       </c>
-      <c r="C30" s="44"/>
+      <c r="C30" s="41"/>
       <c r="D30" s="5"/>
     </row>
     <row r="31" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="43" t="str">
+      <c r="B31" s="40" t="str">
         <f>A29 &amp; "." &amp; B29 &amp; "." &amp; C29 &amp; "-" &amp; B30</f>
         <v>v1.2.0-Better_Default_2</v>
       </c>
-      <c r="C31" s="44"/>
+      <c r="C31" s="41"/>
       <c r="D31" s="5"/>
     </row>
     <row r="32" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2092,21 +2111,21 @@
       <c r="A35" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B35" s="43" t="s">
+      <c r="B35" s="40" t="s">
         <v>60</v>
       </c>
-      <c r="C35" s="44"/>
+      <c r="C35" s="41"/>
       <c r="D35" s="5"/>
     </row>
     <row r="36" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B36" s="43" t="str">
+      <c r="B36" s="40" t="str">
         <f>A34 &amp; "." &amp; B34 &amp; "." &amp; C34 &amp; "-" &amp; B35</f>
         <v>v1.1.1-Better_Default</v>
       </c>
-      <c r="C36" s="44"/>
+      <c r="C36" s="41"/>
       <c r="D36" s="5"/>
     </row>
     <row r="37" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -2146,25 +2165,30 @@
       <c r="A40" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="43" t="s">
+      <c r="B40" s="40" t="s">
         <v>60</v>
       </c>
-      <c r="C40" s="44"/>
+      <c r="C40" s="41"/>
       <c r="D40" s="5"/>
     </row>
     <row r="41" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B41" s="43" t="str">
+      <c r="B41" s="40" t="str">
         <f>A39 &amp; "." &amp; B39 &amp; "." &amp; C39 &amp; "-" &amp; B40</f>
         <v>v1.1.0-Better_Default</v>
       </c>
-      <c r="C41" s="44"/>
+      <c r="C41" s="41"/>
       <c r="D41" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2177,11 +2201,6 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
added straw bed textures
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D503B18-8514-4A87-98DF-A2E142D27EF1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BE53206-2808-4306-9CDF-C5D9345E964B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="74">
   <si>
     <t>Current version in development</t>
   </si>
@@ -253,6 +253,9 @@
   </si>
   <si>
     <t>Added cushion textures</t>
+  </si>
+  <si>
+    <t>Added straw bed textures</t>
   </si>
 </sst>
 </file>
@@ -956,7 +959,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G11" s="11" t="s">
         <v>13</v>
@@ -971,7 +974,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G12" s="11" t="s">
         <v>14</v>
@@ -986,7 +989,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G13" s="11" t="s">
         <v>15</v>
@@ -1000,7 +1003,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>1</v>
@@ -1011,6 +1014,9 @@
       <c r="K14" s="7"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
+        <v>73</v>
+      </c>
       <c r="G15" s="8" t="s">
         <v>5</v>
       </c>
@@ -1737,8 +1743,8 @@
       <c r="I78" s="17"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:B4">
-    <sortCondition descending="1" ref="A3:A4"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A10:A15">
+    <sortCondition ref="A15"/>
   </sortState>
   <mergeCells count="5">
     <mergeCell ref="A1:E1"/>
@@ -2202,6 +2208,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2214,11 +2225,6 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Refactor classic fog calculation algorithm
Improved the classic_fog_value function with a more sophisticated fog rendering approach. The new implementation uses smoothstep interpolation, realistic fog layering, and better value blending to achieve more realistic and visually improved fog effects in the 1.21.6 environmental fog shader.
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BE53206-2808-4306-9CDF-C5D9345E964B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28E11ADD-1A8E-4578-B026-32D5BFE5BA84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="75">
   <si>
     <t>Current version in development</t>
   </si>
@@ -256,6 +256,9 @@
   </si>
   <si>
     <t>Added straw bed textures</t>
+  </si>
+  <si>
+    <t>Updated ultrarealistic fog shaders</t>
   </si>
 </sst>
 </file>
@@ -1022,6 +1025,9 @@
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>74</v>
+      </c>
       <c r="G16" s="9" t="s">
         <v>2</v>
       </c>
@@ -2208,11 +2214,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B30:C30"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B5:C5"/>
@@ -2225,6 +2226,11 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B30:C30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
Add fire and lantern block assets
Added new fire and soul fire textures with animation metadata, along with template models for fire and lantern blocks. Reformatted fire blockstate JSON for better readability.
</commit_message>
<xml_diff>
--- a/version_guide.xlsx
+++ b/version_guide.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PrismLauncher\instances\NeoBeta Remastered\minecraft\resourcepacks\Classic-Reimagined\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28E11ADD-1A8E-4578-B026-32D5BFE5BA84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{796E6E14-E0E0-46CB-90BB-3E6C11F884FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="521" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="78">
   <si>
     <t>Current version in development</t>
   </si>
@@ -243,9 +243,6 @@
     <t>Added 26.3+ shader support</t>
   </si>
   <si>
-    <t>Added leaf textures for Classic Reimagined 11</t>
-  </si>
-  <si>
     <t>Added shelf mushroom textures</t>
   </si>
   <si>
@@ -259,6 +256,18 @@
   </si>
   <si>
     <t>Updated ultrarealistic fog shaders</t>
+  </si>
+  <si>
+    <t>Updated fog model for Classic Reimagined 11</t>
+  </si>
+  <si>
+    <t>Changed leaf textures for Classic Reimagined 11</t>
+  </si>
+  <si>
+    <t>Updated fire textures</t>
+  </si>
+  <si>
+    <t>Updated soul fire textures</t>
   </si>
 </sst>
 </file>
@@ -775,7 +784,7 @@
         <v>62</v>
       </c>
       <c r="B2" s="26">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G2" s="8" t="s">
         <v>5</v>
@@ -822,7 +831,7 @@
       </c>
       <c r="J4" s="10" t="str">
         <f>D8</f>
-        <v>5308-rt5</v>
+        <v>6308-rt6</v>
       </c>
       <c r="K4" s="10">
         <v>26.3</v>
@@ -852,7 +861,7 @@
       </c>
       <c r="B6" s="27">
         <f>(B2*1000)+(B3*100)+B4+((B5-2026)*1000)</f>
-        <v>5308</v>
+        <v>6308</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>14</v>
@@ -882,7 +891,7 @@
       </c>
       <c r="H7" s="12" t="str">
         <f>H6 &amp; "-build-" &amp; J4</f>
-        <v>v10.0.11_3-Classic_Reimagined_11_SE_2.1-build-5308-rt5</v>
+        <v>v10.0.11_3-Classic_Reimagined_11_SE_2.1-build-6308-rt6</v>
       </c>
       <c r="I7" s="13"/>
       <c r="J7" s="14"/>
@@ -890,13 +899,13 @@
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" s="40" t="str">
         <f>G4 &amp; "." &amp; H4 &amp; "_" &amp; I4 &amp; "-build-" &amp; D8</f>
-        <v>v10.0.11_3-build-5308-rt5</v>
+        <v>v10.0.11_3-build-6308-rt6</v>
       </c>
       <c r="B8" s="41"/>
       <c r="C8" s="42"/>
       <c r="D8" s="10" t="str">
         <f>B6&amp;"-rt"&amp;B2</f>
-        <v>5308-rt5</v>
+        <v>6308-rt6</v>
       </c>
       <c r="E8" s="19">
         <f>K10</f>
@@ -954,7 +963,7 @@
       </c>
       <c r="J10" s="10" t="str">
         <f>J4</f>
-        <v>5308-rt5</v>
+        <v>6308-rt6</v>
       </c>
       <c r="K10" s="10">
         <v>26.2</v>
@@ -962,7 +971,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G11" s="11" t="s">
         <v>13</v>
@@ -977,7 +986,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G12" s="11" t="s">
         <v>14</v>
@@ -992,21 +1001,21 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="G13" s="11" t="s">
         <v>15</v>
       </c>
       <c r="H13" s="12" t="str">
         <f>H12 &amp; "-build-" &amp; J10</f>
-        <v>v10.0.11_2-Classic_Reimagined_11_SE_2.1-build-5308-rt5</v>
+        <v>v10.0.11_2-Classic_Reimagined_11_SE_2.1-build-6308-rt6</v>
       </c>
       <c r="I13" s="13"/>
       <c r="J13" s="14"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G14" s="7" t="s">
         <v>1</v>
@@ -1018,7 +1027,7 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="G15" s="8" t="s">
         <v>5</v>
@@ -1026,7 +1035,7 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G16" s="9" t="s">
         <v>2</v>
@@ -1044,7 +1053,10 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="7:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
+        <v>74</v>
+      </c>
       <c r="G17" s="10" t="s">
         <v>11</v>
       </c>
@@ -1056,13 +1068,16 @@
       </c>
       <c r="J17" s="10" t="str">
         <f>J10</f>
-        <v>5308-rt5</v>
+        <v>6308-rt6</v>
       </c>
       <c r="K17" s="10">
         <v>26.1</v>
       </c>
     </row>
-    <row r="18" spans="7:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
+        <v>77</v>
+      </c>
       <c r="G18" s="11" t="s">
         <v>13</v>
       </c>
@@ -1074,7 +1089,10 @@
       <c r="J18" s="14"/>
       <c r="K18" s="15"/>
     </row>
-    <row r="19" spans="7:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
+        <v>73</v>
+      </c>
       <c r="G19" s="11" t="s">
         <v>14</v>
       </c>
@@ -1086,23 +1104,23 @@
       <c r="J19" s="14"/>
       <c r="K19" s="15"/>
     </row>
-    <row r="20" spans="7:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G20" s="11" t="s">
         <v>15</v>
       </c>
       <c r="H20" s="12" t="str">
         <f>H19 &amp; "-build-" &amp; J17</f>
-        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-5308-rt5</v>
+        <v>v10.0.11_1-Classic_Reimagined_10_SE_2.1-build-6308-rt6</v>
       </c>
       <c r="I20" s="13"/>
       <c r="J20" s="14"/>
     </row>
-    <row r="21" spans="7:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G21" s="8" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="22" spans="7:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G22" s="9" t="s">
         <v>17</v>
       </c>
@@ -1116,7 +1134,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="7:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G23" s="10" t="s">
         <v>11</v>
       </c>
@@ -1125,13 +1143,13 @@
       </c>
       <c r="I23" s="10" t="str">
         <f>J17</f>
-        <v>5308-rt5</v>
+        <v>6308-rt6</v>
       </c>
       <c r="J23" s="10" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="7:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G24" s="11" t="s">
         <v>13</v>
       </c>
@@ -1142,7 +1160,7 @@
       <c r="I24" s="17"/>
       <c r="J24" s="15"/>
     </row>
-    <row r="25" spans="7:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G25" s="11" t="s">
         <v>14</v>
       </c>
@@ -1153,17 +1171,17 @@
       <c r="I25" s="17"/>
       <c r="J25" s="15"/>
     </row>
-    <row r="26" spans="7:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G26" s="11" t="s">
         <v>15</v>
       </c>
       <c r="H26" s="16" t="str">
         <f>H25 &amp; "-build-" &amp; I23</f>
-        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-5308-rt5</v>
+        <v>v10.0.10-Classic_Reimagined_10_SE_2-build-6308-rt6</v>
       </c>
       <c r="I26" s="17"/>
     </row>
-    <row r="27" spans="7:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G27" s="9" t="s">
         <v>17</v>
       </c>
@@ -1177,7 +1195,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="7:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G28" s="10" t="s">
         <v>11</v>
       </c>
@@ -1186,13 +1204,13 @@
       </c>
       <c r="I28" s="10" t="str">
         <f>I23</f>
-        <v>5308-rt5</v>
+        <v>6308-rt6</v>
       </c>
       <c r="J28" s="10" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="7:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G29" s="11" t="s">
         <v>13</v>
       </c>
@@ -1203,7 +1221,7 @@
       <c r="I29" s="17"/>
       <c r="J29" s="15"/>
     </row>
-    <row r="30" spans="7:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G30" s="11" t="s">
         <v>14</v>
       </c>
@@ -1214,17 +1232,17 @@
       <c r="I30" s="17"/>
       <c r="J30" s="15"/>
     </row>
-    <row r="31" spans="7:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G31" s="11" t="s">
         <v>15</v>
       </c>
       <c r="H31" s="16" t="str">
         <f>H30 &amp; "-build-" &amp; I28</f>
-        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-5308-rt5</v>
+        <v>v10.0.9-Classic_Reimagined_10_SE_2-build-6308-rt6</v>
       </c>
       <c r="I31" s="17"/>
     </row>
-    <row r="32" spans="7:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G32" s="9" t="s">
         <v>17</v>
       </c>
@@ -1247,7 +1265,7 @@
       </c>
       <c r="I33" s="10" t="str">
         <f>I28</f>
-        <v>5308-rt5</v>
+        <v>6308-rt6</v>
       </c>
       <c r="J33" s="10" t="s">
         <v>20</v>
@@ -1281,7 +1299,7 @@
       </c>
       <c r="H36" s="16" t="str">
         <f>H35 &amp; "-build-" &amp; I33</f>
-        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-5308-rt5</v>
+        <v>v10.0.7-Classic_Reimagined_10_SE_2-build-6308-rt6</v>
       </c>
       <c r="I36" s="17"/>
     </row>
@@ -1308,7 +1326,7 @@
       </c>
       <c r="I38" s="10" t="str">
         <f>I33</f>
-        <v>5308-rt5</v>
+        <v>6308-rt6</v>
       </c>
       <c r="J38" s="10" t="s">
         <v>21</v>
@@ -1342,7 +1360,7 @@
       </c>
       <c r="H41" s="16" t="str">
         <f>H40 &amp; "-build-" &amp; I38</f>
-        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-5308-rt5</v>
+        <v>v10.0.4-Classic_Reimagined_10_SE_2-build-6308-rt6</v>
       </c>
       <c r="I41" s="17"/>
     </row>
@@ -1374,7 +1392,7 @@
       </c>
       <c r="I44" s="10" t="str">
         <f>I38</f>
-        <v>5308-rt5</v>
+        <v>6308-rt6</v>
       </c>
       <c r="J44" s="10" t="s">
         <v>23</v>
@@ -1408,7 +1426,7 @@
       </c>
       <c r="H47" s="16" t="str">
         <f>H46 &amp; "-build-" &amp; I44</f>
-        <v>v10.0.3-Classic_Reimagined_10_SE-build-5308-rt5</v>
+        <v>v10.0.3-Classic_Reimagined_10_SE-build-6308-rt6</v>
       </c>
       <c r="I47" s="17"/>
     </row>
@@ -1440,7 +1458,7 @@
       </c>
       <c r="I50" s="10" t="str">
         <f>I44</f>
-        <v>5308-rt5</v>
+        <v>6308-rt6</v>
       </c>
       <c r="J50" s="10" t="s">
         <v>25</v>
@@ -1473,7 +1491,7 @@
       </c>
       <c r="H53" s="16" t="str">
         <f>H52 &amp; "-build-" &amp; I50</f>
-        <v>v10.0.2-Classic_Reimagined_10s-build-5308-rt5</v>
+        <v>v10.0.2-Classic_Reimagined_10s-build-6308-rt6</v>
       </c>
       <c r="I53" s="17"/>
     </row>
@@ -1505,7 +1523,7 @@
       </c>
       <c r="I56" s="10" t="str">
         <f>I50</f>
-        <v>5308-rt5</v>
+        <v>6308-rt6</v>
       </c>
       <c r="J56" s="10" t="s">
         <v>28</v>
@@ -1538,7 +1556,7 @@
       </c>
       <c r="H59" s="16" t="str">
         <f>H58 &amp; "-build-" &amp; I56</f>
-        <v>v10.0.1-Classic_Reimagined_10-build-5308-rt5</v>
+        <v>v10.0.1-Classic_Reimagined_10-build-6308-rt6</v>
       </c>
       <c r="I59" s="17"/>
     </row>
@@ -1578,7 +1596,7 @@
       </c>
       <c r="I63" s="10" t="str">
         <f>I56</f>
-        <v>5308-rt5</v>
+        <v>6308-rt6</v>
       </c>
       <c r="J63" s="10" t="s">
         <v>33</v>
@@ -1611,7 +1629,7 @@
       </c>
       <c r="H66" s="16" t="str">
         <f>H65 &amp; "-build-" &amp; I63</f>
-        <v>v8.10.32-Classic_Reimagined_8-build-5308-rt5</v>
+        <v>v8.10.32-Classic_Reimagined_8-build-6308-rt6</v>
       </c>
       <c r="I66" s="17"/>
     </row>
@@ -1643,7 +1661,7 @@
       </c>
       <c r="I69" s="10" t="str">
         <f>I63</f>
-        <v>5308-rt5</v>
+        <v>6308-rt6</v>
       </c>
       <c r="J69" s="10" t="s">
         <v>35</v>
@@ -1676,7 +1694,7 @@
       </c>
       <c r="H72" s="16" t="str">
         <f>H71 &amp; "-build-" &amp; I69</f>
-        <v>v8.10.31-Classic_Reimagined_8-build-5308-rt5</v>
+        <v>v8.10.31-Classic_Reimagined_8-build-6308-rt6</v>
       </c>
       <c r="I72" s="17"/>
     </row>
@@ -1711,7 +1729,7 @@
       </c>
       <c r="I75" s="10" t="str">
         <f>I69</f>
-        <v>5308-rt5</v>
+        <v>6308-rt6</v>
       </c>
       <c r="J75" s="10" t="s">
         <v>38</v>
@@ -1744,13 +1762,13 @@
       </c>
       <c r="H78" s="16" t="str">
         <f>H77 &amp; "-build-" &amp; I75</f>
-        <v>v7.11.3-Better_Default_7-build-5308-rt5</v>
+        <v>v7.11.3-Better_Default_7-build-6308-rt6</v>
       </c>
       <c r="I78" s="17"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A10:A15">
-    <sortCondition ref="A15"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A10:A19">
+    <sortCondition ref="A19"/>
   </sortState>
   <mergeCells count="5">
     <mergeCell ref="A1:E1"/>

</xml_diff>